<commit_message>
Added Web stuff and cascade
</commit_message>
<xml_diff>
--- a/tanulókártyák/Tanulókártyák.xlsx
+++ b/tanulókártyák/Tanulókártyák.xlsx
@@ -1,14 +1,14 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="29929"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="30026"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\atesz\OneDrive\Desktop\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{EEA79994-669B-4107-B260-F61FFCDB1D5A}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{E8D087CB-FA50-495D-BA4A-83F5B00F82A8}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12576" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -25,7 +25,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="234" uniqueCount="233">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="270" uniqueCount="269">
   <si>
     <r>
       <rPr>
@@ -4650,6 +4650,831 @@
   </si>
   <si>
     <t>Mi aJDBC?</t>
+  </si>
+  <si>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="10"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <charset val="238"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve">CRUD - HTTP methods:
+</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <charset val="238"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve">CREATE - POST
+READ - GET,
+UPDATE - PUT, 
+DELETE - DELETE
+</t>
+    </r>
+  </si>
+  <si>
+    <t>Mit takar a CRUD betűszó
+és milyen HTTP metódusoknak
+ feleltethetőek meg az elemei?</t>
+  </si>
+  <si>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="10"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <charset val="238"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve">HTTP methods:
+</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <charset val="238"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>POST - Adatküldés, mentés a szerveren
+GET - Adat/információ lekérés a szerverről
+PUT - Adat módosítás a szerveren
+DELETE - Adat törlés a szerveren
+PATCH - Adat módosítás a szerveren
+OPTION - Engedélyeztetések kommunikációs beállítások lekérése
+HEAD - Információ lekérdezés a szerverről (pl: letöltés elött ellenőrizni a fáj méretet)</t>
+    </r>
+  </si>
+  <si>
+    <t>Milyen HTTP netódusok vannak, mit csinálnak?</t>
+  </si>
+  <si>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="10"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <charset val="238"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve">HTTP Response status code:
+</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <charset val="238"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>100 - általános információ a kliensnek. pl: ne vegye figyelembe a szerver választ
+200 - sikeres szerver művelet. pl: sikerült módosítani egy adatot a szerveren
+300 - átirányítás történt. pl: ideiglenesen más szerver szolgálja ki a választ
+400 - hibakód. pl: autentikációs hiba, vagy hibás "path", általában kliens oldali hibára utal.
+500 - hibakód. Szerver oldali hiba.</t>
+    </r>
+  </si>
+  <si>
+    <t>Milyen HTTP response code-okat ismersz?</t>
+  </si>
+  <si>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="10"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <charset val="238"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve">HTTP:
+</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <charset val="238"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>A HTTP protokoll egy adatküldési protokoll, egy olyan szabályrendszer, amely azon szabályokat írja le, amely mentén az interneten a kliensek és a szerverek szöveges adatokat küldenek egymásnak, kérések és válaszok formájában.</t>
+    </r>
+  </si>
+  <si>
+    <t>Mi az HTTP?</t>
+  </si>
+  <si>
+    <t>Mit jelent, hogy az HTTP állpotmentes protokoll?</t>
+  </si>
+  <si>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="10"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <charset val="238"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve">Egy HTTP kérés tartalmazza: </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <charset val="238"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve">
+a kérés metódusát, egy elérési utat, az alkalmazott protokoll verzióját, egy header elemet, és a metódustól függően egy body elemet.
+</t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="10"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <charset val="238"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve">A HTTP válasz kiegészül:
+</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <charset val="238"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>egy státusz kóddal, és egy státusz üzenettel</t>
+    </r>
+  </si>
+  <si>
+    <t>Milyen elemeket tartalmaz
+ egy HTTP kérés és válasz?</t>
+  </si>
+  <si>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="10"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <charset val="238"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve">A HTTP állapotmentes (stateless) protokoll:
+</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <charset val="238"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>azt jelenti, hogy minden kérés független, és nem tárol információt a korábbi kérésekről.
+Az állapotmentesség problémáit általában cookie-k és session-ök használatával kezelik, amelyek lehetővé teszik az állapotinformációk tárolását a kliens és a szerver között.</t>
+    </r>
+  </si>
+  <si>
+    <t>Mi az HTTPS?</t>
+  </si>
+  <si>
+    <r>
+      <t xml:space="preserve">Az </t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="10"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <charset val="238"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>HTTPS</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <charset val="238"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve"> (HTTP Secure) egy kiegészítő protokoll, amely titkosítást használ a kliens és a szerver közötti adatátvitel biztonságának növelése érdekében. Az HTTPS SSL (Secure Sockets Layer) vagy TLS (Transport Layer Security) protokollokon keresztül biztosítja az adatok titkosítását.
+/A TLS az SSL modernizált változata és ma már szinte csak azt használják./</t>
+    </r>
+  </si>
+  <si>
+    <r>
+      <t xml:space="preserve">Az </t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="10"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <charset val="238"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>IP-cím</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <charset val="238"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve"> egy hálózati eszköz egyedi azonosítója.
+Segítségével találják meg egymást az eszközök az interneten vagy egy helyi hálózaton. Olyan, mint egy postacím a digitális világban.
+Az </t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="10"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <charset val="238"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>IPv4</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <charset val="238"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve"> a legelterjedtebb IP-címzési rendszer.
+32 bites címeket használ, például: 192.168.1.1.
+Körülbelül 4,3 milliárd egyedi címet tud kezelni.
+Az</t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="10"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <charset val="238"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve"> IPv6</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <charset val="238"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve"> az IPv4 utódja. 128 bites címeket használ, például: 2001:db8::1. Gyakorlatilag kimeríthetetlen mennyiségű címet biztosít.</t>
+    </r>
+  </si>
+  <si>
+    <t>Mi az IP-cím, 
+mi a különbség az IPv4 és IPv6 között?</t>
+  </si>
+  <si>
+    <r>
+      <t xml:space="preserve">A </t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="10"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <charset val="238"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>DNS</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <charset val="238"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve"> a Domain Name System rövidítése.
+A domainneveket (pl. google.com) IP-címekké alakítja.
+Olyan, mint az internet telefonkönyve.
+A </t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="10"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <charset val="238"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>domain név</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <charset val="238"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve"> egy könnyen megjegyezhető internetes cím.
+Például: google.com vagy openai.com.
+A DNS fordítja le IP-címre.</t>
+    </r>
+  </si>
+  <si>
+    <t>Mi a DNS és a domain név?</t>
+  </si>
+  <si>
+    <t>Mi a TCP és az UDP?</t>
+  </si>
+  <si>
+    <r>
+      <t xml:space="preserve">A </t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="10"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <charset val="238"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>TCP</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <charset val="238"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve"> megbízható adatátviteli protokoll.
+Ellenőrzi, hogy minden csomag megérkezett-e és helyes sorrendben van-e.
+Weboldalak és e-mailek esetén gyakran használják.
+A</t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="10"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <charset val="238"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve"> UDP</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <charset val="238"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve"> gyorsabb, mint a TCP.
+Nem ellenőrzi a csomagok megérkezését vagy sorrendjét.
+Gyakori online játékoknál és videóhívásoknál.</t>
+    </r>
+  </si>
+  <si>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="10"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <charset val="238"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>FTP</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <charset val="238"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve">, </t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="10"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <charset val="238"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>SCP</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <charset val="238"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>: (File Trasfer Protocol, Secure Copy protocol) - fájlok másolásására szolgáló kommunikációs protokoll számítógépek között</t>
+    </r>
+  </si>
+  <si>
+    <t>Mi az FTP és SCP?</t>
+  </si>
+  <si>
+    <r>
+      <t xml:space="preserve">A </t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="10"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <charset val="238"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>REST</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <charset val="238"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve"> (Representational State Transfer) nem egy protokoll, hanem egy architekturális stílus a hálózati alkalmazások, különösen webes szolgáltatások fejlesztéséhez. A REST alapelvei segítségével a fejlesztők egyszerű, skálázható és könnyen karbantartható webes API-kat hozhatnak létre.</t>
+    </r>
+  </si>
+  <si>
+    <r>
+      <t xml:space="preserve">1. </t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="10"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <charset val="238"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>Kliens–szerver elválasztás</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <charset val="238"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve"> : A kliens (pl. böngésző vagy mobilapp) és a szerver külön felelősségi körrel rendelkezik. A kliens kéréseket küld, a szerver adatot és szolgáltatást nyújt.
+2. </t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="10"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <charset val="238"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>Stateless (állapotmentes)</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <charset val="238"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve">: A szerver nem tárolja a kliens korábbi kéréseinek állapotát. Minden kérésnek önmagában tartalmaznia kell minden szükséges információt.
+3. </t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="10"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <charset val="238"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>Erőforrás-alapú működés</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <charset val="238"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve">: Minden adat egy erőforrásként jelenik meg, amelyet URI-val érünk el.
+</t>
+    </r>
+  </si>
+  <si>
+    <t>REST alapelvek (1/2)</t>
+  </si>
+  <si>
+    <t>Mi a REST?</t>
+  </si>
+  <si>
+    <r>
+      <t xml:space="preserve">4. </t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="10"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <charset val="238"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>Egységes interfész (Uniform Interface):</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <charset val="238"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve">
+Az API következetesen használja a HTTP metódusokat.
+5. </t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="10"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <charset val="238"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>Cache-elhetőség:</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <charset val="238"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve">
+A válaszok megjelölhetők gyorsítótárazhatónak.
+Ez csökkenti a szerver terhelését és gyorsítja a válaszidőt.
+6. </t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="10"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <charset val="238"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>Rétegzett architektúra:</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <charset val="238"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve">
+A kliensnek nem kell tudnia, hogy közvetlenül a szerverrel vagy köztes rendszereken (proxy, load balancer, gateway) keresztül kommunikál.</t>
+    </r>
+  </si>
+  <si>
+    <t>REST alapelvek (2/2)</t>
+  </si>
+  <si>
+    <r>
+      <t xml:space="preserve">A </t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="10"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <charset val="238"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>JSON</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <charset val="238"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve"> (JavaScript Object Notation) egy könnyű adatcsere-formátum, amely ember által olvasható szöveges formátumban tárol adatokat. Gyakran használják webes alkalmazásokban adatok küldésére és fogadására a szerver és a kliens között. Előnye, hogy könnyen értelmezhető és generálható a legtöbb programozási nyelven.</t>
+    </r>
+  </si>
+  <si>
+    <t>Mi a JSON?</t>
+  </si>
+  <si>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="10"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <charset val="238"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve">A 4 rétegű TCP/IP modell </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <charset val="238"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve">az internet működését leíró hálózati modell. Egyszerűbb, mint a 7 rétegű OSI modell, és a gyakorlatban ezt használják gyakrabban.
+Röviden:
+1. Alkalmazási réteg (HTTP/HTTPS, DNS, SMTP)
+2. Szállítási réteg (TCP, UDP)
+3. Internet réteg (IPv4, IPv6)
+4. Hálózati hozzáférési réteg (Ethernet kábel, Wi-Fi, optikai hálózat)
+</t>
+    </r>
+  </si>
+  <si>
+    <t>Mi és miből áll a 4 rétegű TCP/IP modell?</t>
+  </si>
+  <si>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="10"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <charset val="238"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>HTTP három fő jellemzője:</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <charset val="238"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve">
+Kapcsolat nélküli (connectionless): a kliens elküldi a kérést, a kapcsolat lezárul, majd megvárja a választ.
+Médiafüggetlen: bármilyen adattípust továbbíthat, ha a kliens és a szerver is támogatja.
+Állapotmentes (stateless): a kérések között nem tárol állapotot, minden kérés önálló.</t>
+    </r>
+  </si>
+  <si>
+    <t>Mi a HTTP három fő jellemzője?</t>
+  </si>
+  <si>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="10"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <charset val="238"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve">Cascade: </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <charset val="238"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>A szülő entitás műveleteit automatikusan továbbítja a kapcsolódó entitásokra.
+CascadeType.PERSIST: Mentéskor a kapcsolódó objektumokat is menti.
+.MERGE: A kapcsolódó objektumokat is frissíti.
+.REMOVE: Törléskor a kapcsolódó objektumokat is törli.
+.REFRESH: Újratölti az adatokat az adatbázisból.
+.DETACH: Leválasztja az entitásokat a persistence contextből.
+.ALL: Az összes cascade műveletet alkalmazza.</t>
+    </r>
+  </si>
+  <si>
+    <t>Mit jelent a cascade, milyen formái vannak?</t>
   </si>
 </sst>
 </file>
@@ -5042,13 +5867,13 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:CR151"/>
+  <dimension ref="A1:DH151"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
-    <col min="1" max="96" width="11" customWidth="1"/>
+    <col min="1" max="112" width="11" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:96" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:112" x14ac:dyDescent="0.3">
       <c r="A1" s="7" t="s">
         <v>0</v>
       </c>
@@ -5193,8 +6018,32 @@
       <c r="CP1" s="8"/>
       <c r="CQ1" s="8"/>
       <c r="CR1" s="8"/>
+      <c r="CS1" s="7" t="s">
+        <v>239</v>
+      </c>
+      <c r="CT1" s="8"/>
+      <c r="CU1" s="8"/>
+      <c r="CV1" s="8"/>
+      <c r="CW1" s="7" t="s">
+        <v>244</v>
+      </c>
+      <c r="CX1" s="8"/>
+      <c r="CY1" s="8"/>
+      <c r="CZ1" s="8"/>
+      <c r="DA1" s="7" t="s">
+        <v>259</v>
+      </c>
+      <c r="DB1" s="8"/>
+      <c r="DC1" s="8"/>
+      <c r="DD1" s="8"/>
+      <c r="DE1" s="7" t="s">
+        <v>261</v>
+      </c>
+      <c r="DF1" s="8"/>
+      <c r="DG1" s="8"/>
+      <c r="DH1" s="8"/>
     </row>
-    <row r="2" spans="1:96" x14ac:dyDescent="0.3">
+    <row r="2" spans="1:112" x14ac:dyDescent="0.3">
       <c r="A2" s="8"/>
       <c r="B2" s="8"/>
       <c r="C2" s="8"/>
@@ -5291,8 +6140,24 @@
       <c r="CP2" s="8"/>
       <c r="CQ2" s="8"/>
       <c r="CR2" s="8"/>
+      <c r="CS2" s="8"/>
+      <c r="CT2" s="8"/>
+      <c r="CU2" s="8"/>
+      <c r="CV2" s="8"/>
+      <c r="CW2" s="8"/>
+      <c r="CX2" s="8"/>
+      <c r="CY2" s="8"/>
+      <c r="CZ2" s="8"/>
+      <c r="DA2" s="8"/>
+      <c r="DB2" s="8"/>
+      <c r="DC2" s="8"/>
+      <c r="DD2" s="8"/>
+      <c r="DE2" s="8"/>
+      <c r="DF2" s="8"/>
+      <c r="DG2" s="8"/>
+      <c r="DH2" s="8"/>
     </row>
-    <row r="3" spans="1:96" x14ac:dyDescent="0.3">
+    <row r="3" spans="1:112" x14ac:dyDescent="0.3">
       <c r="A3" s="8"/>
       <c r="B3" s="8"/>
       <c r="C3" s="8"/>
@@ -5389,8 +6254,24 @@
       <c r="CP3" s="8"/>
       <c r="CQ3" s="8"/>
       <c r="CR3" s="8"/>
+      <c r="CS3" s="8"/>
+      <c r="CT3" s="8"/>
+      <c r="CU3" s="8"/>
+      <c r="CV3" s="8"/>
+      <c r="CW3" s="8"/>
+      <c r="CX3" s="8"/>
+      <c r="CY3" s="8"/>
+      <c r="CZ3" s="8"/>
+      <c r="DA3" s="8"/>
+      <c r="DB3" s="8"/>
+      <c r="DC3" s="8"/>
+      <c r="DD3" s="8"/>
+      <c r="DE3" s="8"/>
+      <c r="DF3" s="8"/>
+      <c r="DG3" s="8"/>
+      <c r="DH3" s="8"/>
     </row>
-    <row r="4" spans="1:96" x14ac:dyDescent="0.3">
+    <row r="4" spans="1:112" x14ac:dyDescent="0.3">
       <c r="A4" s="8"/>
       <c r="B4" s="8"/>
       <c r="C4" s="8"/>
@@ -5487,8 +6368,24 @@
       <c r="CP4" s="8"/>
       <c r="CQ4" s="8"/>
       <c r="CR4" s="8"/>
+      <c r="CS4" s="8"/>
+      <c r="CT4" s="8"/>
+      <c r="CU4" s="8"/>
+      <c r="CV4" s="8"/>
+      <c r="CW4" s="8"/>
+      <c r="CX4" s="8"/>
+      <c r="CY4" s="8"/>
+      <c r="CZ4" s="8"/>
+      <c r="DA4" s="8"/>
+      <c r="DB4" s="8"/>
+      <c r="DC4" s="8"/>
+      <c r="DD4" s="8"/>
+      <c r="DE4" s="8"/>
+      <c r="DF4" s="8"/>
+      <c r="DG4" s="8"/>
+      <c r="DH4" s="8"/>
     </row>
-    <row r="5" spans="1:96" x14ac:dyDescent="0.3">
+    <row r="5" spans="1:112" x14ac:dyDescent="0.3">
       <c r="A5" s="8"/>
       <c r="B5" s="8"/>
       <c r="C5" s="8"/>
@@ -5585,8 +6482,24 @@
       <c r="CP5" s="8"/>
       <c r="CQ5" s="8"/>
       <c r="CR5" s="8"/>
+      <c r="CS5" s="8"/>
+      <c r="CT5" s="8"/>
+      <c r="CU5" s="8"/>
+      <c r="CV5" s="8"/>
+      <c r="CW5" s="8"/>
+      <c r="CX5" s="8"/>
+      <c r="CY5" s="8"/>
+      <c r="CZ5" s="8"/>
+      <c r="DA5" s="8"/>
+      <c r="DB5" s="8"/>
+      <c r="DC5" s="8"/>
+      <c r="DD5" s="8"/>
+      <c r="DE5" s="8"/>
+      <c r="DF5" s="8"/>
+      <c r="DG5" s="8"/>
+      <c r="DH5" s="8"/>
     </row>
-    <row r="6" spans="1:96" x14ac:dyDescent="0.3">
+    <row r="6" spans="1:112" x14ac:dyDescent="0.3">
       <c r="A6" s="8"/>
       <c r="B6" s="8"/>
       <c r="C6" s="8"/>
@@ -5683,8 +6596,24 @@
       <c r="CP6" s="8"/>
       <c r="CQ6" s="8"/>
       <c r="CR6" s="8"/>
+      <c r="CS6" s="8"/>
+      <c r="CT6" s="8"/>
+      <c r="CU6" s="8"/>
+      <c r="CV6" s="8"/>
+      <c r="CW6" s="8"/>
+      <c r="CX6" s="8"/>
+      <c r="CY6" s="8"/>
+      <c r="CZ6" s="8"/>
+      <c r="DA6" s="8"/>
+      <c r="DB6" s="8"/>
+      <c r="DC6" s="8"/>
+      <c r="DD6" s="8"/>
+      <c r="DE6" s="8"/>
+      <c r="DF6" s="8"/>
+      <c r="DG6" s="8"/>
+      <c r="DH6" s="8"/>
     </row>
-    <row r="7" spans="1:96" x14ac:dyDescent="0.3">
+    <row r="7" spans="1:112" x14ac:dyDescent="0.3">
       <c r="A7" s="8"/>
       <c r="B7" s="8"/>
       <c r="C7" s="8"/>
@@ -5781,8 +6710,24 @@
       <c r="CP7" s="8"/>
       <c r="CQ7" s="8"/>
       <c r="CR7" s="8"/>
+      <c r="CS7" s="8"/>
+      <c r="CT7" s="8"/>
+      <c r="CU7" s="8"/>
+      <c r="CV7" s="8"/>
+      <c r="CW7" s="8"/>
+      <c r="CX7" s="8"/>
+      <c r="CY7" s="8"/>
+      <c r="CZ7" s="8"/>
+      <c r="DA7" s="8"/>
+      <c r="DB7" s="8"/>
+      <c r="DC7" s="8"/>
+      <c r="DD7" s="8"/>
+      <c r="DE7" s="8"/>
+      <c r="DF7" s="8"/>
+      <c r="DG7" s="8"/>
+      <c r="DH7" s="8"/>
     </row>
-    <row r="8" spans="1:96" x14ac:dyDescent="0.3">
+    <row r="8" spans="1:112" x14ac:dyDescent="0.3">
       <c r="A8" s="8"/>
       <c r="B8" s="8"/>
       <c r="C8" s="8"/>
@@ -5879,8 +6824,24 @@
       <c r="CP8" s="8"/>
       <c r="CQ8" s="8"/>
       <c r="CR8" s="8"/>
+      <c r="CS8" s="8"/>
+      <c r="CT8" s="8"/>
+      <c r="CU8" s="8"/>
+      <c r="CV8" s="8"/>
+      <c r="CW8" s="8"/>
+      <c r="CX8" s="8"/>
+      <c r="CY8" s="8"/>
+      <c r="CZ8" s="8"/>
+      <c r="DA8" s="8"/>
+      <c r="DB8" s="8"/>
+      <c r="DC8" s="8"/>
+      <c r="DD8" s="8"/>
+      <c r="DE8" s="8"/>
+      <c r="DF8" s="8"/>
+      <c r="DG8" s="8"/>
+      <c r="DH8" s="8"/>
     </row>
-    <row r="9" spans="1:96" x14ac:dyDescent="0.3">
+    <row r="9" spans="1:112" x14ac:dyDescent="0.3">
       <c r="A9" s="8"/>
       <c r="B9" s="8"/>
       <c r="C9" s="8"/>
@@ -5977,8 +6938,24 @@
       <c r="CP9" s="8"/>
       <c r="CQ9" s="8"/>
       <c r="CR9" s="8"/>
+      <c r="CS9" s="8"/>
+      <c r="CT9" s="8"/>
+      <c r="CU9" s="8"/>
+      <c r="CV9" s="8"/>
+      <c r="CW9" s="8"/>
+      <c r="CX9" s="8"/>
+      <c r="CY9" s="8"/>
+      <c r="CZ9" s="8"/>
+      <c r="DA9" s="8"/>
+      <c r="DB9" s="8"/>
+      <c r="DC9" s="8"/>
+      <c r="DD9" s="8"/>
+      <c r="DE9" s="8"/>
+      <c r="DF9" s="8"/>
+      <c r="DG9" s="8"/>
+      <c r="DH9" s="8"/>
     </row>
-    <row r="10" spans="1:96" x14ac:dyDescent="0.3">
+    <row r="10" spans="1:112" x14ac:dyDescent="0.3">
       <c r="A10" s="8"/>
       <c r="B10" s="8"/>
       <c r="C10" s="8"/>
@@ -6075,8 +7052,24 @@
       <c r="CP10" s="8"/>
       <c r="CQ10" s="8"/>
       <c r="CR10" s="8"/>
+      <c r="CS10" s="8"/>
+      <c r="CT10" s="8"/>
+      <c r="CU10" s="8"/>
+      <c r="CV10" s="8"/>
+      <c r="CW10" s="8"/>
+      <c r="CX10" s="8"/>
+      <c r="CY10" s="8"/>
+      <c r="CZ10" s="8"/>
+      <c r="DA10" s="8"/>
+      <c r="DB10" s="8"/>
+      <c r="DC10" s="8"/>
+      <c r="DD10" s="8"/>
+      <c r="DE10" s="8"/>
+      <c r="DF10" s="8"/>
+      <c r="DG10" s="8"/>
+      <c r="DH10" s="8"/>
     </row>
-    <row r="11" spans="1:96" x14ac:dyDescent="0.3">
+    <row r="11" spans="1:112" x14ac:dyDescent="0.3">
       <c r="A11" s="7" t="s">
         <v>2</v>
       </c>
@@ -6221,8 +7214,32 @@
       <c r="CP11" s="8"/>
       <c r="CQ11" s="8"/>
       <c r="CR11" s="8"/>
+      <c r="CS11" s="7" t="s">
+        <v>242</v>
+      </c>
+      <c r="CT11" s="8"/>
+      <c r="CU11" s="8"/>
+      <c r="CV11" s="8"/>
+      <c r="CW11" s="7" t="s">
+        <v>246</v>
+      </c>
+      <c r="CX11" s="8"/>
+      <c r="CY11" s="8"/>
+      <c r="CZ11" s="8"/>
+      <c r="DA11" s="7" t="s">
+        <v>263</v>
+      </c>
+      <c r="DB11" s="8"/>
+      <c r="DC11" s="8"/>
+      <c r="DD11" s="8"/>
+      <c r="DE11" s="7" t="s">
+        <v>265</v>
+      </c>
+      <c r="DF11" s="8"/>
+      <c r="DG11" s="8"/>
+      <c r="DH11" s="8"/>
     </row>
-    <row r="12" spans="1:96" x14ac:dyDescent="0.3">
+    <row r="12" spans="1:112" x14ac:dyDescent="0.3">
       <c r="A12" s="8"/>
       <c r="B12" s="8"/>
       <c r="C12" s="8"/>
@@ -6319,8 +7336,24 @@
       <c r="CP12" s="8"/>
       <c r="CQ12" s="8"/>
       <c r="CR12" s="8"/>
+      <c r="CS12" s="8"/>
+      <c r="CT12" s="8"/>
+      <c r="CU12" s="8"/>
+      <c r="CV12" s="8"/>
+      <c r="CW12" s="8"/>
+      <c r="CX12" s="8"/>
+      <c r="CY12" s="8"/>
+      <c r="CZ12" s="8"/>
+      <c r="DA12" s="8"/>
+      <c r="DB12" s="8"/>
+      <c r="DC12" s="8"/>
+      <c r="DD12" s="8"/>
+      <c r="DE12" s="8"/>
+      <c r="DF12" s="8"/>
+      <c r="DG12" s="8"/>
+      <c r="DH12" s="8"/>
     </row>
-    <row r="13" spans="1:96" x14ac:dyDescent="0.3">
+    <row r="13" spans="1:112" x14ac:dyDescent="0.3">
       <c r="A13" s="8"/>
       <c r="B13" s="8"/>
       <c r="C13" s="8"/>
@@ -6417,8 +7450,24 @@
       <c r="CP13" s="8"/>
       <c r="CQ13" s="8"/>
       <c r="CR13" s="8"/>
+      <c r="CS13" s="8"/>
+      <c r="CT13" s="8"/>
+      <c r="CU13" s="8"/>
+      <c r="CV13" s="8"/>
+      <c r="CW13" s="8"/>
+      <c r="CX13" s="8"/>
+      <c r="CY13" s="8"/>
+      <c r="CZ13" s="8"/>
+      <c r="DA13" s="8"/>
+      <c r="DB13" s="8"/>
+      <c r="DC13" s="8"/>
+      <c r="DD13" s="8"/>
+      <c r="DE13" s="8"/>
+      <c r="DF13" s="8"/>
+      <c r="DG13" s="8"/>
+      <c r="DH13" s="8"/>
     </row>
-    <row r="14" spans="1:96" x14ac:dyDescent="0.3">
+    <row r="14" spans="1:112" x14ac:dyDescent="0.3">
       <c r="A14" s="8"/>
       <c r="B14" s="8"/>
       <c r="C14" s="8"/>
@@ -6515,8 +7564,24 @@
       <c r="CP14" s="8"/>
       <c r="CQ14" s="8"/>
       <c r="CR14" s="8"/>
+      <c r="CS14" s="8"/>
+      <c r="CT14" s="8"/>
+      <c r="CU14" s="8"/>
+      <c r="CV14" s="8"/>
+      <c r="CW14" s="8"/>
+      <c r="CX14" s="8"/>
+      <c r="CY14" s="8"/>
+      <c r="CZ14" s="8"/>
+      <c r="DA14" s="8"/>
+      <c r="DB14" s="8"/>
+      <c r="DC14" s="8"/>
+      <c r="DD14" s="8"/>
+      <c r="DE14" s="8"/>
+      <c r="DF14" s="8"/>
+      <c r="DG14" s="8"/>
+      <c r="DH14" s="8"/>
     </row>
-    <row r="15" spans="1:96" x14ac:dyDescent="0.3">
+    <row r="15" spans="1:112" x14ac:dyDescent="0.3">
       <c r="A15" s="8"/>
       <c r="B15" s="8"/>
       <c r="C15" s="8"/>
@@ -6613,8 +7678,24 @@
       <c r="CP15" s="8"/>
       <c r="CQ15" s="8"/>
       <c r="CR15" s="8"/>
+      <c r="CS15" s="8"/>
+      <c r="CT15" s="8"/>
+      <c r="CU15" s="8"/>
+      <c r="CV15" s="8"/>
+      <c r="CW15" s="8"/>
+      <c r="CX15" s="8"/>
+      <c r="CY15" s="8"/>
+      <c r="CZ15" s="8"/>
+      <c r="DA15" s="8"/>
+      <c r="DB15" s="8"/>
+      <c r="DC15" s="8"/>
+      <c r="DD15" s="8"/>
+      <c r="DE15" s="8"/>
+      <c r="DF15" s="8"/>
+      <c r="DG15" s="8"/>
+      <c r="DH15" s="8"/>
     </row>
-    <row r="16" spans="1:96" x14ac:dyDescent="0.3">
+    <row r="16" spans="1:112" x14ac:dyDescent="0.3">
       <c r="A16" s="8"/>
       <c r="B16" s="8"/>
       <c r="C16" s="8"/>
@@ -6711,8 +7792,24 @@
       <c r="CP16" s="8"/>
       <c r="CQ16" s="8"/>
       <c r="CR16" s="8"/>
+      <c r="CS16" s="8"/>
+      <c r="CT16" s="8"/>
+      <c r="CU16" s="8"/>
+      <c r="CV16" s="8"/>
+      <c r="CW16" s="8"/>
+      <c r="CX16" s="8"/>
+      <c r="CY16" s="8"/>
+      <c r="CZ16" s="8"/>
+      <c r="DA16" s="8"/>
+      <c r="DB16" s="8"/>
+      <c r="DC16" s="8"/>
+      <c r="DD16" s="8"/>
+      <c r="DE16" s="8"/>
+      <c r="DF16" s="8"/>
+      <c r="DG16" s="8"/>
+      <c r="DH16" s="8"/>
     </row>
-    <row r="17" spans="1:96" x14ac:dyDescent="0.3">
+    <row r="17" spans="1:112" x14ac:dyDescent="0.3">
       <c r="A17" s="8"/>
       <c r="B17" s="8"/>
       <c r="C17" s="8"/>
@@ -6809,8 +7906,24 @@
       <c r="CP17" s="8"/>
       <c r="CQ17" s="8"/>
       <c r="CR17" s="8"/>
+      <c r="CS17" s="8"/>
+      <c r="CT17" s="8"/>
+      <c r="CU17" s="8"/>
+      <c r="CV17" s="8"/>
+      <c r="CW17" s="8"/>
+      <c r="CX17" s="8"/>
+      <c r="CY17" s="8"/>
+      <c r="CZ17" s="8"/>
+      <c r="DA17" s="8"/>
+      <c r="DB17" s="8"/>
+      <c r="DC17" s="8"/>
+      <c r="DD17" s="8"/>
+      <c r="DE17" s="8"/>
+      <c r="DF17" s="8"/>
+      <c r="DG17" s="8"/>
+      <c r="DH17" s="8"/>
     </row>
-    <row r="18" spans="1:96" x14ac:dyDescent="0.3">
+    <row r="18" spans="1:112" x14ac:dyDescent="0.3">
       <c r="A18" s="8"/>
       <c r="B18" s="8"/>
       <c r="C18" s="8"/>
@@ -6907,8 +8020,24 @@
       <c r="CP18" s="8"/>
       <c r="CQ18" s="8"/>
       <c r="CR18" s="8"/>
+      <c r="CS18" s="8"/>
+      <c r="CT18" s="8"/>
+      <c r="CU18" s="8"/>
+      <c r="CV18" s="8"/>
+      <c r="CW18" s="8"/>
+      <c r="CX18" s="8"/>
+      <c r="CY18" s="8"/>
+      <c r="CZ18" s="8"/>
+      <c r="DA18" s="8"/>
+      <c r="DB18" s="8"/>
+      <c r="DC18" s="8"/>
+      <c r="DD18" s="8"/>
+      <c r="DE18" s="8"/>
+      <c r="DF18" s="8"/>
+      <c r="DG18" s="8"/>
+      <c r="DH18" s="8"/>
     </row>
-    <row r="19" spans="1:96" x14ac:dyDescent="0.3">
+    <row r="19" spans="1:112" x14ac:dyDescent="0.3">
       <c r="A19" s="8"/>
       <c r="B19" s="8"/>
       <c r="C19" s="8"/>
@@ -7005,8 +8134,24 @@
       <c r="CP19" s="8"/>
       <c r="CQ19" s="8"/>
       <c r="CR19" s="8"/>
+      <c r="CS19" s="8"/>
+      <c r="CT19" s="8"/>
+      <c r="CU19" s="8"/>
+      <c r="CV19" s="8"/>
+      <c r="CW19" s="8"/>
+      <c r="CX19" s="8"/>
+      <c r="CY19" s="8"/>
+      <c r="CZ19" s="8"/>
+      <c r="DA19" s="8"/>
+      <c r="DB19" s="8"/>
+      <c r="DC19" s="8"/>
+      <c r="DD19" s="8"/>
+      <c r="DE19" s="8"/>
+      <c r="DF19" s="8"/>
+      <c r="DG19" s="8"/>
+      <c r="DH19" s="8"/>
     </row>
-    <row r="20" spans="1:96" x14ac:dyDescent="0.3">
+    <row r="20" spans="1:112" x14ac:dyDescent="0.3">
       <c r="A20" s="8"/>
       <c r="B20" s="8"/>
       <c r="C20" s="8"/>
@@ -7103,8 +8248,24 @@
       <c r="CP20" s="8"/>
       <c r="CQ20" s="8"/>
       <c r="CR20" s="8"/>
+      <c r="CS20" s="8"/>
+      <c r="CT20" s="8"/>
+      <c r="CU20" s="8"/>
+      <c r="CV20" s="8"/>
+      <c r="CW20" s="8"/>
+      <c r="CX20" s="8"/>
+      <c r="CY20" s="8"/>
+      <c r="CZ20" s="8"/>
+      <c r="DA20" s="8"/>
+      <c r="DB20" s="8"/>
+      <c r="DC20" s="8"/>
+      <c r="DD20" s="8"/>
+      <c r="DE20" s="8"/>
+      <c r="DF20" s="8"/>
+      <c r="DG20" s="8"/>
+      <c r="DH20" s="8"/>
     </row>
-    <row r="21" spans="1:96" x14ac:dyDescent="0.3">
+    <row r="21" spans="1:112" x14ac:dyDescent="0.3">
       <c r="A21" s="7" t="s">
         <v>4</v>
       </c>
@@ -7249,8 +8410,30 @@
       <c r="CP21" s="8"/>
       <c r="CQ21" s="8"/>
       <c r="CR21" s="8"/>
+      <c r="CS21" s="7" t="s">
+        <v>247</v>
+      </c>
+      <c r="CT21" s="8"/>
+      <c r="CU21" s="8"/>
+      <c r="CV21" s="8"/>
+      <c r="CW21" s="7" t="s">
+        <v>249</v>
+      </c>
+      <c r="CX21" s="8"/>
+      <c r="CY21" s="8"/>
+      <c r="CZ21" s="8"/>
+      <c r="DA21" s="7" t="s">
+        <v>267</v>
+      </c>
+      <c r="DB21" s="8"/>
+      <c r="DC21" s="8"/>
+      <c r="DD21" s="8"/>
+      <c r="DE21" s="7"/>
+      <c r="DF21" s="8"/>
+      <c r="DG21" s="8"/>
+      <c r="DH21" s="8"/>
     </row>
-    <row r="22" spans="1:96" x14ac:dyDescent="0.3">
+    <row r="22" spans="1:112" x14ac:dyDescent="0.3">
       <c r="A22" s="8"/>
       <c r="B22" s="8"/>
       <c r="C22" s="8"/>
@@ -7347,8 +8530,24 @@
       <c r="CP22" s="8"/>
       <c r="CQ22" s="8"/>
       <c r="CR22" s="8"/>
+      <c r="CS22" s="8"/>
+      <c r="CT22" s="8"/>
+      <c r="CU22" s="8"/>
+      <c r="CV22" s="8"/>
+      <c r="CW22" s="8"/>
+      <c r="CX22" s="8"/>
+      <c r="CY22" s="8"/>
+      <c r="CZ22" s="8"/>
+      <c r="DA22" s="8"/>
+      <c r="DB22" s="8"/>
+      <c r="DC22" s="8"/>
+      <c r="DD22" s="8"/>
+      <c r="DE22" s="8"/>
+      <c r="DF22" s="8"/>
+      <c r="DG22" s="8"/>
+      <c r="DH22" s="8"/>
     </row>
-    <row r="23" spans="1:96" x14ac:dyDescent="0.3">
+    <row r="23" spans="1:112" x14ac:dyDescent="0.3">
       <c r="A23" s="8"/>
       <c r="B23" s="8"/>
       <c r="C23" s="8"/>
@@ -7445,8 +8644,24 @@
       <c r="CP23" s="8"/>
       <c r="CQ23" s="8"/>
       <c r="CR23" s="8"/>
+      <c r="CS23" s="8"/>
+      <c r="CT23" s="8"/>
+      <c r="CU23" s="8"/>
+      <c r="CV23" s="8"/>
+      <c r="CW23" s="8"/>
+      <c r="CX23" s="8"/>
+      <c r="CY23" s="8"/>
+      <c r="CZ23" s="8"/>
+      <c r="DA23" s="8"/>
+      <c r="DB23" s="8"/>
+      <c r="DC23" s="8"/>
+      <c r="DD23" s="8"/>
+      <c r="DE23" s="8"/>
+      <c r="DF23" s="8"/>
+      <c r="DG23" s="8"/>
+      <c r="DH23" s="8"/>
     </row>
-    <row r="24" spans="1:96" x14ac:dyDescent="0.3">
+    <row r="24" spans="1:112" x14ac:dyDescent="0.3">
       <c r="A24" s="8"/>
       <c r="B24" s="8"/>
       <c r="C24" s="8"/>
@@ -7543,8 +8758,24 @@
       <c r="CP24" s="8"/>
       <c r="CQ24" s="8"/>
       <c r="CR24" s="8"/>
+      <c r="CS24" s="8"/>
+      <c r="CT24" s="8"/>
+      <c r="CU24" s="8"/>
+      <c r="CV24" s="8"/>
+      <c r="CW24" s="8"/>
+      <c r="CX24" s="8"/>
+      <c r="CY24" s="8"/>
+      <c r="CZ24" s="8"/>
+      <c r="DA24" s="8"/>
+      <c r="DB24" s="8"/>
+      <c r="DC24" s="8"/>
+      <c r="DD24" s="8"/>
+      <c r="DE24" s="8"/>
+      <c r="DF24" s="8"/>
+      <c r="DG24" s="8"/>
+      <c r="DH24" s="8"/>
     </row>
-    <row r="25" spans="1:96" x14ac:dyDescent="0.3">
+    <row r="25" spans="1:112" x14ac:dyDescent="0.3">
       <c r="A25" s="8"/>
       <c r="B25" s="8"/>
       <c r="C25" s="8"/>
@@ -7641,8 +8872,24 @@
       <c r="CP25" s="8"/>
       <c r="CQ25" s="8"/>
       <c r="CR25" s="8"/>
+      <c r="CS25" s="8"/>
+      <c r="CT25" s="8"/>
+      <c r="CU25" s="8"/>
+      <c r="CV25" s="8"/>
+      <c r="CW25" s="8"/>
+      <c r="CX25" s="8"/>
+      <c r="CY25" s="8"/>
+      <c r="CZ25" s="8"/>
+      <c r="DA25" s="8"/>
+      <c r="DB25" s="8"/>
+      <c r="DC25" s="8"/>
+      <c r="DD25" s="8"/>
+      <c r="DE25" s="8"/>
+      <c r="DF25" s="8"/>
+      <c r="DG25" s="8"/>
+      <c r="DH25" s="8"/>
     </row>
-    <row r="26" spans="1:96" x14ac:dyDescent="0.3">
+    <row r="26" spans="1:112" x14ac:dyDescent="0.3">
       <c r="A26" s="8"/>
       <c r="B26" s="8"/>
       <c r="C26" s="8"/>
@@ -7739,8 +8986,24 @@
       <c r="CP26" s="8"/>
       <c r="CQ26" s="8"/>
       <c r="CR26" s="8"/>
+      <c r="CS26" s="8"/>
+      <c r="CT26" s="8"/>
+      <c r="CU26" s="8"/>
+      <c r="CV26" s="8"/>
+      <c r="CW26" s="8"/>
+      <c r="CX26" s="8"/>
+      <c r="CY26" s="8"/>
+      <c r="CZ26" s="8"/>
+      <c r="DA26" s="8"/>
+      <c r="DB26" s="8"/>
+      <c r="DC26" s="8"/>
+      <c r="DD26" s="8"/>
+      <c r="DE26" s="8"/>
+      <c r="DF26" s="8"/>
+      <c r="DG26" s="8"/>
+      <c r="DH26" s="8"/>
     </row>
-    <row r="27" spans="1:96" x14ac:dyDescent="0.3">
+    <row r="27" spans="1:112" x14ac:dyDescent="0.3">
       <c r="A27" s="8"/>
       <c r="B27" s="8"/>
       <c r="C27" s="8"/>
@@ -7837,8 +9100,24 @@
       <c r="CP27" s="8"/>
       <c r="CQ27" s="8"/>
       <c r="CR27" s="8"/>
+      <c r="CS27" s="8"/>
+      <c r="CT27" s="8"/>
+      <c r="CU27" s="8"/>
+      <c r="CV27" s="8"/>
+      <c r="CW27" s="8"/>
+      <c r="CX27" s="8"/>
+      <c r="CY27" s="8"/>
+      <c r="CZ27" s="8"/>
+      <c r="DA27" s="8"/>
+      <c r="DB27" s="8"/>
+      <c r="DC27" s="8"/>
+      <c r="DD27" s="8"/>
+      <c r="DE27" s="8"/>
+      <c r="DF27" s="8"/>
+      <c r="DG27" s="8"/>
+      <c r="DH27" s="8"/>
     </row>
-    <row r="28" spans="1:96" x14ac:dyDescent="0.3">
+    <row r="28" spans="1:112" x14ac:dyDescent="0.3">
       <c r="A28" s="8"/>
       <c r="B28" s="8"/>
       <c r="C28" s="8"/>
@@ -7935,8 +9214,24 @@
       <c r="CP28" s="8"/>
       <c r="CQ28" s="8"/>
       <c r="CR28" s="8"/>
+      <c r="CS28" s="8"/>
+      <c r="CT28" s="8"/>
+      <c r="CU28" s="8"/>
+      <c r="CV28" s="8"/>
+      <c r="CW28" s="8"/>
+      <c r="CX28" s="8"/>
+      <c r="CY28" s="8"/>
+      <c r="CZ28" s="8"/>
+      <c r="DA28" s="8"/>
+      <c r="DB28" s="8"/>
+      <c r="DC28" s="8"/>
+      <c r="DD28" s="8"/>
+      <c r="DE28" s="8"/>
+      <c r="DF28" s="8"/>
+      <c r="DG28" s="8"/>
+      <c r="DH28" s="8"/>
     </row>
-    <row r="29" spans="1:96" x14ac:dyDescent="0.3">
+    <row r="29" spans="1:112" x14ac:dyDescent="0.3">
       <c r="A29" s="8"/>
       <c r="B29" s="8"/>
       <c r="C29" s="8"/>
@@ -8033,8 +9328,24 @@
       <c r="CP29" s="8"/>
       <c r="CQ29" s="8"/>
       <c r="CR29" s="8"/>
+      <c r="CS29" s="8"/>
+      <c r="CT29" s="8"/>
+      <c r="CU29" s="8"/>
+      <c r="CV29" s="8"/>
+      <c r="CW29" s="8"/>
+      <c r="CX29" s="8"/>
+      <c r="CY29" s="8"/>
+      <c r="CZ29" s="8"/>
+      <c r="DA29" s="8"/>
+      <c r="DB29" s="8"/>
+      <c r="DC29" s="8"/>
+      <c r="DD29" s="8"/>
+      <c r="DE29" s="8"/>
+      <c r="DF29" s="8"/>
+      <c r="DG29" s="8"/>
+      <c r="DH29" s="8"/>
     </row>
-    <row r="30" spans="1:96" x14ac:dyDescent="0.3">
+    <row r="30" spans="1:112" x14ac:dyDescent="0.3">
       <c r="A30" s="8"/>
       <c r="B30" s="8"/>
       <c r="C30" s="8"/>
@@ -8131,8 +9442,24 @@
       <c r="CP30" s="8"/>
       <c r="CQ30" s="8"/>
       <c r="CR30" s="8"/>
+      <c r="CS30" s="8"/>
+      <c r="CT30" s="8"/>
+      <c r="CU30" s="8"/>
+      <c r="CV30" s="8"/>
+      <c r="CW30" s="8"/>
+      <c r="CX30" s="8"/>
+      <c r="CY30" s="8"/>
+      <c r="CZ30" s="8"/>
+      <c r="DA30" s="8"/>
+      <c r="DB30" s="8"/>
+      <c r="DC30" s="8"/>
+      <c r="DD30" s="8"/>
+      <c r="DE30" s="8"/>
+      <c r="DF30" s="8"/>
+      <c r="DG30" s="8"/>
+      <c r="DH30" s="8"/>
     </row>
-    <row r="31" spans="1:96" x14ac:dyDescent="0.3">
+    <row r="31" spans="1:112" x14ac:dyDescent="0.3">
       <c r="A31" s="7" t="s">
         <v>13</v>
       </c>
@@ -8271,12 +9598,34 @@
       <c r="CL31" s="8"/>
       <c r="CM31" s="8"/>
       <c r="CN31" s="8"/>
-      <c r="CO31" s="7"/>
+      <c r="CO31" s="7" t="s">
+        <v>233</v>
+      </c>
       <c r="CP31" s="8"/>
       <c r="CQ31" s="8"/>
       <c r="CR31" s="8"/>
+      <c r="CS31" s="7" t="s">
+        <v>253</v>
+      </c>
+      <c r="CT31" s="8"/>
+      <c r="CU31" s="8"/>
+      <c r="CV31" s="8"/>
+      <c r="CW31" s="7" t="s">
+        <v>252</v>
+      </c>
+      <c r="CX31" s="8"/>
+      <c r="CY31" s="8"/>
+      <c r="CZ31" s="8"/>
+      <c r="DA31" s="7"/>
+      <c r="DB31" s="8"/>
+      <c r="DC31" s="8"/>
+      <c r="DD31" s="8"/>
+      <c r="DE31" s="7"/>
+      <c r="DF31" s="8"/>
+      <c r="DG31" s="8"/>
+      <c r="DH31" s="8"/>
     </row>
-    <row r="32" spans="1:96" x14ac:dyDescent="0.3">
+    <row r="32" spans="1:112" x14ac:dyDescent="0.3">
       <c r="A32" s="8"/>
       <c r="B32" s="8"/>
       <c r="C32" s="8"/>
@@ -8373,8 +9722,24 @@
       <c r="CP32" s="8"/>
       <c r="CQ32" s="8"/>
       <c r="CR32" s="8"/>
+      <c r="CS32" s="8"/>
+      <c r="CT32" s="8"/>
+      <c r="CU32" s="8"/>
+      <c r="CV32" s="8"/>
+      <c r="CW32" s="8"/>
+      <c r="CX32" s="8"/>
+      <c r="CY32" s="8"/>
+      <c r="CZ32" s="8"/>
+      <c r="DA32" s="8"/>
+      <c r="DB32" s="8"/>
+      <c r="DC32" s="8"/>
+      <c r="DD32" s="8"/>
+      <c r="DE32" s="8"/>
+      <c r="DF32" s="8"/>
+      <c r="DG32" s="8"/>
+      <c r="DH32" s="8"/>
     </row>
-    <row r="33" spans="1:96" x14ac:dyDescent="0.3">
+    <row r="33" spans="1:112" x14ac:dyDescent="0.3">
       <c r="A33" s="8"/>
       <c r="B33" s="8"/>
       <c r="C33" s="8"/>
@@ -8471,8 +9836,24 @@
       <c r="CP33" s="8"/>
       <c r="CQ33" s="8"/>
       <c r="CR33" s="8"/>
+      <c r="CS33" s="8"/>
+      <c r="CT33" s="8"/>
+      <c r="CU33" s="8"/>
+      <c r="CV33" s="8"/>
+      <c r="CW33" s="8"/>
+      <c r="CX33" s="8"/>
+      <c r="CY33" s="8"/>
+      <c r="CZ33" s="8"/>
+      <c r="DA33" s="8"/>
+      <c r="DB33" s="8"/>
+      <c r="DC33" s="8"/>
+      <c r="DD33" s="8"/>
+      <c r="DE33" s="8"/>
+      <c r="DF33" s="8"/>
+      <c r="DG33" s="8"/>
+      <c r="DH33" s="8"/>
     </row>
-    <row r="34" spans="1:96" x14ac:dyDescent="0.3">
+    <row r="34" spans="1:112" x14ac:dyDescent="0.3">
       <c r="A34" s="8"/>
       <c r="B34" s="8"/>
       <c r="C34" s="8"/>
@@ -8569,8 +9950,24 @@
       <c r="CP34" s="8"/>
       <c r="CQ34" s="8"/>
       <c r="CR34" s="8"/>
+      <c r="CS34" s="8"/>
+      <c r="CT34" s="8"/>
+      <c r="CU34" s="8"/>
+      <c r="CV34" s="8"/>
+      <c r="CW34" s="8"/>
+      <c r="CX34" s="8"/>
+      <c r="CY34" s="8"/>
+      <c r="CZ34" s="8"/>
+      <c r="DA34" s="8"/>
+      <c r="DB34" s="8"/>
+      <c r="DC34" s="8"/>
+      <c r="DD34" s="8"/>
+      <c r="DE34" s="8"/>
+      <c r="DF34" s="8"/>
+      <c r="DG34" s="8"/>
+      <c r="DH34" s="8"/>
     </row>
-    <row r="35" spans="1:96" x14ac:dyDescent="0.3">
+    <row r="35" spans="1:112" x14ac:dyDescent="0.3">
       <c r="A35" s="8"/>
       <c r="B35" s="8"/>
       <c r="C35" s="8"/>
@@ -8667,8 +10064,24 @@
       <c r="CP35" s="8"/>
       <c r="CQ35" s="8"/>
       <c r="CR35" s="8"/>
+      <c r="CS35" s="8"/>
+      <c r="CT35" s="8"/>
+      <c r="CU35" s="8"/>
+      <c r="CV35" s="8"/>
+      <c r="CW35" s="8"/>
+      <c r="CX35" s="8"/>
+      <c r="CY35" s="8"/>
+      <c r="CZ35" s="8"/>
+      <c r="DA35" s="8"/>
+      <c r="DB35" s="8"/>
+      <c r="DC35" s="8"/>
+      <c r="DD35" s="8"/>
+      <c r="DE35" s="8"/>
+      <c r="DF35" s="8"/>
+      <c r="DG35" s="8"/>
+      <c r="DH35" s="8"/>
     </row>
-    <row r="36" spans="1:96" x14ac:dyDescent="0.3">
+    <row r="36" spans="1:112" x14ac:dyDescent="0.3">
       <c r="A36" s="8"/>
       <c r="B36" s="8"/>
       <c r="C36" s="8"/>
@@ -8765,8 +10178,24 @@
       <c r="CP36" s="8"/>
       <c r="CQ36" s="8"/>
       <c r="CR36" s="8"/>
+      <c r="CS36" s="8"/>
+      <c r="CT36" s="8"/>
+      <c r="CU36" s="8"/>
+      <c r="CV36" s="8"/>
+      <c r="CW36" s="8"/>
+      <c r="CX36" s="8"/>
+      <c r="CY36" s="8"/>
+      <c r="CZ36" s="8"/>
+      <c r="DA36" s="8"/>
+      <c r="DB36" s="8"/>
+      <c r="DC36" s="8"/>
+      <c r="DD36" s="8"/>
+      <c r="DE36" s="8"/>
+      <c r="DF36" s="8"/>
+      <c r="DG36" s="8"/>
+      <c r="DH36" s="8"/>
     </row>
-    <row r="37" spans="1:96" x14ac:dyDescent="0.3">
+    <row r="37" spans="1:112" x14ac:dyDescent="0.3">
       <c r="A37" s="8"/>
       <c r="B37" s="8"/>
       <c r="C37" s="8"/>
@@ -8863,8 +10292,24 @@
       <c r="CP37" s="8"/>
       <c r="CQ37" s="8"/>
       <c r="CR37" s="8"/>
+      <c r="CS37" s="8"/>
+      <c r="CT37" s="8"/>
+      <c r="CU37" s="8"/>
+      <c r="CV37" s="8"/>
+      <c r="CW37" s="8"/>
+      <c r="CX37" s="8"/>
+      <c r="CY37" s="8"/>
+      <c r="CZ37" s="8"/>
+      <c r="DA37" s="8"/>
+      <c r="DB37" s="8"/>
+      <c r="DC37" s="8"/>
+      <c r="DD37" s="8"/>
+      <c r="DE37" s="8"/>
+      <c r="DF37" s="8"/>
+      <c r="DG37" s="8"/>
+      <c r="DH37" s="8"/>
     </row>
-    <row r="38" spans="1:96" x14ac:dyDescent="0.3">
+    <row r="38" spans="1:112" x14ac:dyDescent="0.3">
       <c r="A38" s="8"/>
       <c r="B38" s="8"/>
       <c r="C38" s="8"/>
@@ -8961,8 +10406,24 @@
       <c r="CP38" s="8"/>
       <c r="CQ38" s="8"/>
       <c r="CR38" s="8"/>
+      <c r="CS38" s="8"/>
+      <c r="CT38" s="8"/>
+      <c r="CU38" s="8"/>
+      <c r="CV38" s="8"/>
+      <c r="CW38" s="8"/>
+      <c r="CX38" s="8"/>
+      <c r="CY38" s="8"/>
+      <c r="CZ38" s="8"/>
+      <c r="DA38" s="8"/>
+      <c r="DB38" s="8"/>
+      <c r="DC38" s="8"/>
+      <c r="DD38" s="8"/>
+      <c r="DE38" s="8"/>
+      <c r="DF38" s="8"/>
+      <c r="DG38" s="8"/>
+      <c r="DH38" s="8"/>
     </row>
-    <row r="39" spans="1:96" x14ac:dyDescent="0.3">
+    <row r="39" spans="1:112" x14ac:dyDescent="0.3">
       <c r="A39" s="8"/>
       <c r="B39" s="8"/>
       <c r="C39" s="8"/>
@@ -9059,8 +10520,24 @@
       <c r="CP39" s="8"/>
       <c r="CQ39" s="8"/>
       <c r="CR39" s="8"/>
+      <c r="CS39" s="8"/>
+      <c r="CT39" s="8"/>
+      <c r="CU39" s="8"/>
+      <c r="CV39" s="8"/>
+      <c r="CW39" s="8"/>
+      <c r="CX39" s="8"/>
+      <c r="CY39" s="8"/>
+      <c r="CZ39" s="8"/>
+      <c r="DA39" s="8"/>
+      <c r="DB39" s="8"/>
+      <c r="DC39" s="8"/>
+      <c r="DD39" s="8"/>
+      <c r="DE39" s="8"/>
+      <c r="DF39" s="8"/>
+      <c r="DG39" s="8"/>
+      <c r="DH39" s="8"/>
     </row>
-    <row r="40" spans="1:96" x14ac:dyDescent="0.3">
+    <row r="40" spans="1:112" x14ac:dyDescent="0.3">
       <c r="A40" s="8"/>
       <c r="B40" s="8"/>
       <c r="C40" s="8"/>
@@ -9157,8 +10634,24 @@
       <c r="CP40" s="8"/>
       <c r="CQ40" s="8"/>
       <c r="CR40" s="8"/>
+      <c r="CS40" s="8"/>
+      <c r="CT40" s="8"/>
+      <c r="CU40" s="8"/>
+      <c r="CV40" s="8"/>
+      <c r="CW40" s="8"/>
+      <c r="CX40" s="8"/>
+      <c r="CY40" s="8"/>
+      <c r="CZ40" s="8"/>
+      <c r="DA40" s="8"/>
+      <c r="DB40" s="8"/>
+      <c r="DC40" s="8"/>
+      <c r="DD40" s="8"/>
+      <c r="DE40" s="8"/>
+      <c r="DF40" s="8"/>
+      <c r="DG40" s="8"/>
+      <c r="DH40" s="8"/>
     </row>
-    <row r="41" spans="1:96" x14ac:dyDescent="0.3">
+    <row r="41" spans="1:112" x14ac:dyDescent="0.3">
       <c r="A41" s="7" t="s">
         <v>16</v>
       </c>
@@ -9291,16 +10784,40 @@
       <c r="CH41" s="8"/>
       <c r="CI41" s="8"/>
       <c r="CJ41" s="8"/>
-      <c r="CK41" s="7"/>
+      <c r="CK41" s="7" t="s">
+        <v>235</v>
+      </c>
       <c r="CL41" s="8"/>
       <c r="CM41" s="8"/>
       <c r="CN41" s="8"/>
-      <c r="CO41" s="9"/>
+      <c r="CO41" s="9" t="s">
+        <v>237</v>
+      </c>
       <c r="CP41" s="8"/>
       <c r="CQ41" s="8"/>
       <c r="CR41" s="8"/>
+      <c r="CS41" s="7" t="s">
+        <v>255</v>
+      </c>
+      <c r="CT41" s="8"/>
+      <c r="CU41" s="8"/>
+      <c r="CV41" s="8"/>
+      <c r="CW41" s="9" t="s">
+        <v>256</v>
+      </c>
+      <c r="CX41" s="8"/>
+      <c r="CY41" s="8"/>
+      <c r="CZ41" s="8"/>
+      <c r="DA41" s="7"/>
+      <c r="DB41" s="8"/>
+      <c r="DC41" s="8"/>
+      <c r="DD41" s="8"/>
+      <c r="DE41" s="9"/>
+      <c r="DF41" s="8"/>
+      <c r="DG41" s="8"/>
+      <c r="DH41" s="8"/>
     </row>
-    <row r="42" spans="1:96" x14ac:dyDescent="0.3">
+    <row r="42" spans="1:112" x14ac:dyDescent="0.3">
       <c r="A42" s="8"/>
       <c r="B42" s="8"/>
       <c r="C42" s="8"/>
@@ -9397,8 +10914,24 @@
       <c r="CP42" s="8"/>
       <c r="CQ42" s="8"/>
       <c r="CR42" s="8"/>
+      <c r="CS42" s="8"/>
+      <c r="CT42" s="8"/>
+      <c r="CU42" s="8"/>
+      <c r="CV42" s="8"/>
+      <c r="CW42" s="8"/>
+      <c r="CX42" s="8"/>
+      <c r="CY42" s="8"/>
+      <c r="CZ42" s="8"/>
+      <c r="DA42" s="8"/>
+      <c r="DB42" s="8"/>
+      <c r="DC42" s="8"/>
+      <c r="DD42" s="8"/>
+      <c r="DE42" s="8"/>
+      <c r="DF42" s="8"/>
+      <c r="DG42" s="8"/>
+      <c r="DH42" s="8"/>
     </row>
-    <row r="43" spans="1:96" x14ac:dyDescent="0.3">
+    <row r="43" spans="1:112" x14ac:dyDescent="0.3">
       <c r="A43" s="8"/>
       <c r="B43" s="8"/>
       <c r="C43" s="8"/>
@@ -9495,8 +11028,24 @@
       <c r="CP43" s="8"/>
       <c r="CQ43" s="8"/>
       <c r="CR43" s="8"/>
+      <c r="CS43" s="8"/>
+      <c r="CT43" s="8"/>
+      <c r="CU43" s="8"/>
+      <c r="CV43" s="8"/>
+      <c r="CW43" s="8"/>
+      <c r="CX43" s="8"/>
+      <c r="CY43" s="8"/>
+      <c r="CZ43" s="8"/>
+      <c r="DA43" s="8"/>
+      <c r="DB43" s="8"/>
+      <c r="DC43" s="8"/>
+      <c r="DD43" s="8"/>
+      <c r="DE43" s="8"/>
+      <c r="DF43" s="8"/>
+      <c r="DG43" s="8"/>
+      <c r="DH43" s="8"/>
     </row>
-    <row r="44" spans="1:96" x14ac:dyDescent="0.3">
+    <row r="44" spans="1:112" x14ac:dyDescent="0.3">
       <c r="A44" s="8"/>
       <c r="B44" s="8"/>
       <c r="C44" s="8"/>
@@ -9593,8 +11142,24 @@
       <c r="CP44" s="8"/>
       <c r="CQ44" s="8"/>
       <c r="CR44" s="8"/>
+      <c r="CS44" s="8"/>
+      <c r="CT44" s="8"/>
+      <c r="CU44" s="8"/>
+      <c r="CV44" s="8"/>
+      <c r="CW44" s="8"/>
+      <c r="CX44" s="8"/>
+      <c r="CY44" s="8"/>
+      <c r="CZ44" s="8"/>
+      <c r="DA44" s="8"/>
+      <c r="DB44" s="8"/>
+      <c r="DC44" s="8"/>
+      <c r="DD44" s="8"/>
+      <c r="DE44" s="8"/>
+      <c r="DF44" s="8"/>
+      <c r="DG44" s="8"/>
+      <c r="DH44" s="8"/>
     </row>
-    <row r="45" spans="1:96" x14ac:dyDescent="0.3">
+    <row r="45" spans="1:112" x14ac:dyDescent="0.3">
       <c r="A45" s="8"/>
       <c r="B45" s="8"/>
       <c r="C45" s="8"/>
@@ -9691,8 +11256,24 @@
       <c r="CP45" s="8"/>
       <c r="CQ45" s="8"/>
       <c r="CR45" s="8"/>
+      <c r="CS45" s="8"/>
+      <c r="CT45" s="8"/>
+      <c r="CU45" s="8"/>
+      <c r="CV45" s="8"/>
+      <c r="CW45" s="8"/>
+      <c r="CX45" s="8"/>
+      <c r="CY45" s="8"/>
+      <c r="CZ45" s="8"/>
+      <c r="DA45" s="8"/>
+      <c r="DB45" s="8"/>
+      <c r="DC45" s="8"/>
+      <c r="DD45" s="8"/>
+      <c r="DE45" s="8"/>
+      <c r="DF45" s="8"/>
+      <c r="DG45" s="8"/>
+      <c r="DH45" s="8"/>
     </row>
-    <row r="46" spans="1:96" x14ac:dyDescent="0.3">
+    <row r="46" spans="1:112" x14ac:dyDescent="0.3">
       <c r="A46" s="8"/>
       <c r="B46" s="8"/>
       <c r="C46" s="8"/>
@@ -9789,8 +11370,24 @@
       <c r="CP46" s="8"/>
       <c r="CQ46" s="8"/>
       <c r="CR46" s="8"/>
+      <c r="CS46" s="8"/>
+      <c r="CT46" s="8"/>
+      <c r="CU46" s="8"/>
+      <c r="CV46" s="8"/>
+      <c r="CW46" s="8"/>
+      <c r="CX46" s="8"/>
+      <c r="CY46" s="8"/>
+      <c r="CZ46" s="8"/>
+      <c r="DA46" s="8"/>
+      <c r="DB46" s="8"/>
+      <c r="DC46" s="8"/>
+      <c r="DD46" s="8"/>
+      <c r="DE46" s="8"/>
+      <c r="DF46" s="8"/>
+      <c r="DG46" s="8"/>
+      <c r="DH46" s="8"/>
     </row>
-    <row r="47" spans="1:96" x14ac:dyDescent="0.3">
+    <row r="47" spans="1:112" x14ac:dyDescent="0.3">
       <c r="A47" s="8"/>
       <c r="B47" s="8"/>
       <c r="C47" s="8"/>
@@ -9887,8 +11484,24 @@
       <c r="CP47" s="8"/>
       <c r="CQ47" s="8"/>
       <c r="CR47" s="8"/>
+      <c r="CS47" s="8"/>
+      <c r="CT47" s="8"/>
+      <c r="CU47" s="8"/>
+      <c r="CV47" s="8"/>
+      <c r="CW47" s="8"/>
+      <c r="CX47" s="8"/>
+      <c r="CY47" s="8"/>
+      <c r="CZ47" s="8"/>
+      <c r="DA47" s="8"/>
+      <c r="DB47" s="8"/>
+      <c r="DC47" s="8"/>
+      <c r="DD47" s="8"/>
+      <c r="DE47" s="8"/>
+      <c r="DF47" s="8"/>
+      <c r="DG47" s="8"/>
+      <c r="DH47" s="8"/>
     </row>
-    <row r="48" spans="1:96" x14ac:dyDescent="0.3">
+    <row r="48" spans="1:112" x14ac:dyDescent="0.3">
       <c r="A48" s="8"/>
       <c r="B48" s="8"/>
       <c r="C48" s="8"/>
@@ -9985,8 +11598,24 @@
       <c r="CP48" s="8"/>
       <c r="CQ48" s="8"/>
       <c r="CR48" s="8"/>
+      <c r="CS48" s="8"/>
+      <c r="CT48" s="8"/>
+      <c r="CU48" s="8"/>
+      <c r="CV48" s="8"/>
+      <c r="CW48" s="8"/>
+      <c r="CX48" s="8"/>
+      <c r="CY48" s="8"/>
+      <c r="CZ48" s="8"/>
+      <c r="DA48" s="8"/>
+      <c r="DB48" s="8"/>
+      <c r="DC48" s="8"/>
+      <c r="DD48" s="8"/>
+      <c r="DE48" s="8"/>
+      <c r="DF48" s="8"/>
+      <c r="DG48" s="8"/>
+      <c r="DH48" s="8"/>
     </row>
-    <row r="49" spans="1:96" x14ac:dyDescent="0.3">
+    <row r="49" spans="1:112" x14ac:dyDescent="0.3">
       <c r="A49" s="8"/>
       <c r="B49" s="8"/>
       <c r="C49" s="8"/>
@@ -10083,8 +11712,24 @@
       <c r="CP49" s="8"/>
       <c r="CQ49" s="8"/>
       <c r="CR49" s="8"/>
+      <c r="CS49" s="8"/>
+      <c r="CT49" s="8"/>
+      <c r="CU49" s="8"/>
+      <c r="CV49" s="8"/>
+      <c r="CW49" s="8"/>
+      <c r="CX49" s="8"/>
+      <c r="CY49" s="8"/>
+      <c r="CZ49" s="8"/>
+      <c r="DA49" s="8"/>
+      <c r="DB49" s="8"/>
+      <c r="DC49" s="8"/>
+      <c r="DD49" s="8"/>
+      <c r="DE49" s="8"/>
+      <c r="DF49" s="8"/>
+      <c r="DG49" s="8"/>
+      <c r="DH49" s="8"/>
     </row>
-    <row r="50" spans="1:96" x14ac:dyDescent="0.3">
+    <row r="50" spans="1:112" x14ac:dyDescent="0.3">
       <c r="A50" s="8"/>
       <c r="B50" s="8"/>
       <c r="C50" s="8"/>
@@ -10181,8 +11826,24 @@
       <c r="CP50" s="8"/>
       <c r="CQ50" s="8"/>
       <c r="CR50" s="8"/>
+      <c r="CS50" s="8"/>
+      <c r="CT50" s="8"/>
+      <c r="CU50" s="8"/>
+      <c r="CV50" s="8"/>
+      <c r="CW50" s="8"/>
+      <c r="CX50" s="8"/>
+      <c r="CY50" s="8"/>
+      <c r="CZ50" s="8"/>
+      <c r="DA50" s="8"/>
+      <c r="DB50" s="8"/>
+      <c r="DC50" s="8"/>
+      <c r="DD50" s="8"/>
+      <c r="DE50" s="8"/>
+      <c r="DF50" s="8"/>
+      <c r="DG50" s="8"/>
+      <c r="DH50" s="8"/>
     </row>
-    <row r="51" spans="1:96" x14ac:dyDescent="0.3">
+    <row r="51" spans="1:112" x14ac:dyDescent="0.3">
       <c r="A51" s="5" t="s">
         <v>6</v>
       </c>
@@ -10327,8 +11988,32 @@
       <c r="CP51" s="6"/>
       <c r="CQ51" s="6"/>
       <c r="CR51" s="6"/>
+      <c r="CS51" s="5" t="s">
+        <v>241</v>
+      </c>
+      <c r="CT51" s="6"/>
+      <c r="CU51" s="6"/>
+      <c r="CV51" s="6"/>
+      <c r="CW51" s="5" t="s">
+        <v>240</v>
+      </c>
+      <c r="CX51" s="6"/>
+      <c r="CY51" s="6"/>
+      <c r="CZ51" s="6"/>
+      <c r="DA51" s="5" t="s">
+        <v>262</v>
+      </c>
+      <c r="DB51" s="6"/>
+      <c r="DC51" s="6"/>
+      <c r="DD51" s="6"/>
+      <c r="DE51" s="5" t="s">
+        <v>260</v>
+      </c>
+      <c r="DF51" s="6"/>
+      <c r="DG51" s="6"/>
+      <c r="DH51" s="6"/>
     </row>
-    <row r="52" spans="1:96" x14ac:dyDescent="0.3">
+    <row r="52" spans="1:112" x14ac:dyDescent="0.3">
       <c r="A52" s="6"/>
       <c r="B52" s="6"/>
       <c r="C52" s="6"/>
@@ -10425,8 +12110,24 @@
       <c r="CP52" s="6"/>
       <c r="CQ52" s="6"/>
       <c r="CR52" s="6"/>
+      <c r="CS52" s="6"/>
+      <c r="CT52" s="6"/>
+      <c r="CU52" s="6"/>
+      <c r="CV52" s="6"/>
+      <c r="CW52" s="6"/>
+      <c r="CX52" s="6"/>
+      <c r="CY52" s="6"/>
+      <c r="CZ52" s="6"/>
+      <c r="DA52" s="6"/>
+      <c r="DB52" s="6"/>
+      <c r="DC52" s="6"/>
+      <c r="DD52" s="6"/>
+      <c r="DE52" s="6"/>
+      <c r="DF52" s="6"/>
+      <c r="DG52" s="6"/>
+      <c r="DH52" s="6"/>
     </row>
-    <row r="53" spans="1:96" x14ac:dyDescent="0.3">
+    <row r="53" spans="1:112" x14ac:dyDescent="0.3">
       <c r="A53" s="6"/>
       <c r="B53" s="6"/>
       <c r="C53" s="6"/>
@@ -10523,8 +12224,24 @@
       <c r="CP53" s="6"/>
       <c r="CQ53" s="6"/>
       <c r="CR53" s="6"/>
+      <c r="CS53" s="6"/>
+      <c r="CT53" s="6"/>
+      <c r="CU53" s="6"/>
+      <c r="CV53" s="6"/>
+      <c r="CW53" s="6"/>
+      <c r="CX53" s="6"/>
+      <c r="CY53" s="6"/>
+      <c r="CZ53" s="6"/>
+      <c r="DA53" s="6"/>
+      <c r="DB53" s="6"/>
+      <c r="DC53" s="6"/>
+      <c r="DD53" s="6"/>
+      <c r="DE53" s="6"/>
+      <c r="DF53" s="6"/>
+      <c r="DG53" s="6"/>
+      <c r="DH53" s="6"/>
     </row>
-    <row r="54" spans="1:96" x14ac:dyDescent="0.3">
+    <row r="54" spans="1:112" x14ac:dyDescent="0.3">
       <c r="A54" s="6"/>
       <c r="B54" s="6"/>
       <c r="C54" s="6"/>
@@ -10621,8 +12338,24 @@
       <c r="CP54" s="6"/>
       <c r="CQ54" s="6"/>
       <c r="CR54" s="6"/>
+      <c r="CS54" s="6"/>
+      <c r="CT54" s="6"/>
+      <c r="CU54" s="6"/>
+      <c r="CV54" s="6"/>
+      <c r="CW54" s="6"/>
+      <c r="CX54" s="6"/>
+      <c r="CY54" s="6"/>
+      <c r="CZ54" s="6"/>
+      <c r="DA54" s="6"/>
+      <c r="DB54" s="6"/>
+      <c r="DC54" s="6"/>
+      <c r="DD54" s="6"/>
+      <c r="DE54" s="6"/>
+      <c r="DF54" s="6"/>
+      <c r="DG54" s="6"/>
+      <c r="DH54" s="6"/>
     </row>
-    <row r="55" spans="1:96" x14ac:dyDescent="0.3">
+    <row r="55" spans="1:112" x14ac:dyDescent="0.3">
       <c r="A55" s="6"/>
       <c r="B55" s="6"/>
       <c r="C55" s="6"/>
@@ -10719,8 +12452,24 @@
       <c r="CP55" s="6"/>
       <c r="CQ55" s="6"/>
       <c r="CR55" s="6"/>
+      <c r="CS55" s="6"/>
+      <c r="CT55" s="6"/>
+      <c r="CU55" s="6"/>
+      <c r="CV55" s="6"/>
+      <c r="CW55" s="6"/>
+      <c r="CX55" s="6"/>
+      <c r="CY55" s="6"/>
+      <c r="CZ55" s="6"/>
+      <c r="DA55" s="6"/>
+      <c r="DB55" s="6"/>
+      <c r="DC55" s="6"/>
+      <c r="DD55" s="6"/>
+      <c r="DE55" s="6"/>
+      <c r="DF55" s="6"/>
+      <c r="DG55" s="6"/>
+      <c r="DH55" s="6"/>
     </row>
-    <row r="56" spans="1:96" x14ac:dyDescent="0.3">
+    <row r="56" spans="1:112" x14ac:dyDescent="0.3">
       <c r="A56" s="6"/>
       <c r="B56" s="6"/>
       <c r="C56" s="6"/>
@@ -10817,8 +12566,24 @@
       <c r="CP56" s="6"/>
       <c r="CQ56" s="6"/>
       <c r="CR56" s="6"/>
+      <c r="CS56" s="6"/>
+      <c r="CT56" s="6"/>
+      <c r="CU56" s="6"/>
+      <c r="CV56" s="6"/>
+      <c r="CW56" s="6"/>
+      <c r="CX56" s="6"/>
+      <c r="CY56" s="6"/>
+      <c r="CZ56" s="6"/>
+      <c r="DA56" s="6"/>
+      <c r="DB56" s="6"/>
+      <c r="DC56" s="6"/>
+      <c r="DD56" s="6"/>
+      <c r="DE56" s="6"/>
+      <c r="DF56" s="6"/>
+      <c r="DG56" s="6"/>
+      <c r="DH56" s="6"/>
     </row>
-    <row r="57" spans="1:96" x14ac:dyDescent="0.3">
+    <row r="57" spans="1:112" x14ac:dyDescent="0.3">
       <c r="A57" s="6"/>
       <c r="B57" s="6"/>
       <c r="C57" s="6"/>
@@ -10915,8 +12680,24 @@
       <c r="CP57" s="6"/>
       <c r="CQ57" s="6"/>
       <c r="CR57" s="6"/>
+      <c r="CS57" s="6"/>
+      <c r="CT57" s="6"/>
+      <c r="CU57" s="6"/>
+      <c r="CV57" s="6"/>
+      <c r="CW57" s="6"/>
+      <c r="CX57" s="6"/>
+      <c r="CY57" s="6"/>
+      <c r="CZ57" s="6"/>
+      <c r="DA57" s="6"/>
+      <c r="DB57" s="6"/>
+      <c r="DC57" s="6"/>
+      <c r="DD57" s="6"/>
+      <c r="DE57" s="6"/>
+      <c r="DF57" s="6"/>
+      <c r="DG57" s="6"/>
+      <c r="DH57" s="6"/>
     </row>
-    <row r="58" spans="1:96" x14ac:dyDescent="0.3">
+    <row r="58" spans="1:112" x14ac:dyDescent="0.3">
       <c r="A58" s="6"/>
       <c r="B58" s="6"/>
       <c r="C58" s="6"/>
@@ -11013,8 +12794,24 @@
       <c r="CP58" s="6"/>
       <c r="CQ58" s="6"/>
       <c r="CR58" s="6"/>
+      <c r="CS58" s="6"/>
+      <c r="CT58" s="6"/>
+      <c r="CU58" s="6"/>
+      <c r="CV58" s="6"/>
+      <c r="CW58" s="6"/>
+      <c r="CX58" s="6"/>
+      <c r="CY58" s="6"/>
+      <c r="CZ58" s="6"/>
+      <c r="DA58" s="6"/>
+      <c r="DB58" s="6"/>
+      <c r="DC58" s="6"/>
+      <c r="DD58" s="6"/>
+      <c r="DE58" s="6"/>
+      <c r="DF58" s="6"/>
+      <c r="DG58" s="6"/>
+      <c r="DH58" s="6"/>
     </row>
-    <row r="59" spans="1:96" x14ac:dyDescent="0.3">
+    <row r="59" spans="1:112" x14ac:dyDescent="0.3">
       <c r="A59" s="6"/>
       <c r="B59" s="6"/>
       <c r="C59" s="6"/>
@@ -11111,8 +12908,24 @@
       <c r="CP59" s="6"/>
       <c r="CQ59" s="6"/>
       <c r="CR59" s="6"/>
+      <c r="CS59" s="6"/>
+      <c r="CT59" s="6"/>
+      <c r="CU59" s="6"/>
+      <c r="CV59" s="6"/>
+      <c r="CW59" s="6"/>
+      <c r="CX59" s="6"/>
+      <c r="CY59" s="6"/>
+      <c r="CZ59" s="6"/>
+      <c r="DA59" s="6"/>
+      <c r="DB59" s="6"/>
+      <c r="DC59" s="6"/>
+      <c r="DD59" s="6"/>
+      <c r="DE59" s="6"/>
+      <c r="DF59" s="6"/>
+      <c r="DG59" s="6"/>
+      <c r="DH59" s="6"/>
     </row>
-    <row r="60" spans="1:96" x14ac:dyDescent="0.3">
+    <row r="60" spans="1:112" x14ac:dyDescent="0.3">
       <c r="A60" s="6"/>
       <c r="B60" s="6"/>
       <c r="C60" s="6"/>
@@ -11209,8 +13022,24 @@
       <c r="CP60" s="6"/>
       <c r="CQ60" s="6"/>
       <c r="CR60" s="6"/>
+      <c r="CS60" s="6"/>
+      <c r="CT60" s="6"/>
+      <c r="CU60" s="6"/>
+      <c r="CV60" s="6"/>
+      <c r="CW60" s="6"/>
+      <c r="CX60" s="6"/>
+      <c r="CY60" s="6"/>
+      <c r="CZ60" s="6"/>
+      <c r="DA60" s="6"/>
+      <c r="DB60" s="6"/>
+      <c r="DC60" s="6"/>
+      <c r="DD60" s="6"/>
+      <c r="DE60" s="6"/>
+      <c r="DF60" s="6"/>
+      <c r="DG60" s="6"/>
+      <c r="DH60" s="6"/>
     </row>
-    <row r="61" spans="1:96" x14ac:dyDescent="0.3">
+    <row r="61" spans="1:112" x14ac:dyDescent="0.3">
       <c r="A61" s="5" t="s">
         <v>8</v>
       </c>
@@ -11355,8 +13184,32 @@
       <c r="CP61" s="6"/>
       <c r="CQ61" s="6"/>
       <c r="CR61" s="6"/>
+      <c r="CS61" s="5" t="s">
+        <v>245</v>
+      </c>
+      <c r="CT61" s="6"/>
+      <c r="CU61" s="6"/>
+      <c r="CV61" s="6"/>
+      <c r="CW61" s="5" t="s">
+        <v>243</v>
+      </c>
+      <c r="CX61" s="6"/>
+      <c r="CY61" s="6"/>
+      <c r="CZ61" s="6"/>
+      <c r="DA61" s="5" t="s">
+        <v>266</v>
+      </c>
+      <c r="DB61" s="6"/>
+      <c r="DC61" s="6"/>
+      <c r="DD61" s="6"/>
+      <c r="DE61" s="5" t="s">
+        <v>264</v>
+      </c>
+      <c r="DF61" s="6"/>
+      <c r="DG61" s="6"/>
+      <c r="DH61" s="6"/>
     </row>
-    <row r="62" spans="1:96" x14ac:dyDescent="0.3">
+    <row r="62" spans="1:112" x14ac:dyDescent="0.3">
       <c r="A62" s="6"/>
       <c r="B62" s="6"/>
       <c r="C62" s="6"/>
@@ -11453,8 +13306,24 @@
       <c r="CP62" s="6"/>
       <c r="CQ62" s="6"/>
       <c r="CR62" s="6"/>
+      <c r="CS62" s="6"/>
+      <c r="CT62" s="6"/>
+      <c r="CU62" s="6"/>
+      <c r="CV62" s="6"/>
+      <c r="CW62" s="6"/>
+      <c r="CX62" s="6"/>
+      <c r="CY62" s="6"/>
+      <c r="CZ62" s="6"/>
+      <c r="DA62" s="6"/>
+      <c r="DB62" s="6"/>
+      <c r="DC62" s="6"/>
+      <c r="DD62" s="6"/>
+      <c r="DE62" s="6"/>
+      <c r="DF62" s="6"/>
+      <c r="DG62" s="6"/>
+      <c r="DH62" s="6"/>
     </row>
-    <row r="63" spans="1:96" x14ac:dyDescent="0.3">
+    <row r="63" spans="1:112" x14ac:dyDescent="0.3">
       <c r="A63" s="6"/>
       <c r="B63" s="6"/>
       <c r="C63" s="6"/>
@@ -11551,8 +13420,24 @@
       <c r="CP63" s="6"/>
       <c r="CQ63" s="6"/>
       <c r="CR63" s="6"/>
+      <c r="CS63" s="6"/>
+      <c r="CT63" s="6"/>
+      <c r="CU63" s="6"/>
+      <c r="CV63" s="6"/>
+      <c r="CW63" s="6"/>
+      <c r="CX63" s="6"/>
+      <c r="CY63" s="6"/>
+      <c r="CZ63" s="6"/>
+      <c r="DA63" s="6"/>
+      <c r="DB63" s="6"/>
+      <c r="DC63" s="6"/>
+      <c r="DD63" s="6"/>
+      <c r="DE63" s="6"/>
+      <c r="DF63" s="6"/>
+      <c r="DG63" s="6"/>
+      <c r="DH63" s="6"/>
     </row>
-    <row r="64" spans="1:96" x14ac:dyDescent="0.3">
+    <row r="64" spans="1:112" x14ac:dyDescent="0.3">
       <c r="A64" s="6"/>
       <c r="B64" s="6"/>
       <c r="C64" s="6"/>
@@ -11649,8 +13534,24 @@
       <c r="CP64" s="6"/>
       <c r="CQ64" s="6"/>
       <c r="CR64" s="6"/>
+      <c r="CS64" s="6"/>
+      <c r="CT64" s="6"/>
+      <c r="CU64" s="6"/>
+      <c r="CV64" s="6"/>
+      <c r="CW64" s="6"/>
+      <c r="CX64" s="6"/>
+      <c r="CY64" s="6"/>
+      <c r="CZ64" s="6"/>
+      <c r="DA64" s="6"/>
+      <c r="DB64" s="6"/>
+      <c r="DC64" s="6"/>
+      <c r="DD64" s="6"/>
+      <c r="DE64" s="6"/>
+      <c r="DF64" s="6"/>
+      <c r="DG64" s="6"/>
+      <c r="DH64" s="6"/>
     </row>
-    <row r="65" spans="1:96" x14ac:dyDescent="0.3">
+    <row r="65" spans="1:112" x14ac:dyDescent="0.3">
       <c r="A65" s="6"/>
       <c r="B65" s="6"/>
       <c r="C65" s="6"/>
@@ -11747,8 +13648,24 @@
       <c r="CP65" s="6"/>
       <c r="CQ65" s="6"/>
       <c r="CR65" s="6"/>
+      <c r="CS65" s="6"/>
+      <c r="CT65" s="6"/>
+      <c r="CU65" s="6"/>
+      <c r="CV65" s="6"/>
+      <c r="CW65" s="6"/>
+      <c r="CX65" s="6"/>
+      <c r="CY65" s="6"/>
+      <c r="CZ65" s="6"/>
+      <c r="DA65" s="6"/>
+      <c r="DB65" s="6"/>
+      <c r="DC65" s="6"/>
+      <c r="DD65" s="6"/>
+      <c r="DE65" s="6"/>
+      <c r="DF65" s="6"/>
+      <c r="DG65" s="6"/>
+      <c r="DH65" s="6"/>
     </row>
-    <row r="66" spans="1:96" x14ac:dyDescent="0.3">
+    <row r="66" spans="1:112" x14ac:dyDescent="0.3">
       <c r="A66" s="6"/>
       <c r="B66" s="6"/>
       <c r="C66" s="6"/>
@@ -11845,8 +13762,24 @@
       <c r="CP66" s="6"/>
       <c r="CQ66" s="6"/>
       <c r="CR66" s="6"/>
+      <c r="CS66" s="6"/>
+      <c r="CT66" s="6"/>
+      <c r="CU66" s="6"/>
+      <c r="CV66" s="6"/>
+      <c r="CW66" s="6"/>
+      <c r="CX66" s="6"/>
+      <c r="CY66" s="6"/>
+      <c r="CZ66" s="6"/>
+      <c r="DA66" s="6"/>
+      <c r="DB66" s="6"/>
+      <c r="DC66" s="6"/>
+      <c r="DD66" s="6"/>
+      <c r="DE66" s="6"/>
+      <c r="DF66" s="6"/>
+      <c r="DG66" s="6"/>
+      <c r="DH66" s="6"/>
     </row>
-    <row r="67" spans="1:96" x14ac:dyDescent="0.3">
+    <row r="67" spans="1:112" x14ac:dyDescent="0.3">
       <c r="A67" s="6"/>
       <c r="B67" s="6"/>
       <c r="C67" s="6"/>
@@ -11943,8 +13876,24 @@
       <c r="CP67" s="6"/>
       <c r="CQ67" s="6"/>
       <c r="CR67" s="6"/>
+      <c r="CS67" s="6"/>
+      <c r="CT67" s="6"/>
+      <c r="CU67" s="6"/>
+      <c r="CV67" s="6"/>
+      <c r="CW67" s="6"/>
+      <c r="CX67" s="6"/>
+      <c r="CY67" s="6"/>
+      <c r="CZ67" s="6"/>
+      <c r="DA67" s="6"/>
+      <c r="DB67" s="6"/>
+      <c r="DC67" s="6"/>
+      <c r="DD67" s="6"/>
+      <c r="DE67" s="6"/>
+      <c r="DF67" s="6"/>
+      <c r="DG67" s="6"/>
+      <c r="DH67" s="6"/>
     </row>
-    <row r="68" spans="1:96" x14ac:dyDescent="0.3">
+    <row r="68" spans="1:112" x14ac:dyDescent="0.3">
       <c r="A68" s="6"/>
       <c r="B68" s="6"/>
       <c r="C68" s="6"/>
@@ -12041,8 +13990,24 @@
       <c r="CP68" s="6"/>
       <c r="CQ68" s="6"/>
       <c r="CR68" s="6"/>
+      <c r="CS68" s="6"/>
+      <c r="CT68" s="6"/>
+      <c r="CU68" s="6"/>
+      <c r="CV68" s="6"/>
+      <c r="CW68" s="6"/>
+      <c r="CX68" s="6"/>
+      <c r="CY68" s="6"/>
+      <c r="CZ68" s="6"/>
+      <c r="DA68" s="6"/>
+      <c r="DB68" s="6"/>
+      <c r="DC68" s="6"/>
+      <c r="DD68" s="6"/>
+      <c r="DE68" s="6"/>
+      <c r="DF68" s="6"/>
+      <c r="DG68" s="6"/>
+      <c r="DH68" s="6"/>
     </row>
-    <row r="69" spans="1:96" x14ac:dyDescent="0.3">
+    <row r="69" spans="1:112" x14ac:dyDescent="0.3">
       <c r="A69" s="6"/>
       <c r="B69" s="6"/>
       <c r="C69" s="6"/>
@@ -12139,8 +14104,24 @@
       <c r="CP69" s="6"/>
       <c r="CQ69" s="6"/>
       <c r="CR69" s="6"/>
+      <c r="CS69" s="6"/>
+      <c r="CT69" s="6"/>
+      <c r="CU69" s="6"/>
+      <c r="CV69" s="6"/>
+      <c r="CW69" s="6"/>
+      <c r="CX69" s="6"/>
+      <c r="CY69" s="6"/>
+      <c r="CZ69" s="6"/>
+      <c r="DA69" s="6"/>
+      <c r="DB69" s="6"/>
+      <c r="DC69" s="6"/>
+      <c r="DD69" s="6"/>
+      <c r="DE69" s="6"/>
+      <c r="DF69" s="6"/>
+      <c r="DG69" s="6"/>
+      <c r="DH69" s="6"/>
     </row>
-    <row r="70" spans="1:96" x14ac:dyDescent="0.3">
+    <row r="70" spans="1:112" x14ac:dyDescent="0.3">
       <c r="A70" s="6"/>
       <c r="B70" s="6"/>
       <c r="C70" s="6"/>
@@ -12237,8 +14218,24 @@
       <c r="CP70" s="6"/>
       <c r="CQ70" s="6"/>
       <c r="CR70" s="6"/>
+      <c r="CS70" s="6"/>
+      <c r="CT70" s="6"/>
+      <c r="CU70" s="6"/>
+      <c r="CV70" s="6"/>
+      <c r="CW70" s="6"/>
+      <c r="CX70" s="6"/>
+      <c r="CY70" s="6"/>
+      <c r="CZ70" s="6"/>
+      <c r="DA70" s="6"/>
+      <c r="DB70" s="6"/>
+      <c r="DC70" s="6"/>
+      <c r="DD70" s="6"/>
+      <c r="DE70" s="6"/>
+      <c r="DF70" s="6"/>
+      <c r="DG70" s="6"/>
+      <c r="DH70" s="6"/>
     </row>
-    <row r="71" spans="1:96" ht="14.4" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="71" spans="1:112" ht="14.4" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A71" s="5" t="s">
         <v>11</v>
       </c>
@@ -12383,8 +14380,30 @@
       <c r="CP71" s="6"/>
       <c r="CQ71" s="6"/>
       <c r="CR71" s="6"/>
+      <c r="CS71" s="5" t="s">
+        <v>250</v>
+      </c>
+      <c r="CT71" s="6"/>
+      <c r="CU71" s="6"/>
+      <c r="CV71" s="6"/>
+      <c r="CW71" s="5" t="s">
+        <v>248</v>
+      </c>
+      <c r="CX71" s="6"/>
+      <c r="CY71" s="6"/>
+      <c r="CZ71" s="6"/>
+      <c r="DA71" s="5"/>
+      <c r="DB71" s="6"/>
+      <c r="DC71" s="6"/>
+      <c r="DD71" s="6"/>
+      <c r="DE71" s="5" t="s">
+        <v>268</v>
+      </c>
+      <c r="DF71" s="6"/>
+      <c r="DG71" s="6"/>
+      <c r="DH71" s="6"/>
     </row>
-    <row r="72" spans="1:96" x14ac:dyDescent="0.3">
+    <row r="72" spans="1:112" x14ac:dyDescent="0.3">
       <c r="A72" s="6"/>
       <c r="B72" s="6"/>
       <c r="C72" s="6"/>
@@ -12481,8 +14500,24 @@
       <c r="CP72" s="6"/>
       <c r="CQ72" s="6"/>
       <c r="CR72" s="6"/>
+      <c r="CS72" s="6"/>
+      <c r="CT72" s="6"/>
+      <c r="CU72" s="6"/>
+      <c r="CV72" s="6"/>
+      <c r="CW72" s="6"/>
+      <c r="CX72" s="6"/>
+      <c r="CY72" s="6"/>
+      <c r="CZ72" s="6"/>
+      <c r="DA72" s="6"/>
+      <c r="DB72" s="6"/>
+      <c r="DC72" s="6"/>
+      <c r="DD72" s="6"/>
+      <c r="DE72" s="6"/>
+      <c r="DF72" s="6"/>
+      <c r="DG72" s="6"/>
+      <c r="DH72" s="6"/>
     </row>
-    <row r="73" spans="1:96" x14ac:dyDescent="0.3">
+    <row r="73" spans="1:112" x14ac:dyDescent="0.3">
       <c r="A73" s="6"/>
       <c r="B73" s="6"/>
       <c r="C73" s="6"/>
@@ -12579,8 +14614,24 @@
       <c r="CP73" s="6"/>
       <c r="CQ73" s="6"/>
       <c r="CR73" s="6"/>
+      <c r="CS73" s="6"/>
+      <c r="CT73" s="6"/>
+      <c r="CU73" s="6"/>
+      <c r="CV73" s="6"/>
+      <c r="CW73" s="6"/>
+      <c r="CX73" s="6"/>
+      <c r="CY73" s="6"/>
+      <c r="CZ73" s="6"/>
+      <c r="DA73" s="6"/>
+      <c r="DB73" s="6"/>
+      <c r="DC73" s="6"/>
+      <c r="DD73" s="6"/>
+      <c r="DE73" s="6"/>
+      <c r="DF73" s="6"/>
+      <c r="DG73" s="6"/>
+      <c r="DH73" s="6"/>
     </row>
-    <row r="74" spans="1:96" x14ac:dyDescent="0.3">
+    <row r="74" spans="1:112" x14ac:dyDescent="0.3">
       <c r="A74" s="6"/>
       <c r="B74" s="6"/>
       <c r="C74" s="6"/>
@@ -12677,8 +14728,24 @@
       <c r="CP74" s="6"/>
       <c r="CQ74" s="6"/>
       <c r="CR74" s="6"/>
+      <c r="CS74" s="6"/>
+      <c r="CT74" s="6"/>
+      <c r="CU74" s="6"/>
+      <c r="CV74" s="6"/>
+      <c r="CW74" s="6"/>
+      <c r="CX74" s="6"/>
+      <c r="CY74" s="6"/>
+      <c r="CZ74" s="6"/>
+      <c r="DA74" s="6"/>
+      <c r="DB74" s="6"/>
+      <c r="DC74" s="6"/>
+      <c r="DD74" s="6"/>
+      <c r="DE74" s="6"/>
+      <c r="DF74" s="6"/>
+      <c r="DG74" s="6"/>
+      <c r="DH74" s="6"/>
     </row>
-    <row r="75" spans="1:96" x14ac:dyDescent="0.3">
+    <row r="75" spans="1:112" x14ac:dyDescent="0.3">
       <c r="A75" s="6"/>
       <c r="B75" s="6"/>
       <c r="C75" s="6"/>
@@ -12775,8 +14842,24 @@
       <c r="CP75" s="6"/>
       <c r="CQ75" s="6"/>
       <c r="CR75" s="6"/>
+      <c r="CS75" s="6"/>
+      <c r="CT75" s="6"/>
+      <c r="CU75" s="6"/>
+      <c r="CV75" s="6"/>
+      <c r="CW75" s="6"/>
+      <c r="CX75" s="6"/>
+      <c r="CY75" s="6"/>
+      <c r="CZ75" s="6"/>
+      <c r="DA75" s="6"/>
+      <c r="DB75" s="6"/>
+      <c r="DC75" s="6"/>
+      <c r="DD75" s="6"/>
+      <c r="DE75" s="6"/>
+      <c r="DF75" s="6"/>
+      <c r="DG75" s="6"/>
+      <c r="DH75" s="6"/>
     </row>
-    <row r="76" spans="1:96" x14ac:dyDescent="0.3">
+    <row r="76" spans="1:112" x14ac:dyDescent="0.3">
       <c r="A76" s="6"/>
       <c r="B76" s="6"/>
       <c r="C76" s="6"/>
@@ -12873,8 +14956,24 @@
       <c r="CP76" s="6"/>
       <c r="CQ76" s="6"/>
       <c r="CR76" s="6"/>
+      <c r="CS76" s="6"/>
+      <c r="CT76" s="6"/>
+      <c r="CU76" s="6"/>
+      <c r="CV76" s="6"/>
+      <c r="CW76" s="6"/>
+      <c r="CX76" s="6"/>
+      <c r="CY76" s="6"/>
+      <c r="CZ76" s="6"/>
+      <c r="DA76" s="6"/>
+      <c r="DB76" s="6"/>
+      <c r="DC76" s="6"/>
+      <c r="DD76" s="6"/>
+      <c r="DE76" s="6"/>
+      <c r="DF76" s="6"/>
+      <c r="DG76" s="6"/>
+      <c r="DH76" s="6"/>
     </row>
-    <row r="77" spans="1:96" x14ac:dyDescent="0.3">
+    <row r="77" spans="1:112" x14ac:dyDescent="0.3">
       <c r="A77" s="6"/>
       <c r="B77" s="6"/>
       <c r="C77" s="6"/>
@@ -12971,8 +15070,24 @@
       <c r="CP77" s="6"/>
       <c r="CQ77" s="6"/>
       <c r="CR77" s="6"/>
+      <c r="CS77" s="6"/>
+      <c r="CT77" s="6"/>
+      <c r="CU77" s="6"/>
+      <c r="CV77" s="6"/>
+      <c r="CW77" s="6"/>
+      <c r="CX77" s="6"/>
+      <c r="CY77" s="6"/>
+      <c r="CZ77" s="6"/>
+      <c r="DA77" s="6"/>
+      <c r="DB77" s="6"/>
+      <c r="DC77" s="6"/>
+      <c r="DD77" s="6"/>
+      <c r="DE77" s="6"/>
+      <c r="DF77" s="6"/>
+      <c r="DG77" s="6"/>
+      <c r="DH77" s="6"/>
     </row>
-    <row r="78" spans="1:96" x14ac:dyDescent="0.3">
+    <row r="78" spans="1:112" x14ac:dyDescent="0.3">
       <c r="A78" s="6"/>
       <c r="B78" s="6"/>
       <c r="C78" s="6"/>
@@ -13069,8 +15184,24 @@
       <c r="CP78" s="6"/>
       <c r="CQ78" s="6"/>
       <c r="CR78" s="6"/>
+      <c r="CS78" s="6"/>
+      <c r="CT78" s="6"/>
+      <c r="CU78" s="6"/>
+      <c r="CV78" s="6"/>
+      <c r="CW78" s="6"/>
+      <c r="CX78" s="6"/>
+      <c r="CY78" s="6"/>
+      <c r="CZ78" s="6"/>
+      <c r="DA78" s="6"/>
+      <c r="DB78" s="6"/>
+      <c r="DC78" s="6"/>
+      <c r="DD78" s="6"/>
+      <c r="DE78" s="6"/>
+      <c r="DF78" s="6"/>
+      <c r="DG78" s="6"/>
+      <c r="DH78" s="6"/>
     </row>
-    <row r="79" spans="1:96" x14ac:dyDescent="0.3">
+    <row r="79" spans="1:112" x14ac:dyDescent="0.3">
       <c r="A79" s="6"/>
       <c r="B79" s="6"/>
       <c r="C79" s="6"/>
@@ -13167,8 +15298,24 @@
       <c r="CP79" s="6"/>
       <c r="CQ79" s="6"/>
       <c r="CR79" s="6"/>
+      <c r="CS79" s="6"/>
+      <c r="CT79" s="6"/>
+      <c r="CU79" s="6"/>
+      <c r="CV79" s="6"/>
+      <c r="CW79" s="6"/>
+      <c r="CX79" s="6"/>
+      <c r="CY79" s="6"/>
+      <c r="CZ79" s="6"/>
+      <c r="DA79" s="6"/>
+      <c r="DB79" s="6"/>
+      <c r="DC79" s="6"/>
+      <c r="DD79" s="6"/>
+      <c r="DE79" s="6"/>
+      <c r="DF79" s="6"/>
+      <c r="DG79" s="6"/>
+      <c r="DH79" s="6"/>
     </row>
-    <row r="80" spans="1:96" x14ac:dyDescent="0.3">
+    <row r="80" spans="1:112" x14ac:dyDescent="0.3">
       <c r="A80" s="6"/>
       <c r="B80" s="6"/>
       <c r="C80" s="6"/>
@@ -13265,8 +15412,24 @@
       <c r="CP80" s="6"/>
       <c r="CQ80" s="6"/>
       <c r="CR80" s="6"/>
+      <c r="CS80" s="6"/>
+      <c r="CT80" s="6"/>
+      <c r="CU80" s="6"/>
+      <c r="CV80" s="6"/>
+      <c r="CW80" s="6"/>
+      <c r="CX80" s="6"/>
+      <c r="CY80" s="6"/>
+      <c r="CZ80" s="6"/>
+      <c r="DA80" s="6"/>
+      <c r="DB80" s="6"/>
+      <c r="DC80" s="6"/>
+      <c r="DD80" s="6"/>
+      <c r="DE80" s="6"/>
+      <c r="DF80" s="6"/>
+      <c r="DG80" s="6"/>
+      <c r="DH80" s="6"/>
     </row>
-    <row r="81" spans="1:96" x14ac:dyDescent="0.3">
+    <row r="81" spans="1:112" x14ac:dyDescent="0.3">
       <c r="A81" s="5" t="s">
         <v>15</v>
       </c>
@@ -13399,7 +15562,9 @@
       <c r="CH81" s="6"/>
       <c r="CI81" s="6"/>
       <c r="CJ81" s="6"/>
-      <c r="CK81" s="5"/>
+      <c r="CK81" s="5" t="s">
+        <v>234</v>
+      </c>
       <c r="CL81" s="6"/>
       <c r="CM81" s="6"/>
       <c r="CN81" s="6"/>
@@ -13409,8 +15574,28 @@
       <c r="CP81" s="6"/>
       <c r="CQ81" s="6"/>
       <c r="CR81" s="6"/>
+      <c r="CS81" s="5" t="s">
+        <v>251</v>
+      </c>
+      <c r="CT81" s="6"/>
+      <c r="CU81" s="6"/>
+      <c r="CV81" s="6"/>
+      <c r="CW81" s="5" t="s">
+        <v>254</v>
+      </c>
+      <c r="CX81" s="6"/>
+      <c r="CY81" s="6"/>
+      <c r="CZ81" s="6"/>
+      <c r="DA81" s="5"/>
+      <c r="DB81" s="6"/>
+      <c r="DC81" s="6"/>
+      <c r="DD81" s="6"/>
+      <c r="DE81" s="5"/>
+      <c r="DF81" s="6"/>
+      <c r="DG81" s="6"/>
+      <c r="DH81" s="6"/>
     </row>
-    <row r="82" spans="1:96" x14ac:dyDescent="0.3">
+    <row r="82" spans="1:112" x14ac:dyDescent="0.3">
       <c r="A82" s="6"/>
       <c r="B82" s="6"/>
       <c r="C82" s="6"/>
@@ -13507,8 +15692,24 @@
       <c r="CP82" s="6"/>
       <c r="CQ82" s="6"/>
       <c r="CR82" s="6"/>
+      <c r="CS82" s="6"/>
+      <c r="CT82" s="6"/>
+      <c r="CU82" s="6"/>
+      <c r="CV82" s="6"/>
+      <c r="CW82" s="6"/>
+      <c r="CX82" s="6"/>
+      <c r="CY82" s="6"/>
+      <c r="CZ82" s="6"/>
+      <c r="DA82" s="6"/>
+      <c r="DB82" s="6"/>
+      <c r="DC82" s="6"/>
+      <c r="DD82" s="6"/>
+      <c r="DE82" s="6"/>
+      <c r="DF82" s="6"/>
+      <c r="DG82" s="6"/>
+      <c r="DH82" s="6"/>
     </row>
-    <row r="83" spans="1:96" x14ac:dyDescent="0.3">
+    <row r="83" spans="1:112" x14ac:dyDescent="0.3">
       <c r="A83" s="6"/>
       <c r="B83" s="6"/>
       <c r="C83" s="6"/>
@@ -13605,8 +15806,24 @@
       <c r="CP83" s="6"/>
       <c r="CQ83" s="6"/>
       <c r="CR83" s="6"/>
+      <c r="CS83" s="6"/>
+      <c r="CT83" s="6"/>
+      <c r="CU83" s="6"/>
+      <c r="CV83" s="6"/>
+      <c r="CW83" s="6"/>
+      <c r="CX83" s="6"/>
+      <c r="CY83" s="6"/>
+      <c r="CZ83" s="6"/>
+      <c r="DA83" s="6"/>
+      <c r="DB83" s="6"/>
+      <c r="DC83" s="6"/>
+      <c r="DD83" s="6"/>
+      <c r="DE83" s="6"/>
+      <c r="DF83" s="6"/>
+      <c r="DG83" s="6"/>
+      <c r="DH83" s="6"/>
     </row>
-    <row r="84" spans="1:96" x14ac:dyDescent="0.3">
+    <row r="84" spans="1:112" x14ac:dyDescent="0.3">
       <c r="A84" s="6"/>
       <c r="B84" s="6"/>
       <c r="C84" s="6"/>
@@ -13703,8 +15920,24 @@
       <c r="CP84" s="6"/>
       <c r="CQ84" s="6"/>
       <c r="CR84" s="6"/>
+      <c r="CS84" s="6"/>
+      <c r="CT84" s="6"/>
+      <c r="CU84" s="6"/>
+      <c r="CV84" s="6"/>
+      <c r="CW84" s="6"/>
+      <c r="CX84" s="6"/>
+      <c r="CY84" s="6"/>
+      <c r="CZ84" s="6"/>
+      <c r="DA84" s="6"/>
+      <c r="DB84" s="6"/>
+      <c r="DC84" s="6"/>
+      <c r="DD84" s="6"/>
+      <c r="DE84" s="6"/>
+      <c r="DF84" s="6"/>
+      <c r="DG84" s="6"/>
+      <c r="DH84" s="6"/>
     </row>
-    <row r="85" spans="1:96" x14ac:dyDescent="0.3">
+    <row r="85" spans="1:112" x14ac:dyDescent="0.3">
       <c r="A85" s="6"/>
       <c r="B85" s="6"/>
       <c r="C85" s="6"/>
@@ -13801,8 +16034,24 @@
       <c r="CP85" s="6"/>
       <c r="CQ85" s="6"/>
       <c r="CR85" s="6"/>
+      <c r="CS85" s="6"/>
+      <c r="CT85" s="6"/>
+      <c r="CU85" s="6"/>
+      <c r="CV85" s="6"/>
+      <c r="CW85" s="6"/>
+      <c r="CX85" s="6"/>
+      <c r="CY85" s="6"/>
+      <c r="CZ85" s="6"/>
+      <c r="DA85" s="6"/>
+      <c r="DB85" s="6"/>
+      <c r="DC85" s="6"/>
+      <c r="DD85" s="6"/>
+      <c r="DE85" s="6"/>
+      <c r="DF85" s="6"/>
+      <c r="DG85" s="6"/>
+      <c r="DH85" s="6"/>
     </row>
-    <row r="86" spans="1:96" x14ac:dyDescent="0.3">
+    <row r="86" spans="1:112" x14ac:dyDescent="0.3">
       <c r="A86" s="6"/>
       <c r="B86" s="6"/>
       <c r="C86" s="6"/>
@@ -13899,8 +16148,24 @@
       <c r="CP86" s="6"/>
       <c r="CQ86" s="6"/>
       <c r="CR86" s="6"/>
+      <c r="CS86" s="6"/>
+      <c r="CT86" s="6"/>
+      <c r="CU86" s="6"/>
+      <c r="CV86" s="6"/>
+      <c r="CW86" s="6"/>
+      <c r="CX86" s="6"/>
+      <c r="CY86" s="6"/>
+      <c r="CZ86" s="6"/>
+      <c r="DA86" s="6"/>
+      <c r="DB86" s="6"/>
+      <c r="DC86" s="6"/>
+      <c r="DD86" s="6"/>
+      <c r="DE86" s="6"/>
+      <c r="DF86" s="6"/>
+      <c r="DG86" s="6"/>
+      <c r="DH86" s="6"/>
     </row>
-    <row r="87" spans="1:96" x14ac:dyDescent="0.3">
+    <row r="87" spans="1:112" x14ac:dyDescent="0.3">
       <c r="A87" s="6"/>
       <c r="B87" s="6"/>
       <c r="C87" s="6"/>
@@ -13997,8 +16262,24 @@
       <c r="CP87" s="6"/>
       <c r="CQ87" s="6"/>
       <c r="CR87" s="6"/>
+      <c r="CS87" s="6"/>
+      <c r="CT87" s="6"/>
+      <c r="CU87" s="6"/>
+      <c r="CV87" s="6"/>
+      <c r="CW87" s="6"/>
+      <c r="CX87" s="6"/>
+      <c r="CY87" s="6"/>
+      <c r="CZ87" s="6"/>
+      <c r="DA87" s="6"/>
+      <c r="DB87" s="6"/>
+      <c r="DC87" s="6"/>
+      <c r="DD87" s="6"/>
+      <c r="DE87" s="6"/>
+      <c r="DF87" s="6"/>
+      <c r="DG87" s="6"/>
+      <c r="DH87" s="6"/>
     </row>
-    <row r="88" spans="1:96" x14ac:dyDescent="0.3">
+    <row r="88" spans="1:112" x14ac:dyDescent="0.3">
       <c r="A88" s="6"/>
       <c r="B88" s="6"/>
       <c r="C88" s="6"/>
@@ -14095,8 +16376,24 @@
       <c r="CP88" s="6"/>
       <c r="CQ88" s="6"/>
       <c r="CR88" s="6"/>
+      <c r="CS88" s="6"/>
+      <c r="CT88" s="6"/>
+      <c r="CU88" s="6"/>
+      <c r="CV88" s="6"/>
+      <c r="CW88" s="6"/>
+      <c r="CX88" s="6"/>
+      <c r="CY88" s="6"/>
+      <c r="CZ88" s="6"/>
+      <c r="DA88" s="6"/>
+      <c r="DB88" s="6"/>
+      <c r="DC88" s="6"/>
+      <c r="DD88" s="6"/>
+      <c r="DE88" s="6"/>
+      <c r="DF88" s="6"/>
+      <c r="DG88" s="6"/>
+      <c r="DH88" s="6"/>
     </row>
-    <row r="89" spans="1:96" x14ac:dyDescent="0.3">
+    <row r="89" spans="1:112" x14ac:dyDescent="0.3">
       <c r="A89" s="6"/>
       <c r="B89" s="6"/>
       <c r="C89" s="6"/>
@@ -14193,8 +16490,24 @@
       <c r="CP89" s="6"/>
       <c r="CQ89" s="6"/>
       <c r="CR89" s="6"/>
+      <c r="CS89" s="6"/>
+      <c r="CT89" s="6"/>
+      <c r="CU89" s="6"/>
+      <c r="CV89" s="6"/>
+      <c r="CW89" s="6"/>
+      <c r="CX89" s="6"/>
+      <c r="CY89" s="6"/>
+      <c r="CZ89" s="6"/>
+      <c r="DA89" s="6"/>
+      <c r="DB89" s="6"/>
+      <c r="DC89" s="6"/>
+      <c r="DD89" s="6"/>
+      <c r="DE89" s="6"/>
+      <c r="DF89" s="6"/>
+      <c r="DG89" s="6"/>
+      <c r="DH89" s="6"/>
     </row>
-    <row r="90" spans="1:96" x14ac:dyDescent="0.3">
+    <row r="90" spans="1:112" x14ac:dyDescent="0.3">
       <c r="A90" s="6"/>
       <c r="B90" s="6"/>
       <c r="C90" s="6"/>
@@ -14291,8 +16604,24 @@
       <c r="CP90" s="6"/>
       <c r="CQ90" s="6"/>
       <c r="CR90" s="6"/>
+      <c r="CS90" s="6"/>
+      <c r="CT90" s="6"/>
+      <c r="CU90" s="6"/>
+      <c r="CV90" s="6"/>
+      <c r="CW90" s="6"/>
+      <c r="CX90" s="6"/>
+      <c r="CY90" s="6"/>
+      <c r="CZ90" s="6"/>
+      <c r="DA90" s="6"/>
+      <c r="DB90" s="6"/>
+      <c r="DC90" s="6"/>
+      <c r="DD90" s="6"/>
+      <c r="DE90" s="6"/>
+      <c r="DF90" s="6"/>
+      <c r="DG90" s="6"/>
+      <c r="DH90" s="6"/>
     </row>
-    <row r="91" spans="1:96" x14ac:dyDescent="0.3">
+    <row r="91" spans="1:112" x14ac:dyDescent="0.3">
       <c r="A91" s="5" t="s">
         <v>19</v>
       </c>
@@ -14425,16 +16754,40 @@
       <c r="CH91" s="6"/>
       <c r="CI91" s="6"/>
       <c r="CJ91" s="6"/>
-      <c r="CK91" s="5"/>
+      <c r="CK91" s="5" t="s">
+        <v>238</v>
+      </c>
       <c r="CL91" s="6"/>
       <c r="CM91" s="6"/>
       <c r="CN91" s="6"/>
-      <c r="CO91" s="5"/>
+      <c r="CO91" s="5" t="s">
+        <v>236</v>
+      </c>
       <c r="CP91" s="6"/>
       <c r="CQ91" s="6"/>
       <c r="CR91" s="6"/>
+      <c r="CS91" s="5" t="s">
+        <v>257</v>
+      </c>
+      <c r="CT91" s="6"/>
+      <c r="CU91" s="6"/>
+      <c r="CV91" s="6"/>
+      <c r="CW91" s="5" t="s">
+        <v>258</v>
+      </c>
+      <c r="CX91" s="6"/>
+      <c r="CY91" s="6"/>
+      <c r="CZ91" s="6"/>
+      <c r="DA91" s="5"/>
+      <c r="DB91" s="6"/>
+      <c r="DC91" s="6"/>
+      <c r="DD91" s="6"/>
+      <c r="DE91" s="5"/>
+      <c r="DF91" s="6"/>
+      <c r="DG91" s="6"/>
+      <c r="DH91" s="6"/>
     </row>
-    <row r="92" spans="1:96" x14ac:dyDescent="0.3">
+    <row r="92" spans="1:112" x14ac:dyDescent="0.3">
       <c r="A92" s="6"/>
       <c r="B92" s="6"/>
       <c r="C92" s="6"/>
@@ -14531,8 +16884,24 @@
       <c r="CP92" s="6"/>
       <c r="CQ92" s="6"/>
       <c r="CR92" s="6"/>
+      <c r="CS92" s="6"/>
+      <c r="CT92" s="6"/>
+      <c r="CU92" s="6"/>
+      <c r="CV92" s="6"/>
+      <c r="CW92" s="6"/>
+      <c r="CX92" s="6"/>
+      <c r="CY92" s="6"/>
+      <c r="CZ92" s="6"/>
+      <c r="DA92" s="6"/>
+      <c r="DB92" s="6"/>
+      <c r="DC92" s="6"/>
+      <c r="DD92" s="6"/>
+      <c r="DE92" s="6"/>
+      <c r="DF92" s="6"/>
+      <c r="DG92" s="6"/>
+      <c r="DH92" s="6"/>
     </row>
-    <row r="93" spans="1:96" x14ac:dyDescent="0.3">
+    <row r="93" spans="1:112" x14ac:dyDescent="0.3">
       <c r="A93" s="6"/>
       <c r="B93" s="6"/>
       <c r="C93" s="6"/>
@@ -14629,8 +16998,24 @@
       <c r="CP93" s="6"/>
       <c r="CQ93" s="6"/>
       <c r="CR93" s="6"/>
+      <c r="CS93" s="6"/>
+      <c r="CT93" s="6"/>
+      <c r="CU93" s="6"/>
+      <c r="CV93" s="6"/>
+      <c r="CW93" s="6"/>
+      <c r="CX93" s="6"/>
+      <c r="CY93" s="6"/>
+      <c r="CZ93" s="6"/>
+      <c r="DA93" s="6"/>
+      <c r="DB93" s="6"/>
+      <c r="DC93" s="6"/>
+      <c r="DD93" s="6"/>
+      <c r="DE93" s="6"/>
+      <c r="DF93" s="6"/>
+      <c r="DG93" s="6"/>
+      <c r="DH93" s="6"/>
     </row>
-    <row r="94" spans="1:96" x14ac:dyDescent="0.3">
+    <row r="94" spans="1:112" x14ac:dyDescent="0.3">
       <c r="A94" s="6"/>
       <c r="B94" s="6"/>
       <c r="C94" s="6"/>
@@ -14727,8 +17112,24 @@
       <c r="CP94" s="6"/>
       <c r="CQ94" s="6"/>
       <c r="CR94" s="6"/>
+      <c r="CS94" s="6"/>
+      <c r="CT94" s="6"/>
+      <c r="CU94" s="6"/>
+      <c r="CV94" s="6"/>
+      <c r="CW94" s="6"/>
+      <c r="CX94" s="6"/>
+      <c r="CY94" s="6"/>
+      <c r="CZ94" s="6"/>
+      <c r="DA94" s="6"/>
+      <c r="DB94" s="6"/>
+      <c r="DC94" s="6"/>
+      <c r="DD94" s="6"/>
+      <c r="DE94" s="6"/>
+      <c r="DF94" s="6"/>
+      <c r="DG94" s="6"/>
+      <c r="DH94" s="6"/>
     </row>
-    <row r="95" spans="1:96" x14ac:dyDescent="0.3">
+    <row r="95" spans="1:112" x14ac:dyDescent="0.3">
       <c r="A95" s="6"/>
       <c r="B95" s="6"/>
       <c r="C95" s="6"/>
@@ -14825,8 +17226,24 @@
       <c r="CP95" s="6"/>
       <c r="CQ95" s="6"/>
       <c r="CR95" s="6"/>
+      <c r="CS95" s="6"/>
+      <c r="CT95" s="6"/>
+      <c r="CU95" s="6"/>
+      <c r="CV95" s="6"/>
+      <c r="CW95" s="6"/>
+      <c r="CX95" s="6"/>
+      <c r="CY95" s="6"/>
+      <c r="CZ95" s="6"/>
+      <c r="DA95" s="6"/>
+      <c r="DB95" s="6"/>
+      <c r="DC95" s="6"/>
+      <c r="DD95" s="6"/>
+      <c r="DE95" s="6"/>
+      <c r="DF95" s="6"/>
+      <c r="DG95" s="6"/>
+      <c r="DH95" s="6"/>
     </row>
-    <row r="96" spans="1:96" x14ac:dyDescent="0.3">
+    <row r="96" spans="1:112" x14ac:dyDescent="0.3">
       <c r="A96" s="6"/>
       <c r="B96" s="6"/>
       <c r="C96" s="6"/>
@@ -14923,8 +17340,24 @@
       <c r="CP96" s="6"/>
       <c r="CQ96" s="6"/>
       <c r="CR96" s="6"/>
+      <c r="CS96" s="6"/>
+      <c r="CT96" s="6"/>
+      <c r="CU96" s="6"/>
+      <c r="CV96" s="6"/>
+      <c r="CW96" s="6"/>
+      <c r="CX96" s="6"/>
+      <c r="CY96" s="6"/>
+      <c r="CZ96" s="6"/>
+      <c r="DA96" s="6"/>
+      <c r="DB96" s="6"/>
+      <c r="DC96" s="6"/>
+      <c r="DD96" s="6"/>
+      <c r="DE96" s="6"/>
+      <c r="DF96" s="6"/>
+      <c r="DG96" s="6"/>
+      <c r="DH96" s="6"/>
     </row>
-    <row r="97" spans="1:96" x14ac:dyDescent="0.3">
+    <row r="97" spans="1:112" x14ac:dyDescent="0.3">
       <c r="A97" s="6"/>
       <c r="B97" s="6"/>
       <c r="C97" s="6"/>
@@ -15021,8 +17454,24 @@
       <c r="CP97" s="6"/>
       <c r="CQ97" s="6"/>
       <c r="CR97" s="6"/>
+      <c r="CS97" s="6"/>
+      <c r="CT97" s="6"/>
+      <c r="CU97" s="6"/>
+      <c r="CV97" s="6"/>
+      <c r="CW97" s="6"/>
+      <c r="CX97" s="6"/>
+      <c r="CY97" s="6"/>
+      <c r="CZ97" s="6"/>
+      <c r="DA97" s="6"/>
+      <c r="DB97" s="6"/>
+      <c r="DC97" s="6"/>
+      <c r="DD97" s="6"/>
+      <c r="DE97" s="6"/>
+      <c r="DF97" s="6"/>
+      <c r="DG97" s="6"/>
+      <c r="DH97" s="6"/>
     </row>
-    <row r="98" spans="1:96" x14ac:dyDescent="0.3">
+    <row r="98" spans="1:112" x14ac:dyDescent="0.3">
       <c r="A98" s="6"/>
       <c r="B98" s="6"/>
       <c r="C98" s="6"/>
@@ -15119,8 +17568,24 @@
       <c r="CP98" s="6"/>
       <c r="CQ98" s="6"/>
       <c r="CR98" s="6"/>
+      <c r="CS98" s="6"/>
+      <c r="CT98" s="6"/>
+      <c r="CU98" s="6"/>
+      <c r="CV98" s="6"/>
+      <c r="CW98" s="6"/>
+      <c r="CX98" s="6"/>
+      <c r="CY98" s="6"/>
+      <c r="CZ98" s="6"/>
+      <c r="DA98" s="6"/>
+      <c r="DB98" s="6"/>
+      <c r="DC98" s="6"/>
+      <c r="DD98" s="6"/>
+      <c r="DE98" s="6"/>
+      <c r="DF98" s="6"/>
+      <c r="DG98" s="6"/>
+      <c r="DH98" s="6"/>
     </row>
-    <row r="99" spans="1:96" x14ac:dyDescent="0.3">
+    <row r="99" spans="1:112" x14ac:dyDescent="0.3">
       <c r="A99" s="6"/>
       <c r="B99" s="6"/>
       <c r="C99" s="6"/>
@@ -15217,8 +17682,24 @@
       <c r="CP99" s="6"/>
       <c r="CQ99" s="6"/>
       <c r="CR99" s="6"/>
+      <c r="CS99" s="6"/>
+      <c r="CT99" s="6"/>
+      <c r="CU99" s="6"/>
+      <c r="CV99" s="6"/>
+      <c r="CW99" s="6"/>
+      <c r="CX99" s="6"/>
+      <c r="CY99" s="6"/>
+      <c r="CZ99" s="6"/>
+      <c r="DA99" s="6"/>
+      <c r="DB99" s="6"/>
+      <c r="DC99" s="6"/>
+      <c r="DD99" s="6"/>
+      <c r="DE99" s="6"/>
+      <c r="DF99" s="6"/>
+      <c r="DG99" s="6"/>
+      <c r="DH99" s="6"/>
     </row>
-    <row r="100" spans="1:96" x14ac:dyDescent="0.3">
+    <row r="100" spans="1:112" x14ac:dyDescent="0.3">
       <c r="A100" s="6"/>
       <c r="B100" s="6"/>
       <c r="C100" s="6"/>
@@ -15315,8 +17796,24 @@
       <c r="CP100" s="6"/>
       <c r="CQ100" s="6"/>
       <c r="CR100" s="6"/>
+      <c r="CS100" s="6"/>
+      <c r="CT100" s="6"/>
+      <c r="CU100" s="6"/>
+      <c r="CV100" s="6"/>
+      <c r="CW100" s="6"/>
+      <c r="CX100" s="6"/>
+      <c r="CY100" s="6"/>
+      <c r="CZ100" s="6"/>
+      <c r="DA100" s="6"/>
+      <c r="DB100" s="6"/>
+      <c r="DC100" s="6"/>
+      <c r="DD100" s="6"/>
+      <c r="DE100" s="6"/>
+      <c r="DF100" s="6"/>
+      <c r="DG100" s="6"/>
+      <c r="DH100" s="6"/>
     </row>
-    <row r="101" spans="1:96" ht="14.4" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="101" spans="1:112" ht="14.4" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A101" s="1"/>
       <c r="B101" s="2"/>
       <c r="C101" s="2"/>
@@ -15330,7 +17827,7 @@
       <c r="K101" s="4"/>
       <c r="L101" s="4"/>
     </row>
-    <row r="102" spans="1:96" x14ac:dyDescent="0.3">
+    <row r="102" spans="1:112" x14ac:dyDescent="0.3">
       <c r="A102" s="2"/>
       <c r="B102" s="3"/>
       <c r="C102" s="4"/>
@@ -15344,7 +17841,7 @@
       <c r="K102" s="4"/>
       <c r="L102" s="4"/>
     </row>
-    <row r="103" spans="1:96" x14ac:dyDescent="0.3">
+    <row r="103" spans="1:112" x14ac:dyDescent="0.3">
       <c r="A103" s="2"/>
       <c r="B103" s="4"/>
       <c r="C103" s="4"/>
@@ -15358,7 +17855,7 @@
       <c r="K103" s="4"/>
       <c r="L103" s="4"/>
     </row>
-    <row r="104" spans="1:96" x14ac:dyDescent="0.3">
+    <row r="104" spans="1:112" x14ac:dyDescent="0.3">
       <c r="A104" s="2"/>
       <c r="B104" s="4"/>
       <c r="C104" s="4"/>
@@ -15372,7 +17869,7 @@
       <c r="K104" s="4"/>
       <c r="L104" s="4"/>
     </row>
-    <row r="105" spans="1:96" x14ac:dyDescent="0.3">
+    <row r="105" spans="1:112" x14ac:dyDescent="0.3">
       <c r="A105" s="2"/>
       <c r="B105" s="4"/>
       <c r="C105" s="4"/>
@@ -15386,7 +17883,7 @@
       <c r="K105" s="4"/>
       <c r="L105" s="4"/>
     </row>
-    <row r="106" spans="1:96" x14ac:dyDescent="0.3">
+    <row r="106" spans="1:112" x14ac:dyDescent="0.3">
       <c r="A106" s="2"/>
       <c r="B106" s="4"/>
       <c r="C106" s="4"/>
@@ -15400,7 +17897,7 @@
       <c r="K106" s="4"/>
       <c r="L106" s="4"/>
     </row>
-    <row r="107" spans="1:96" x14ac:dyDescent="0.3">
+    <row r="107" spans="1:112" x14ac:dyDescent="0.3">
       <c r="A107" s="2"/>
       <c r="B107" s="4"/>
       <c r="C107" s="4"/>
@@ -15414,7 +17911,7 @@
       <c r="K107" s="4"/>
       <c r="L107" s="4"/>
     </row>
-    <row r="108" spans="1:96" x14ac:dyDescent="0.3">
+    <row r="108" spans="1:112" x14ac:dyDescent="0.3">
       <c r="A108" s="2"/>
       <c r="B108" s="4"/>
       <c r="C108" s="4"/>
@@ -15428,7 +17925,7 @@
       <c r="K108" s="4"/>
       <c r="L108" s="4"/>
     </row>
-    <row r="109" spans="1:96" x14ac:dyDescent="0.3">
+    <row r="109" spans="1:112" x14ac:dyDescent="0.3">
       <c r="A109" s="2"/>
       <c r="B109" s="4"/>
       <c r="C109" s="4"/>
@@ -15442,7 +17939,7 @@
       <c r="K109" s="4"/>
       <c r="L109" s="4"/>
     </row>
-    <row r="110" spans="1:96" x14ac:dyDescent="0.3">
+    <row r="110" spans="1:112" x14ac:dyDescent="0.3">
       <c r="A110" s="2"/>
       <c r="B110" s="4"/>
       <c r="C110" s="4"/>
@@ -15456,7 +17953,7 @@
       <c r="K110" s="4"/>
       <c r="L110" s="4"/>
     </row>
-    <row r="111" spans="1:96" ht="14.4" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="111" spans="1:112" ht="14.4" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A111" s="1"/>
       <c r="B111" s="4"/>
       <c r="C111" s="4"/>
@@ -15470,7 +17967,7 @@
       <c r="K111" s="4"/>
       <c r="L111" s="4"/>
     </row>
-    <row r="112" spans="1:96" x14ac:dyDescent="0.3">
+    <row r="112" spans="1:112" x14ac:dyDescent="0.3">
       <c r="A112" s="2"/>
       <c r="B112" s="3"/>
       <c r="C112" s="4"/>
@@ -16023,7 +18520,47 @@
       <c r="E151" s="4"/>
     </row>
   </sheetData>
-  <mergeCells count="240">
+  <mergeCells count="280">
+    <mergeCell ref="DA51:DD60"/>
+    <mergeCell ref="DE51:DH60"/>
+    <mergeCell ref="DA61:DD70"/>
+    <mergeCell ref="DE61:DH70"/>
+    <mergeCell ref="DA71:DD80"/>
+    <mergeCell ref="DE71:DH80"/>
+    <mergeCell ref="DA81:DD90"/>
+    <mergeCell ref="DE81:DH90"/>
+    <mergeCell ref="DA91:DD100"/>
+    <mergeCell ref="DE91:DH100"/>
+    <mergeCell ref="DA1:DD10"/>
+    <mergeCell ref="DE1:DH10"/>
+    <mergeCell ref="DA11:DD20"/>
+    <mergeCell ref="DE11:DH20"/>
+    <mergeCell ref="DA21:DD30"/>
+    <mergeCell ref="DE21:DH30"/>
+    <mergeCell ref="DA31:DD40"/>
+    <mergeCell ref="DE31:DH40"/>
+    <mergeCell ref="DA41:DD50"/>
+    <mergeCell ref="DE41:DH50"/>
+    <mergeCell ref="CS51:CV60"/>
+    <mergeCell ref="CW51:CZ60"/>
+    <mergeCell ref="CS61:CV70"/>
+    <mergeCell ref="CW61:CZ70"/>
+    <mergeCell ref="CS71:CV80"/>
+    <mergeCell ref="CW71:CZ80"/>
+    <mergeCell ref="CS81:CV90"/>
+    <mergeCell ref="CW81:CZ90"/>
+    <mergeCell ref="CS91:CV100"/>
+    <mergeCell ref="CW91:CZ100"/>
+    <mergeCell ref="CS1:CV10"/>
+    <mergeCell ref="CW1:CZ10"/>
+    <mergeCell ref="CS11:CV20"/>
+    <mergeCell ref="CW11:CZ20"/>
+    <mergeCell ref="CS21:CV30"/>
+    <mergeCell ref="CW21:CZ30"/>
+    <mergeCell ref="CS31:CV40"/>
+    <mergeCell ref="CW31:CZ40"/>
+    <mergeCell ref="CS41:CV50"/>
+    <mergeCell ref="CW41:CZ50"/>
     <mergeCell ref="BU51:BX60"/>
     <mergeCell ref="BY51:CB60"/>
     <mergeCell ref="BU61:BX70"/>

</xml_diff>

<commit_message>
Added Big O and algortihms questions
</commit_message>
<xml_diff>
--- a/tanulókártyák/Tanulókártyák.xlsx
+++ b/tanulókártyák/Tanulókártyák.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\atesz\OneDrive\Desktop\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{E8D087CB-FA50-495D-BA4A-83F5B00F82A8}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{A96CE3FD-5B42-41A7-B079-2A4EA36B5A78}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12576" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -25,7 +25,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="270" uniqueCount="269">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="292" uniqueCount="291">
   <si>
     <r>
       <rPr>
@@ -1817,55 +1817,6 @@
       </rPr>
       <t xml:space="preserve"> - a Java memória egy speciális területe, ahol a JVM a String literálokat tárolja és újrahasznosítja a memóriahatékonyság érdekében.
 Ha két String ugyanazzal az értékkel jön létre literálként, akkor ugyanarra a memóriabeli objektumra hivatkoznak.</t>
-    </r>
-  </si>
-  <si>
-    <r>
-      <rPr>
-        <b/>
-        <sz val="10"/>
-        <color theme="1"/>
-        <rFont val="Calibri"/>
-        <family val="2"/>
-        <charset val="238"/>
-        <scheme val="minor"/>
-      </rPr>
-      <t xml:space="preserve">Stack - </t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="10"/>
-        <color theme="1"/>
-        <rFont val="Calibri"/>
-        <family val="2"/>
-        <charset val="238"/>
-        <scheme val="minor"/>
-      </rPr>
-      <t xml:space="preserve">a memória azon része, ahol a metódushívásokhoz tartozó lokális változók és a hívási verem (call stack) tárolódik. Gyors, automatikusan kezelt memória, amely LIFO (Last In, First Out) elven működik.
-</t>
-    </r>
-    <r>
-      <rPr>
-        <b/>
-        <sz val="10"/>
-        <color theme="1"/>
-        <rFont val="Calibri"/>
-        <family val="2"/>
-        <charset val="238"/>
-        <scheme val="minor"/>
-      </rPr>
-      <t xml:space="preserve">Heap - </t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="10"/>
-        <color theme="1"/>
-        <rFont val="Calibri"/>
-        <family val="2"/>
-        <charset val="238"/>
-        <scheme val="minor"/>
-      </rPr>
-      <t>a memória azon része, ahol az objektumok és példányok dinamikusan kerülnek lefoglalásra. A heap memóriát a Garbage Collector kezeli, és az objektumok addig maradnak benne, amíg van rájuk hivatkozás.</t>
     </r>
   </si>
   <si>
@@ -5475,6 +5426,718 @@
   </si>
   <si>
     <t>Mit jelent a cascade, milyen formái vannak?</t>
+  </si>
+  <si>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="10"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <charset val="238"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve">API: </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <charset val="238"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>egy előre definiált szabványos felület, amely megmondja, hogyan használhatok valamit anélkül, hogy ismerném a belső működését.
+Web API - itt két alkalmazás kommunikál.
+JPA API - itt nem két alkalmazás kommunikál, hanem a Java programod használ egy szabványos interfészt adatbázis-kezelésre.
+Collections API - itt az API a Java által biztosított gyűjteményosztályok és interfészek összessége.</t>
+    </r>
+  </si>
+  <si>
+    <t>Mit jelent az API?
+Mondj pár példát.</t>
+  </si>
+  <si>
+    <t>Mi az URI?
+Miben tér el az URL-től?</t>
+  </si>
+  <si>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="10"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <charset val="238"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve">URI </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <charset val="238"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve">(uniform resource identifier): egy erőforrás egyedi azonosítója. Segítségével egy erőforrás (pl. felhasználó, fájl, weboldal) azonosítható egy rendszerben.
+Példa: /users/1 vagy /products/42
+</t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="10"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <charset val="238"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve">URI vs URL </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <charset val="238"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>(uniform resource locator):
+URI = azonosító (/users/1)
+URL = azonosító + elérési hely (https://example.com/users/1)</t>
+    </r>
+  </si>
+  <si>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="10"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <charset val="238"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve">Stack - </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <charset val="238"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve">a memória azon része, ahol a metódushívásokhoz tartozó lokális változók és más fontos adatok tárolódnak. Gyors, automatikusan kezelt memória, amely LIFO (Last In, First Out) elven működik.
+</t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="10"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <charset val="238"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve">Heap - </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <charset val="238"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>a memória azon része, ahol az objektumok és példányok dinamikusan kerülnek lefoglalásra. A heap memóriát a Garbage Collector kezeli, és az objektumok addig maradnak benne, amíg van rájuk hivatkozás.</t>
+    </r>
+  </si>
+  <si>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="10"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <charset val="238"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>Mit tárol pontosan a JVM Stack?</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <charset val="238"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve">
+Minden thread-nek saját stack-je van, és ezen belül:
+Stack frame-ek tárolódhatnak.
+Egy frame egy metódushíváshoz tartozik.
+A Stack Frame tartalma:
+lokális változók (primitive-ek és referenciák)
+metódus paraméterek
+operand stack (számítások ideiglenes eredményei)
+visszatérési cím (hova menjen vissza a futás)</t>
+    </r>
+  </si>
+  <si>
+    <t>Mit tárol pontosan a JVM Stack?
+(pontosító kérdés a Stack-hez)</t>
+  </si>
+  <si>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="10"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <charset val="238"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve">Big O </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <charset val="238"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve">- Az algoritmus futási idejének (vagy memóriahasználatának) növekedési ütemét írja le.
+</t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="10"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <charset val="238"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>Időkomplexitás</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <charset val="238"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve"> - Megmutatja, hogyan nő a futási idő a bemenet méretével.
+</t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="10"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <charset val="238"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>Térkomplexitás</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <charset val="238"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve"> - Megmutatja, mennyi extra memória kell az algoritmusnak.</t>
+    </r>
+  </si>
+  <si>
+    <t>Mi a big O, az időkomplexitás és térkomplexitás?</t>
+  </si>
+  <si>
+    <t>Milyen gyakori komplexitásokat ismersz?</t>
+  </si>
+  <si>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="10"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <charset val="238"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>O(1)</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <charset val="238"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve"> – konstans - a futási idő nem függ a bemenet méretétől. (Tömb elemének elérése)
+</t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="10"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <charset val="238"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve">O(log n) </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <charset val="238"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve">– logaritmikus - a probléma mérete minden lépésben csökken (pl. bináris keresés).
+</t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="10"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <charset val="238"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>O(n)</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <charset val="238"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve"> – lineáris - minden elemet egyszer végignéz.
+</t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="10"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <charset val="238"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve">O(n log n) </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <charset val="238"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve">- hatékony rendezési algoritmusok (pl. mergesort, heapsort).
+</t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="10"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <charset val="238"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>O(n²)</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <charset val="238"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve"> – kvadratikus - beágyazott ciklusok, minden elem minden elemmel összehasonlítva.
+</t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="10"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <charset val="238"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>O(2ⁿ)</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <charset val="238"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve"> -Exponenciális növekedés, pl. bruteforce.</t>
+    </r>
+  </si>
+  <si>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="10"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <charset val="238"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve">Big O példák:
+</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <charset val="238"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>O(1) példa - Tömb egy elemének elérése: arr[5]
+O(n) példa - Lista végigiterálása for ciklussal
+O(n²) példa - Két egymásba ágyazott ciklus
+Adatszerkezetek működése:
+Array - O(1) access, O(n) insert/delete
+LinkedList - O(n) access, O(1) insert/delete (ha a node adott)
+HashMap - Átlag O(1) keresés, beszúrás, törlés</t>
+    </r>
+  </si>
+  <si>
+    <t>Milyen gyakori Big O példákat tudnál mondani?
+(komplexitás / adatszerkezetek működése)</t>
+  </si>
+  <si>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="10"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <charset val="238"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>Algoritmus</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <charset val="238"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve">
+Lépések sorozata egy probléma megoldására.
+Bemenetet vesz és kimenetet ad.
+Végrehajtható és egyértelmű utasításokból áll.</t>
+    </r>
+  </si>
+  <si>
+    <t>Mi az algoritmus?</t>
+  </si>
+  <si>
+    <t>Hogyan működik a binary és a linear search?</t>
+  </si>
+  <si>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="10"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <charset val="238"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>Binary Search</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <charset val="238"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve">
+Rendezett listában kereső algoritmus.
+Mindig a középső elemet vizsgálja, és felezi a keresési tartományt.
+Időkomplexitás: O(log n).
+</t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="10"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <charset val="238"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>Linear Search</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <charset val="238"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve">
+Egyszerű keresés, minden elemet sorban végignéz.
+Akkor is működik, ha a lista nincs rendezve.
+Időkomplexitás: O(n).</t>
+    </r>
+  </si>
+  <si>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="10"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <charset val="238"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>Rekurzió</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <charset val="238"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve">
+Olyan függvényhívás, amely saját magát hívja meg.
+Kell egy base case, hogy megálljon.
+Gyakran fa-szerű problémákra használják (pl. Fibonacci).</t>
+    </r>
+  </si>
+  <si>
+    <t>Mi a rekurzió?</t>
+  </si>
+  <si>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="10"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <charset val="238"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve">Quick Sort - </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <charset val="238"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve">Pivot elemet választ, és kisebb/nagyobb részre bont. Rekurzívan rendezi a részeket. 
+Átlag: O(n log n), worst case: O(n²)
+</t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="10"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <charset val="238"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve">Merge Sort </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <charset val="238"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve">- Divide and Conquer (oszd meg és uralkodj). A listát felezi, majd összefésüli rendezve.
+Időkomplexitás: O(n log n)
+</t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="10"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <charset val="238"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>Bubble Sort</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <charset val="238"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve"> - Rendezési algoritmus, ami szomszédos elemeket hasonlít össze és cserél. A legnagyobb elemek “felbuborékolnak” a végére.
+Időkomplexitás: O(n²).</t>
+    </r>
+  </si>
+  <si>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="10"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <charset val="238"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve">Selection Sort </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <charset val="238"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve">- Minden lépésben kiválasztja a legkisebb elemet, és előre teszi. A lista elejét fokozatosan “felépíti” rendezetté.
+Időkomplexitás: O(n²)
+</t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="10"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <charset val="238"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve">Insertion Sort </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <charset val="238"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>-</t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="10"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <charset val="238"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve"> </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <charset val="238"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve">Egyesével beszúrja az elemeket a már rendezett részbe. Olyan, mint amikor kézzel rendezel kártyákat.
+Időkomplexitás: O(n²) 
+(de majdnem rendezett listán O(n))
+</t>
+    </r>
+  </si>
+  <si>
+    <t>Selection, insertion sort</t>
+  </si>
+  <si>
+    <t>Quick, Merge, Bubble sort</t>
   </si>
 </sst>
 </file>
@@ -5867,13 +6530,13 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:DH151"/>
+  <dimension ref="A1:DP151"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
-    <col min="1" max="112" width="11" customWidth="1"/>
+    <col min="1" max="120" width="11" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:112" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:120" x14ac:dyDescent="0.3">
       <c r="A1" s="7" t="s">
         <v>0</v>
       </c>
@@ -5947,103 +6610,115 @@
       <c r="AU1" s="8"/>
       <c r="AV1" s="8"/>
       <c r="AW1" s="7" t="s">
-        <v>116</v>
+        <v>115</v>
       </c>
       <c r="AX1" s="8"/>
       <c r="AY1" s="8"/>
       <c r="AZ1" s="8"/>
       <c r="BA1" s="7" t="s">
-        <v>118</v>
+        <v>117</v>
       </c>
       <c r="BB1" s="8"/>
       <c r="BC1" s="8"/>
       <c r="BD1" s="8"/>
       <c r="BE1" s="7" t="s">
-        <v>137</v>
+        <v>136</v>
       </c>
       <c r="BF1" s="8"/>
       <c r="BG1" s="8"/>
       <c r="BH1" s="8"/>
       <c r="BI1" s="7" t="s">
-        <v>138</v>
+        <v>137</v>
       </c>
       <c r="BJ1" s="8"/>
       <c r="BK1" s="8"/>
       <c r="BL1" s="8"/>
       <c r="BM1" s="7" t="s">
-        <v>158</v>
+        <v>157</v>
       </c>
       <c r="BN1" s="8"/>
       <c r="BO1" s="8"/>
       <c r="BP1" s="8"/>
       <c r="BQ1" s="7" t="s">
-        <v>160</v>
+        <v>159</v>
       </c>
       <c r="BR1" s="8"/>
       <c r="BS1" s="8"/>
       <c r="BT1" s="8"/>
       <c r="BU1" s="7" t="s">
-        <v>178</v>
+        <v>177</v>
       </c>
       <c r="BV1" s="8"/>
       <c r="BW1" s="8"/>
       <c r="BX1" s="8"/>
       <c r="BY1" s="7" t="s">
-        <v>180</v>
+        <v>179</v>
       </c>
       <c r="BZ1" s="8"/>
       <c r="CA1" s="8"/>
       <c r="CB1" s="8"/>
       <c r="CC1" s="7" t="s">
-        <v>198</v>
+        <v>197</v>
       </c>
       <c r="CD1" s="8"/>
       <c r="CE1" s="8"/>
       <c r="CF1" s="8"/>
       <c r="CG1" s="7" t="s">
-        <v>200</v>
+        <v>199</v>
       </c>
       <c r="CH1" s="8"/>
       <c r="CI1" s="8"/>
       <c r="CJ1" s="8"/>
       <c r="CK1" s="7" t="s">
-        <v>219</v>
+        <v>218</v>
       </c>
       <c r="CL1" s="8"/>
       <c r="CM1" s="8"/>
       <c r="CN1" s="8"/>
       <c r="CO1" s="7" t="s">
-        <v>220</v>
+        <v>219</v>
       </c>
       <c r="CP1" s="8"/>
       <c r="CQ1" s="8"/>
       <c r="CR1" s="8"/>
       <c r="CS1" s="7" t="s">
-        <v>239</v>
+        <v>238</v>
       </c>
       <c r="CT1" s="8"/>
       <c r="CU1" s="8"/>
       <c r="CV1" s="8"/>
       <c r="CW1" s="7" t="s">
-        <v>244</v>
+        <v>243</v>
       </c>
       <c r="CX1" s="8"/>
       <c r="CY1" s="8"/>
       <c r="CZ1" s="8"/>
       <c r="DA1" s="7" t="s">
-        <v>259</v>
+        <v>258</v>
       </c>
       <c r="DB1" s="8"/>
       <c r="DC1" s="8"/>
       <c r="DD1" s="8"/>
       <c r="DE1" s="7" t="s">
-        <v>261</v>
+        <v>260</v>
       </c>
       <c r="DF1" s="8"/>
       <c r="DG1" s="8"/>
       <c r="DH1" s="8"/>
+      <c r="DI1" s="7" t="s">
+        <v>279</v>
+      </c>
+      <c r="DJ1" s="8"/>
+      <c r="DK1" s="8"/>
+      <c r="DL1" s="8"/>
+      <c r="DM1" s="7" t="s">
+        <v>281</v>
+      </c>
+      <c r="DN1" s="8"/>
+      <c r="DO1" s="8"/>
+      <c r="DP1" s="8"/>
     </row>
-    <row r="2" spans="1:112" x14ac:dyDescent="0.3">
+    <row r="2" spans="1:120" x14ac:dyDescent="0.3">
       <c r="A2" s="8"/>
       <c r="B2" s="8"/>
       <c r="C2" s="8"/>
@@ -6156,8 +6831,16 @@
       <c r="DF2" s="8"/>
       <c r="DG2" s="8"/>
       <c r="DH2" s="8"/>
+      <c r="DI2" s="8"/>
+      <c r="DJ2" s="8"/>
+      <c r="DK2" s="8"/>
+      <c r="DL2" s="8"/>
+      <c r="DM2" s="8"/>
+      <c r="DN2" s="8"/>
+      <c r="DO2" s="8"/>
+      <c r="DP2" s="8"/>
     </row>
-    <row r="3" spans="1:112" x14ac:dyDescent="0.3">
+    <row r="3" spans="1:120" x14ac:dyDescent="0.3">
       <c r="A3" s="8"/>
       <c r="B3" s="8"/>
       <c r="C3" s="8"/>
@@ -6270,8 +6953,16 @@
       <c r="DF3" s="8"/>
       <c r="DG3" s="8"/>
       <c r="DH3" s="8"/>
+      <c r="DI3" s="8"/>
+      <c r="DJ3" s="8"/>
+      <c r="DK3" s="8"/>
+      <c r="DL3" s="8"/>
+      <c r="DM3" s="8"/>
+      <c r="DN3" s="8"/>
+      <c r="DO3" s="8"/>
+      <c r="DP3" s="8"/>
     </row>
-    <row r="4" spans="1:112" x14ac:dyDescent="0.3">
+    <row r="4" spans="1:120" x14ac:dyDescent="0.3">
       <c r="A4" s="8"/>
       <c r="B4" s="8"/>
       <c r="C4" s="8"/>
@@ -6384,8 +7075,16 @@
       <c r="DF4" s="8"/>
       <c r="DG4" s="8"/>
       <c r="DH4" s="8"/>
+      <c r="DI4" s="8"/>
+      <c r="DJ4" s="8"/>
+      <c r="DK4" s="8"/>
+      <c r="DL4" s="8"/>
+      <c r="DM4" s="8"/>
+      <c r="DN4" s="8"/>
+      <c r="DO4" s="8"/>
+      <c r="DP4" s="8"/>
     </row>
-    <row r="5" spans="1:112" x14ac:dyDescent="0.3">
+    <row r="5" spans="1:120" x14ac:dyDescent="0.3">
       <c r="A5" s="8"/>
       <c r="B5" s="8"/>
       <c r="C5" s="8"/>
@@ -6498,8 +7197,16 @@
       <c r="DF5" s="8"/>
       <c r="DG5" s="8"/>
       <c r="DH5" s="8"/>
+      <c r="DI5" s="8"/>
+      <c r="DJ5" s="8"/>
+      <c r="DK5" s="8"/>
+      <c r="DL5" s="8"/>
+      <c r="DM5" s="8"/>
+      <c r="DN5" s="8"/>
+      <c r="DO5" s="8"/>
+      <c r="DP5" s="8"/>
     </row>
-    <row r="6" spans="1:112" x14ac:dyDescent="0.3">
+    <row r="6" spans="1:120" x14ac:dyDescent="0.3">
       <c r="A6" s="8"/>
       <c r="B6" s="8"/>
       <c r="C6" s="8"/>
@@ -6612,8 +7319,16 @@
       <c r="DF6" s="8"/>
       <c r="DG6" s="8"/>
       <c r="DH6" s="8"/>
+      <c r="DI6" s="8"/>
+      <c r="DJ6" s="8"/>
+      <c r="DK6" s="8"/>
+      <c r="DL6" s="8"/>
+      <c r="DM6" s="8"/>
+      <c r="DN6" s="8"/>
+      <c r="DO6" s="8"/>
+      <c r="DP6" s="8"/>
     </row>
-    <row r="7" spans="1:112" x14ac:dyDescent="0.3">
+    <row r="7" spans="1:120" x14ac:dyDescent="0.3">
       <c r="A7" s="8"/>
       <c r="B7" s="8"/>
       <c r="C7" s="8"/>
@@ -6726,8 +7441,16 @@
       <c r="DF7" s="8"/>
       <c r="DG7" s="8"/>
       <c r="DH7" s="8"/>
+      <c r="DI7" s="8"/>
+      <c r="DJ7" s="8"/>
+      <c r="DK7" s="8"/>
+      <c r="DL7" s="8"/>
+      <c r="DM7" s="8"/>
+      <c r="DN7" s="8"/>
+      <c r="DO7" s="8"/>
+      <c r="DP7" s="8"/>
     </row>
-    <row r="8" spans="1:112" x14ac:dyDescent="0.3">
+    <row r="8" spans="1:120" x14ac:dyDescent="0.3">
       <c r="A8" s="8"/>
       <c r="B8" s="8"/>
       <c r="C8" s="8"/>
@@ -6840,8 +7563,16 @@
       <c r="DF8" s="8"/>
       <c r="DG8" s="8"/>
       <c r="DH8" s="8"/>
+      <c r="DI8" s="8"/>
+      <c r="DJ8" s="8"/>
+      <c r="DK8" s="8"/>
+      <c r="DL8" s="8"/>
+      <c r="DM8" s="8"/>
+      <c r="DN8" s="8"/>
+      <c r="DO8" s="8"/>
+      <c r="DP8" s="8"/>
     </row>
-    <row r="9" spans="1:112" x14ac:dyDescent="0.3">
+    <row r="9" spans="1:120" x14ac:dyDescent="0.3">
       <c r="A9" s="8"/>
       <c r="B9" s="8"/>
       <c r="C9" s="8"/>
@@ -6954,8 +7685,16 @@
       <c r="DF9" s="8"/>
       <c r="DG9" s="8"/>
       <c r="DH9" s="8"/>
+      <c r="DI9" s="8"/>
+      <c r="DJ9" s="8"/>
+      <c r="DK9" s="8"/>
+      <c r="DL9" s="8"/>
+      <c r="DM9" s="8"/>
+      <c r="DN9" s="8"/>
+      <c r="DO9" s="8"/>
+      <c r="DP9" s="8"/>
     </row>
-    <row r="10" spans="1:112" x14ac:dyDescent="0.3">
+    <row r="10" spans="1:120" x14ac:dyDescent="0.3">
       <c r="A10" s="8"/>
       <c r="B10" s="8"/>
       <c r="C10" s="8"/>
@@ -7068,8 +7807,16 @@
       <c r="DF10" s="8"/>
       <c r="DG10" s="8"/>
       <c r="DH10" s="8"/>
+      <c r="DI10" s="8"/>
+      <c r="DJ10" s="8"/>
+      <c r="DK10" s="8"/>
+      <c r="DL10" s="8"/>
+      <c r="DM10" s="8"/>
+      <c r="DN10" s="8"/>
+      <c r="DO10" s="8"/>
+      <c r="DP10" s="8"/>
     </row>
-    <row r="11" spans="1:112" x14ac:dyDescent="0.3">
+    <row r="11" spans="1:120" x14ac:dyDescent="0.3">
       <c r="A11" s="7" t="s">
         <v>2</v>
       </c>
@@ -7137,109 +7884,121 @@
       <c r="AQ11" s="8"/>
       <c r="AR11" s="8"/>
       <c r="AS11" s="7" t="s">
-        <v>101</v>
+        <v>272</v>
       </c>
       <c r="AT11" s="8"/>
       <c r="AU11" s="8"/>
       <c r="AV11" s="8"/>
       <c r="AW11" s="7" t="s">
-        <v>120</v>
+        <v>119</v>
       </c>
       <c r="AX11" s="8"/>
       <c r="AY11" s="8"/>
       <c r="AZ11" s="8"/>
       <c r="BA11" s="7" t="s">
-        <v>127</v>
+        <v>126</v>
       </c>
       <c r="BB11" s="8"/>
       <c r="BC11" s="8"/>
       <c r="BD11" s="8"/>
       <c r="BE11" s="7" t="s">
-        <v>142</v>
+        <v>141</v>
       </c>
       <c r="BF11" s="8"/>
       <c r="BG11" s="8"/>
       <c r="BH11" s="8"/>
       <c r="BI11" s="7" t="s">
-        <v>141</v>
+        <v>140</v>
       </c>
       <c r="BJ11" s="8"/>
       <c r="BK11" s="8"/>
       <c r="BL11" s="8"/>
       <c r="BM11" s="7" t="s">
-        <v>162</v>
+        <v>161</v>
       </c>
       <c r="BN11" s="8"/>
       <c r="BO11" s="8"/>
       <c r="BP11" s="8"/>
       <c r="BQ11" s="7" t="s">
-        <v>164</v>
+        <v>163</v>
       </c>
       <c r="BR11" s="8"/>
       <c r="BS11" s="8"/>
       <c r="BT11" s="8"/>
       <c r="BU11" s="7" t="s">
-        <v>183</v>
+        <v>182</v>
       </c>
       <c r="BV11" s="8"/>
       <c r="BW11" s="8"/>
       <c r="BX11" s="8"/>
       <c r="BY11" s="7" t="s">
-        <v>182</v>
+        <v>181</v>
       </c>
       <c r="BZ11" s="8"/>
       <c r="CA11" s="8"/>
       <c r="CB11" s="8"/>
       <c r="CC11" s="7" t="s">
-        <v>202</v>
+        <v>201</v>
       </c>
       <c r="CD11" s="8"/>
       <c r="CE11" s="8"/>
       <c r="CF11" s="8"/>
       <c r="CG11" s="7" t="s">
-        <v>204</v>
+        <v>203</v>
       </c>
       <c r="CH11" s="8"/>
       <c r="CI11" s="8"/>
       <c r="CJ11" s="8"/>
       <c r="CK11" s="7" t="s">
-        <v>222</v>
+        <v>221</v>
       </c>
       <c r="CL11" s="8"/>
       <c r="CM11" s="8"/>
       <c r="CN11" s="8"/>
       <c r="CO11" s="7" t="s">
-        <v>224</v>
+        <v>223</v>
       </c>
       <c r="CP11" s="8"/>
       <c r="CQ11" s="8"/>
       <c r="CR11" s="8"/>
       <c r="CS11" s="7" t="s">
-        <v>242</v>
+        <v>241</v>
       </c>
       <c r="CT11" s="8"/>
       <c r="CU11" s="8"/>
       <c r="CV11" s="8"/>
       <c r="CW11" s="7" t="s">
-        <v>246</v>
+        <v>245</v>
       </c>
       <c r="CX11" s="8"/>
       <c r="CY11" s="8"/>
       <c r="CZ11" s="8"/>
       <c r="DA11" s="7" t="s">
-        <v>263</v>
+        <v>262</v>
       </c>
       <c r="DB11" s="8"/>
       <c r="DC11" s="8"/>
       <c r="DD11" s="8"/>
       <c r="DE11" s="7" t="s">
-        <v>265</v>
+        <v>264</v>
       </c>
       <c r="DF11" s="8"/>
       <c r="DG11" s="8"/>
       <c r="DH11" s="8"/>
+      <c r="DI11" s="7" t="s">
+        <v>284</v>
+      </c>
+      <c r="DJ11" s="8"/>
+      <c r="DK11" s="8"/>
+      <c r="DL11" s="8"/>
+      <c r="DM11" s="7" t="s">
+        <v>285</v>
+      </c>
+      <c r="DN11" s="8"/>
+      <c r="DO11" s="8"/>
+      <c r="DP11" s="8"/>
     </row>
-    <row r="12" spans="1:112" x14ac:dyDescent="0.3">
+    <row r="12" spans="1:120" x14ac:dyDescent="0.3">
       <c r="A12" s="8"/>
       <c r="B12" s="8"/>
       <c r="C12" s="8"/>
@@ -7352,8 +8111,16 @@
       <c r="DF12" s="8"/>
       <c r="DG12" s="8"/>
       <c r="DH12" s="8"/>
+      <c r="DI12" s="8"/>
+      <c r="DJ12" s="8"/>
+      <c r="DK12" s="8"/>
+      <c r="DL12" s="8"/>
+      <c r="DM12" s="8"/>
+      <c r="DN12" s="8"/>
+      <c r="DO12" s="8"/>
+      <c r="DP12" s="8"/>
     </row>
-    <row r="13" spans="1:112" x14ac:dyDescent="0.3">
+    <row r="13" spans="1:120" x14ac:dyDescent="0.3">
       <c r="A13" s="8"/>
       <c r="B13" s="8"/>
       <c r="C13" s="8"/>
@@ -7466,8 +8233,16 @@
       <c r="DF13" s="8"/>
       <c r="DG13" s="8"/>
       <c r="DH13" s="8"/>
+      <c r="DI13" s="8"/>
+      <c r="DJ13" s="8"/>
+      <c r="DK13" s="8"/>
+      <c r="DL13" s="8"/>
+      <c r="DM13" s="8"/>
+      <c r="DN13" s="8"/>
+      <c r="DO13" s="8"/>
+      <c r="DP13" s="8"/>
     </row>
-    <row r="14" spans="1:112" x14ac:dyDescent="0.3">
+    <row r="14" spans="1:120" x14ac:dyDescent="0.3">
       <c r="A14" s="8"/>
       <c r="B14" s="8"/>
       <c r="C14" s="8"/>
@@ -7580,8 +8355,16 @@
       <c r="DF14" s="8"/>
       <c r="DG14" s="8"/>
       <c r="DH14" s="8"/>
+      <c r="DI14" s="8"/>
+      <c r="DJ14" s="8"/>
+      <c r="DK14" s="8"/>
+      <c r="DL14" s="8"/>
+      <c r="DM14" s="8"/>
+      <c r="DN14" s="8"/>
+      <c r="DO14" s="8"/>
+      <c r="DP14" s="8"/>
     </row>
-    <row r="15" spans="1:112" x14ac:dyDescent="0.3">
+    <row r="15" spans="1:120" x14ac:dyDescent="0.3">
       <c r="A15" s="8"/>
       <c r="B15" s="8"/>
       <c r="C15" s="8"/>
@@ -7694,8 +8477,16 @@
       <c r="DF15" s="8"/>
       <c r="DG15" s="8"/>
       <c r="DH15" s="8"/>
+      <c r="DI15" s="8"/>
+      <c r="DJ15" s="8"/>
+      <c r="DK15" s="8"/>
+      <c r="DL15" s="8"/>
+      <c r="DM15" s="8"/>
+      <c r="DN15" s="8"/>
+      <c r="DO15" s="8"/>
+      <c r="DP15" s="8"/>
     </row>
-    <row r="16" spans="1:112" x14ac:dyDescent="0.3">
+    <row r="16" spans="1:120" x14ac:dyDescent="0.3">
       <c r="A16" s="8"/>
       <c r="B16" s="8"/>
       <c r="C16" s="8"/>
@@ -7808,8 +8599,16 @@
       <c r="DF16" s="8"/>
       <c r="DG16" s="8"/>
       <c r="DH16" s="8"/>
+      <c r="DI16" s="8"/>
+      <c r="DJ16" s="8"/>
+      <c r="DK16" s="8"/>
+      <c r="DL16" s="8"/>
+      <c r="DM16" s="8"/>
+      <c r="DN16" s="8"/>
+      <c r="DO16" s="8"/>
+      <c r="DP16" s="8"/>
     </row>
-    <row r="17" spans="1:112" x14ac:dyDescent="0.3">
+    <row r="17" spans="1:120" x14ac:dyDescent="0.3">
       <c r="A17" s="8"/>
       <c r="B17" s="8"/>
       <c r="C17" s="8"/>
@@ -7922,8 +8721,16 @@
       <c r="DF17" s="8"/>
       <c r="DG17" s="8"/>
       <c r="DH17" s="8"/>
+      <c r="DI17" s="8"/>
+      <c r="DJ17" s="8"/>
+      <c r="DK17" s="8"/>
+      <c r="DL17" s="8"/>
+      <c r="DM17" s="8"/>
+      <c r="DN17" s="8"/>
+      <c r="DO17" s="8"/>
+      <c r="DP17" s="8"/>
     </row>
-    <row r="18" spans="1:112" x14ac:dyDescent="0.3">
+    <row r="18" spans="1:120" x14ac:dyDescent="0.3">
       <c r="A18" s="8"/>
       <c r="B18" s="8"/>
       <c r="C18" s="8"/>
@@ -8036,8 +8843,16 @@
       <c r="DF18" s="8"/>
       <c r="DG18" s="8"/>
       <c r="DH18" s="8"/>
+      <c r="DI18" s="8"/>
+      <c r="DJ18" s="8"/>
+      <c r="DK18" s="8"/>
+      <c r="DL18" s="8"/>
+      <c r="DM18" s="8"/>
+      <c r="DN18" s="8"/>
+      <c r="DO18" s="8"/>
+      <c r="DP18" s="8"/>
     </row>
-    <row r="19" spans="1:112" x14ac:dyDescent="0.3">
+    <row r="19" spans="1:120" x14ac:dyDescent="0.3">
       <c r="A19" s="8"/>
       <c r="B19" s="8"/>
       <c r="C19" s="8"/>
@@ -8150,8 +8965,16 @@
       <c r="DF19" s="8"/>
       <c r="DG19" s="8"/>
       <c r="DH19" s="8"/>
+      <c r="DI19" s="8"/>
+      <c r="DJ19" s="8"/>
+      <c r="DK19" s="8"/>
+      <c r="DL19" s="8"/>
+      <c r="DM19" s="8"/>
+      <c r="DN19" s="8"/>
+      <c r="DO19" s="8"/>
+      <c r="DP19" s="8"/>
     </row>
-    <row r="20" spans="1:112" x14ac:dyDescent="0.3">
+    <row r="20" spans="1:120" x14ac:dyDescent="0.3">
       <c r="A20" s="8"/>
       <c r="B20" s="8"/>
       <c r="C20" s="8"/>
@@ -8264,8 +9087,16 @@
       <c r="DF20" s="8"/>
       <c r="DG20" s="8"/>
       <c r="DH20" s="8"/>
+      <c r="DI20" s="8"/>
+      <c r="DJ20" s="8"/>
+      <c r="DK20" s="8"/>
+      <c r="DL20" s="8"/>
+      <c r="DM20" s="8"/>
+      <c r="DN20" s="8"/>
+      <c r="DO20" s="8"/>
+      <c r="DP20" s="8"/>
     </row>
-    <row r="21" spans="1:112" x14ac:dyDescent="0.3">
+    <row r="21" spans="1:120" x14ac:dyDescent="0.3">
       <c r="A21" s="7" t="s">
         <v>4</v>
       </c>
@@ -8285,7 +9116,7 @@
       <c r="K21" s="8"/>
       <c r="L21" s="8"/>
       <c r="M21" s="7" t="s">
-        <v>124</v>
+        <v>123</v>
       </c>
       <c r="N21" s="8"/>
       <c r="O21" s="8"/>
@@ -8327,113 +9158,127 @@
       <c r="AM21" s="8"/>
       <c r="AN21" s="8"/>
       <c r="AO21" s="7" t="s">
-        <v>104</v>
+        <v>103</v>
       </c>
       <c r="AP21" s="8"/>
       <c r="AQ21" s="8"/>
       <c r="AR21" s="8"/>
       <c r="AS21" s="7" t="s">
-        <v>106</v>
+        <v>105</v>
       </c>
       <c r="AT21" s="8"/>
       <c r="AU21" s="8"/>
       <c r="AV21" s="8"/>
       <c r="AW21" s="7" t="s">
-        <v>128</v>
+        <v>127</v>
       </c>
       <c r="AX21" s="8"/>
       <c r="AY21" s="8"/>
       <c r="AZ21" s="8"/>
       <c r="BA21" s="7" t="s">
-        <v>125</v>
+        <v>124</v>
       </c>
       <c r="BB21" s="8"/>
       <c r="BC21" s="8"/>
       <c r="BD21" s="8"/>
       <c r="BE21" s="7" t="s">
-        <v>143</v>
+        <v>142</v>
       </c>
       <c r="BF21" s="8"/>
       <c r="BG21" s="8"/>
       <c r="BH21" s="8"/>
       <c r="BI21" s="7" t="s">
-        <v>147</v>
+        <v>146</v>
       </c>
       <c r="BJ21" s="8"/>
       <c r="BK21" s="8"/>
       <c r="BL21" s="8"/>
       <c r="BM21" s="7" t="s">
-        <v>166</v>
+        <v>165</v>
       </c>
       <c r="BN21" s="8"/>
       <c r="BO21" s="8"/>
       <c r="BP21" s="8"/>
       <c r="BQ21" s="7" t="s">
-        <v>168</v>
+        <v>167</v>
       </c>
       <c r="BR21" s="8"/>
       <c r="BS21" s="8"/>
       <c r="BT21" s="8"/>
       <c r="BU21" s="7" t="s">
-        <v>186</v>
+        <v>185</v>
       </c>
       <c r="BV21" s="8"/>
       <c r="BW21" s="8"/>
       <c r="BX21" s="8"/>
       <c r="BY21" s="7" t="s">
-        <v>187</v>
+        <v>186</v>
       </c>
       <c r="BZ21" s="8"/>
       <c r="CA21" s="8"/>
       <c r="CB21" s="8"/>
       <c r="CC21" s="7" t="s">
-        <v>207</v>
+        <v>206</v>
       </c>
       <c r="CD21" s="8"/>
       <c r="CE21" s="8"/>
       <c r="CF21" s="8"/>
       <c r="CG21" s="7" t="s">
-        <v>208</v>
+        <v>207</v>
       </c>
       <c r="CH21" s="8"/>
       <c r="CI21" s="8"/>
       <c r="CJ21" s="8"/>
       <c r="CK21" s="7" t="s">
-        <v>226</v>
+        <v>225</v>
       </c>
       <c r="CL21" s="8"/>
       <c r="CM21" s="8"/>
       <c r="CN21" s="8"/>
       <c r="CO21" s="7" t="s">
-        <v>228</v>
+        <v>227</v>
       </c>
       <c r="CP21" s="8"/>
       <c r="CQ21" s="8"/>
       <c r="CR21" s="8"/>
       <c r="CS21" s="7" t="s">
-        <v>247</v>
+        <v>246</v>
       </c>
       <c r="CT21" s="8"/>
       <c r="CU21" s="8"/>
       <c r="CV21" s="8"/>
       <c r="CW21" s="7" t="s">
-        <v>249</v>
+        <v>248</v>
       </c>
       <c r="CX21" s="8"/>
       <c r="CY21" s="8"/>
       <c r="CZ21" s="8"/>
       <c r="DA21" s="7" t="s">
-        <v>267</v>
+        <v>266</v>
       </c>
       <c r="DB21" s="8"/>
       <c r="DC21" s="8"/>
       <c r="DD21" s="8"/>
-      <c r="DE21" s="7"/>
+      <c r="DE21" s="7" t="s">
+        <v>268</v>
+      </c>
       <c r="DF21" s="8"/>
       <c r="DG21" s="8"/>
       <c r="DH21" s="8"/>
+      <c r="DI21" s="7" t="s">
+        <v>287</v>
+      </c>
+      <c r="DJ21" s="8"/>
+      <c r="DK21" s="8"/>
+      <c r="DL21" s="8"/>
+      <c r="DM21" s="7" t="s">
+        <v>288</v>
+      </c>
+      <c r="DN21" s="8"/>
+      <c r="DO21" s="8"/>
+      <c r="DP21" s="8"/>
     </row>
-    <row r="22" spans="1:112" x14ac:dyDescent="0.3">
+    <row r="22" spans="1:120" x14ac:dyDescent="0.3">
       <c r="A22" s="8"/>
       <c r="B22" s="8"/>
       <c r="C22" s="8"/>
@@ -8546,8 +9391,16 @@
       <c r="DF22" s="8"/>
       <c r="DG22" s="8"/>
       <c r="DH22" s="8"/>
+      <c r="DI22" s="8"/>
+      <c r="DJ22" s="8"/>
+      <c r="DK22" s="8"/>
+      <c r="DL22" s="8"/>
+      <c r="DM22" s="8"/>
+      <c r="DN22" s="8"/>
+      <c r="DO22" s="8"/>
+      <c r="DP22" s="8"/>
     </row>
-    <row r="23" spans="1:112" x14ac:dyDescent="0.3">
+    <row r="23" spans="1:120" x14ac:dyDescent="0.3">
       <c r="A23" s="8"/>
       <c r="B23" s="8"/>
       <c r="C23" s="8"/>
@@ -8660,8 +9513,16 @@
       <c r="DF23" s="8"/>
       <c r="DG23" s="8"/>
       <c r="DH23" s="8"/>
+      <c r="DI23" s="8"/>
+      <c r="DJ23" s="8"/>
+      <c r="DK23" s="8"/>
+      <c r="DL23" s="8"/>
+      <c r="DM23" s="8"/>
+      <c r="DN23" s="8"/>
+      <c r="DO23" s="8"/>
+      <c r="DP23" s="8"/>
     </row>
-    <row r="24" spans="1:112" x14ac:dyDescent="0.3">
+    <row r="24" spans="1:120" x14ac:dyDescent="0.3">
       <c r="A24" s="8"/>
       <c r="B24" s="8"/>
       <c r="C24" s="8"/>
@@ -8774,8 +9635,16 @@
       <c r="DF24" s="8"/>
       <c r="DG24" s="8"/>
       <c r="DH24" s="8"/>
+      <c r="DI24" s="8"/>
+      <c r="DJ24" s="8"/>
+      <c r="DK24" s="8"/>
+      <c r="DL24" s="8"/>
+      <c r="DM24" s="8"/>
+      <c r="DN24" s="8"/>
+      <c r="DO24" s="8"/>
+      <c r="DP24" s="8"/>
     </row>
-    <row r="25" spans="1:112" x14ac:dyDescent="0.3">
+    <row r="25" spans="1:120" x14ac:dyDescent="0.3">
       <c r="A25" s="8"/>
       <c r="B25" s="8"/>
       <c r="C25" s="8"/>
@@ -8888,8 +9757,16 @@
       <c r="DF25" s="8"/>
       <c r="DG25" s="8"/>
       <c r="DH25" s="8"/>
+      <c r="DI25" s="8"/>
+      <c r="DJ25" s="8"/>
+      <c r="DK25" s="8"/>
+      <c r="DL25" s="8"/>
+      <c r="DM25" s="8"/>
+      <c r="DN25" s="8"/>
+      <c r="DO25" s="8"/>
+      <c r="DP25" s="8"/>
     </row>
-    <row r="26" spans="1:112" x14ac:dyDescent="0.3">
+    <row r="26" spans="1:120" x14ac:dyDescent="0.3">
       <c r="A26" s="8"/>
       <c r="B26" s="8"/>
       <c r="C26" s="8"/>
@@ -9002,8 +9879,16 @@
       <c r="DF26" s="8"/>
       <c r="DG26" s="8"/>
       <c r="DH26" s="8"/>
+      <c r="DI26" s="8"/>
+      <c r="DJ26" s="8"/>
+      <c r="DK26" s="8"/>
+      <c r="DL26" s="8"/>
+      <c r="DM26" s="8"/>
+      <c r="DN26" s="8"/>
+      <c r="DO26" s="8"/>
+      <c r="DP26" s="8"/>
     </row>
-    <row r="27" spans="1:112" x14ac:dyDescent="0.3">
+    <row r="27" spans="1:120" x14ac:dyDescent="0.3">
       <c r="A27" s="8"/>
       <c r="B27" s="8"/>
       <c r="C27" s="8"/>
@@ -9116,8 +10001,16 @@
       <c r="DF27" s="8"/>
       <c r="DG27" s="8"/>
       <c r="DH27" s="8"/>
+      <c r="DI27" s="8"/>
+      <c r="DJ27" s="8"/>
+      <c r="DK27" s="8"/>
+      <c r="DL27" s="8"/>
+      <c r="DM27" s="8"/>
+      <c r="DN27" s="8"/>
+      <c r="DO27" s="8"/>
+      <c r="DP27" s="8"/>
     </row>
-    <row r="28" spans="1:112" x14ac:dyDescent="0.3">
+    <row r="28" spans="1:120" x14ac:dyDescent="0.3">
       <c r="A28" s="8"/>
       <c r="B28" s="8"/>
       <c r="C28" s="8"/>
@@ -9230,8 +10123,16 @@
       <c r="DF28" s="8"/>
       <c r="DG28" s="8"/>
       <c r="DH28" s="8"/>
+      <c r="DI28" s="8"/>
+      <c r="DJ28" s="8"/>
+      <c r="DK28" s="8"/>
+      <c r="DL28" s="8"/>
+      <c r="DM28" s="8"/>
+      <c r="DN28" s="8"/>
+      <c r="DO28" s="8"/>
+      <c r="DP28" s="8"/>
     </row>
-    <row r="29" spans="1:112" x14ac:dyDescent="0.3">
+    <row r="29" spans="1:120" x14ac:dyDescent="0.3">
       <c r="A29" s="8"/>
       <c r="B29" s="8"/>
       <c r="C29" s="8"/>
@@ -9344,8 +10245,16 @@
       <c r="DF29" s="8"/>
       <c r="DG29" s="8"/>
       <c r="DH29" s="8"/>
+      <c r="DI29" s="8"/>
+      <c r="DJ29" s="8"/>
+      <c r="DK29" s="8"/>
+      <c r="DL29" s="8"/>
+      <c r="DM29" s="8"/>
+      <c r="DN29" s="8"/>
+      <c r="DO29" s="8"/>
+      <c r="DP29" s="8"/>
     </row>
-    <row r="30" spans="1:112" x14ac:dyDescent="0.3">
+    <row r="30" spans="1:120" x14ac:dyDescent="0.3">
       <c r="A30" s="8"/>
       <c r="B30" s="8"/>
       <c r="C30" s="8"/>
@@ -9458,8 +10367,16 @@
       <c r="DF30" s="8"/>
       <c r="DG30" s="8"/>
       <c r="DH30" s="8"/>
+      <c r="DI30" s="8"/>
+      <c r="DJ30" s="8"/>
+      <c r="DK30" s="8"/>
+      <c r="DL30" s="8"/>
+      <c r="DM30" s="8"/>
+      <c r="DN30" s="8"/>
+      <c r="DO30" s="8"/>
+      <c r="DP30" s="8"/>
     </row>
-    <row r="31" spans="1:112" x14ac:dyDescent="0.3">
+    <row r="31" spans="1:120" x14ac:dyDescent="0.3">
       <c r="A31" s="7" t="s">
         <v>13</v>
       </c>
@@ -9521,111 +10438,123 @@
       <c r="AM31" s="8"/>
       <c r="AN31" s="8"/>
       <c r="AO31" s="7" t="s">
-        <v>108</v>
+        <v>107</v>
       </c>
       <c r="AP31" s="8"/>
       <c r="AQ31" s="8"/>
       <c r="AR31" s="8"/>
       <c r="AS31" s="7" t="s">
-        <v>110</v>
+        <v>109</v>
       </c>
       <c r="AT31" s="8"/>
       <c r="AU31" s="8"/>
       <c r="AV31" s="8"/>
       <c r="AW31" s="7" t="s">
-        <v>129</v>
+        <v>128</v>
       </c>
       <c r="AX31" s="8"/>
       <c r="AY31" s="8"/>
       <c r="AZ31" s="8"/>
       <c r="BA31" s="7" t="s">
-        <v>132</v>
+        <v>131</v>
       </c>
       <c r="BB31" s="8"/>
       <c r="BC31" s="8"/>
       <c r="BD31" s="8"/>
       <c r="BE31" s="7" t="s">
-        <v>148</v>
+        <v>147</v>
       </c>
       <c r="BF31" s="8"/>
       <c r="BG31" s="8"/>
       <c r="BH31" s="8"/>
       <c r="BI31" s="7" t="s">
-        <v>151</v>
+        <v>150</v>
       </c>
       <c r="BJ31" s="8"/>
       <c r="BK31" s="8"/>
       <c r="BL31" s="8"/>
       <c r="BM31" s="7" t="s">
-        <v>170</v>
+        <v>169</v>
       </c>
       <c r="BN31" s="8"/>
       <c r="BO31" s="8"/>
       <c r="BP31" s="8"/>
       <c r="BQ31" s="7" t="s">
-        <v>172</v>
+        <v>171</v>
       </c>
       <c r="BR31" s="8"/>
       <c r="BS31" s="8"/>
       <c r="BT31" s="8"/>
       <c r="BU31" s="7" t="s">
-        <v>189</v>
+        <v>188</v>
       </c>
       <c r="BV31" s="8"/>
       <c r="BW31" s="8"/>
       <c r="BX31" s="8"/>
       <c r="BY31" s="7" t="s">
-        <v>192</v>
+        <v>191</v>
       </c>
       <c r="BZ31" s="8"/>
       <c r="CA31" s="8"/>
       <c r="CB31" s="8"/>
       <c r="CC31" s="7" t="s">
-        <v>210</v>
+        <v>209</v>
       </c>
       <c r="CD31" s="8"/>
       <c r="CE31" s="8"/>
       <c r="CF31" s="8"/>
       <c r="CG31" s="7" t="s">
-        <v>212</v>
+        <v>211</v>
       </c>
       <c r="CH31" s="8"/>
       <c r="CI31" s="8"/>
       <c r="CJ31" s="8"/>
       <c r="CK31" s="7" t="s">
-        <v>230</v>
+        <v>229</v>
       </c>
       <c r="CL31" s="8"/>
       <c r="CM31" s="8"/>
       <c r="CN31" s="8"/>
       <c r="CO31" s="7" t="s">
-        <v>233</v>
+        <v>232</v>
       </c>
       <c r="CP31" s="8"/>
       <c r="CQ31" s="8"/>
       <c r="CR31" s="8"/>
       <c r="CS31" s="7" t="s">
-        <v>253</v>
+        <v>252</v>
       </c>
       <c r="CT31" s="8"/>
       <c r="CU31" s="8"/>
       <c r="CV31" s="8"/>
       <c r="CW31" s="7" t="s">
-        <v>252</v>
+        <v>251</v>
       </c>
       <c r="CX31" s="8"/>
       <c r="CY31" s="8"/>
       <c r="CZ31" s="8"/>
-      <c r="DA31" s="7"/>
+      <c r="DA31" s="7" t="s">
+        <v>271</v>
+      </c>
       <c r="DB31" s="8"/>
       <c r="DC31" s="8"/>
       <c r="DD31" s="8"/>
-      <c r="DE31" s="7"/>
+      <c r="DE31" s="7" t="s">
+        <v>273</v>
+      </c>
       <c r="DF31" s="8"/>
       <c r="DG31" s="8"/>
       <c r="DH31" s="8"/>
+      <c r="DI31" s="7"/>
+      <c r="DJ31" s="8"/>
+      <c r="DK31" s="8"/>
+      <c r="DL31" s="8"/>
+      <c r="DM31" s="7"/>
+      <c r="DN31" s="8"/>
+      <c r="DO31" s="8"/>
+      <c r="DP31" s="8"/>
     </row>
-    <row r="32" spans="1:112" x14ac:dyDescent="0.3">
+    <row r="32" spans="1:120" x14ac:dyDescent="0.3">
       <c r="A32" s="8"/>
       <c r="B32" s="8"/>
       <c r="C32" s="8"/>
@@ -9738,8 +10667,16 @@
       <c r="DF32" s="8"/>
       <c r="DG32" s="8"/>
       <c r="DH32" s="8"/>
+      <c r="DI32" s="8"/>
+      <c r="DJ32" s="8"/>
+      <c r="DK32" s="8"/>
+      <c r="DL32" s="8"/>
+      <c r="DM32" s="8"/>
+      <c r="DN32" s="8"/>
+      <c r="DO32" s="8"/>
+      <c r="DP32" s="8"/>
     </row>
-    <row r="33" spans="1:112" x14ac:dyDescent="0.3">
+    <row r="33" spans="1:120" x14ac:dyDescent="0.3">
       <c r="A33" s="8"/>
       <c r="B33" s="8"/>
       <c r="C33" s="8"/>
@@ -9852,8 +10789,16 @@
       <c r="DF33" s="8"/>
       <c r="DG33" s="8"/>
       <c r="DH33" s="8"/>
+      <c r="DI33" s="8"/>
+      <c r="DJ33" s="8"/>
+      <c r="DK33" s="8"/>
+      <c r="DL33" s="8"/>
+      <c r="DM33" s="8"/>
+      <c r="DN33" s="8"/>
+      <c r="DO33" s="8"/>
+      <c r="DP33" s="8"/>
     </row>
-    <row r="34" spans="1:112" x14ac:dyDescent="0.3">
+    <row r="34" spans="1:120" x14ac:dyDescent="0.3">
       <c r="A34" s="8"/>
       <c r="B34" s="8"/>
       <c r="C34" s="8"/>
@@ -9966,8 +10911,16 @@
       <c r="DF34" s="8"/>
       <c r="DG34" s="8"/>
       <c r="DH34" s="8"/>
+      <c r="DI34" s="8"/>
+      <c r="DJ34" s="8"/>
+      <c r="DK34" s="8"/>
+      <c r="DL34" s="8"/>
+      <c r="DM34" s="8"/>
+      <c r="DN34" s="8"/>
+      <c r="DO34" s="8"/>
+      <c r="DP34" s="8"/>
     </row>
-    <row r="35" spans="1:112" x14ac:dyDescent="0.3">
+    <row r="35" spans="1:120" x14ac:dyDescent="0.3">
       <c r="A35" s="8"/>
       <c r="B35" s="8"/>
       <c r="C35" s="8"/>
@@ -10080,8 +11033,16 @@
       <c r="DF35" s="8"/>
       <c r="DG35" s="8"/>
       <c r="DH35" s="8"/>
+      <c r="DI35" s="8"/>
+      <c r="DJ35" s="8"/>
+      <c r="DK35" s="8"/>
+      <c r="DL35" s="8"/>
+      <c r="DM35" s="8"/>
+      <c r="DN35" s="8"/>
+      <c r="DO35" s="8"/>
+      <c r="DP35" s="8"/>
     </row>
-    <row r="36" spans="1:112" x14ac:dyDescent="0.3">
+    <row r="36" spans="1:120" x14ac:dyDescent="0.3">
       <c r="A36" s="8"/>
       <c r="B36" s="8"/>
       <c r="C36" s="8"/>
@@ -10194,8 +11155,16 @@
       <c r="DF36" s="8"/>
       <c r="DG36" s="8"/>
       <c r="DH36" s="8"/>
+      <c r="DI36" s="8"/>
+      <c r="DJ36" s="8"/>
+      <c r="DK36" s="8"/>
+      <c r="DL36" s="8"/>
+      <c r="DM36" s="8"/>
+      <c r="DN36" s="8"/>
+      <c r="DO36" s="8"/>
+      <c r="DP36" s="8"/>
     </row>
-    <row r="37" spans="1:112" x14ac:dyDescent="0.3">
+    <row r="37" spans="1:120" x14ac:dyDescent="0.3">
       <c r="A37" s="8"/>
       <c r="B37" s="8"/>
       <c r="C37" s="8"/>
@@ -10308,8 +11277,16 @@
       <c r="DF37" s="8"/>
       <c r="DG37" s="8"/>
       <c r="DH37" s="8"/>
+      <c r="DI37" s="8"/>
+      <c r="DJ37" s="8"/>
+      <c r="DK37" s="8"/>
+      <c r="DL37" s="8"/>
+      <c r="DM37" s="8"/>
+      <c r="DN37" s="8"/>
+      <c r="DO37" s="8"/>
+      <c r="DP37" s="8"/>
     </row>
-    <row r="38" spans="1:112" x14ac:dyDescent="0.3">
+    <row r="38" spans="1:120" x14ac:dyDescent="0.3">
       <c r="A38" s="8"/>
       <c r="B38" s="8"/>
       <c r="C38" s="8"/>
@@ -10422,8 +11399,16 @@
       <c r="DF38" s="8"/>
       <c r="DG38" s="8"/>
       <c r="DH38" s="8"/>
+      <c r="DI38" s="8"/>
+      <c r="DJ38" s="8"/>
+      <c r="DK38" s="8"/>
+      <c r="DL38" s="8"/>
+      <c r="DM38" s="8"/>
+      <c r="DN38" s="8"/>
+      <c r="DO38" s="8"/>
+      <c r="DP38" s="8"/>
     </row>
-    <row r="39" spans="1:112" x14ac:dyDescent="0.3">
+    <row r="39" spans="1:120" x14ac:dyDescent="0.3">
       <c r="A39" s="8"/>
       <c r="B39" s="8"/>
       <c r="C39" s="8"/>
@@ -10536,8 +11521,16 @@
       <c r="DF39" s="8"/>
       <c r="DG39" s="8"/>
       <c r="DH39" s="8"/>
+      <c r="DI39" s="8"/>
+      <c r="DJ39" s="8"/>
+      <c r="DK39" s="8"/>
+      <c r="DL39" s="8"/>
+      <c r="DM39" s="8"/>
+      <c r="DN39" s="8"/>
+      <c r="DO39" s="8"/>
+      <c r="DP39" s="8"/>
     </row>
-    <row r="40" spans="1:112" x14ac:dyDescent="0.3">
+    <row r="40" spans="1:120" x14ac:dyDescent="0.3">
       <c r="A40" s="8"/>
       <c r="B40" s="8"/>
       <c r="C40" s="8"/>
@@ -10650,8 +11643,16 @@
       <c r="DF40" s="8"/>
       <c r="DG40" s="8"/>
       <c r="DH40" s="8"/>
+      <c r="DI40" s="8"/>
+      <c r="DJ40" s="8"/>
+      <c r="DK40" s="8"/>
+      <c r="DL40" s="8"/>
+      <c r="DM40" s="8"/>
+      <c r="DN40" s="8"/>
+      <c r="DO40" s="8"/>
+      <c r="DP40" s="8"/>
     </row>
-    <row r="41" spans="1:112" x14ac:dyDescent="0.3">
+    <row r="41" spans="1:120" x14ac:dyDescent="0.3">
       <c r="A41" s="7" t="s">
         <v>16</v>
       </c>
@@ -10689,7 +11690,7 @@
       <c r="W41" s="8"/>
       <c r="X41" s="8"/>
       <c r="Y41" s="7" t="s">
-        <v>131</v>
+        <v>130</v>
       </c>
       <c r="Z41" s="8"/>
       <c r="AA41" s="8"/>
@@ -10713,111 +11714,123 @@
       <c r="AM41" s="8"/>
       <c r="AN41" s="8"/>
       <c r="AO41" s="7" t="s">
-        <v>112</v>
+        <v>111</v>
       </c>
       <c r="AP41" s="8"/>
       <c r="AQ41" s="8"/>
       <c r="AR41" s="8"/>
       <c r="AS41" s="7" t="s">
-        <v>114</v>
+        <v>113</v>
       </c>
       <c r="AT41" s="8"/>
       <c r="AU41" s="8"/>
       <c r="AV41" s="8"/>
       <c r="AW41" s="7" t="s">
-        <v>134</v>
+        <v>133</v>
       </c>
       <c r="AX41" s="8"/>
       <c r="AY41" s="8"/>
       <c r="AZ41" s="8"/>
       <c r="BA41" s="7" t="s">
-        <v>153</v>
+        <v>152</v>
       </c>
       <c r="BB41" s="8"/>
       <c r="BC41" s="8"/>
       <c r="BD41" s="8"/>
       <c r="BE41" s="7" t="s">
-        <v>154</v>
+        <v>153</v>
       </c>
       <c r="BF41" s="8"/>
       <c r="BG41" s="8"/>
       <c r="BH41" s="8"/>
       <c r="BI41" s="7" t="s">
-        <v>156</v>
+        <v>155</v>
       </c>
       <c r="BJ41" s="8"/>
       <c r="BK41" s="8"/>
       <c r="BL41" s="8"/>
       <c r="BM41" s="7" t="s">
-        <v>174</v>
+        <v>173</v>
       </c>
       <c r="BN41" s="8"/>
       <c r="BO41" s="8"/>
       <c r="BP41" s="8"/>
       <c r="BQ41" s="9" t="s">
-        <v>177</v>
+        <v>176</v>
       </c>
       <c r="BR41" s="8"/>
       <c r="BS41" s="8"/>
       <c r="BT41" s="8"/>
       <c r="BU41" s="7" t="s">
-        <v>194</v>
+        <v>193</v>
       </c>
       <c r="BV41" s="8"/>
       <c r="BW41" s="8"/>
       <c r="BX41" s="8"/>
       <c r="BY41" s="9" t="s">
-        <v>195</v>
+        <v>194</v>
       </c>
       <c r="BZ41" s="8"/>
       <c r="CA41" s="8"/>
       <c r="CB41" s="8"/>
       <c r="CC41" s="7" t="s">
-        <v>215</v>
+        <v>214</v>
       </c>
       <c r="CD41" s="8"/>
       <c r="CE41" s="8"/>
       <c r="CF41" s="8"/>
       <c r="CG41" s="9" t="s">
-        <v>216</v>
+        <v>215</v>
       </c>
       <c r="CH41" s="8"/>
       <c r="CI41" s="8"/>
       <c r="CJ41" s="8"/>
       <c r="CK41" s="7" t="s">
-        <v>235</v>
+        <v>234</v>
       </c>
       <c r="CL41" s="8"/>
       <c r="CM41" s="8"/>
       <c r="CN41" s="8"/>
       <c r="CO41" s="9" t="s">
-        <v>237</v>
+        <v>236</v>
       </c>
       <c r="CP41" s="8"/>
       <c r="CQ41" s="8"/>
       <c r="CR41" s="8"/>
       <c r="CS41" s="7" t="s">
-        <v>255</v>
+        <v>254</v>
       </c>
       <c r="CT41" s="8"/>
       <c r="CU41" s="8"/>
       <c r="CV41" s="8"/>
       <c r="CW41" s="9" t="s">
-        <v>256</v>
+        <v>255</v>
       </c>
       <c r="CX41" s="8"/>
       <c r="CY41" s="8"/>
       <c r="CZ41" s="8"/>
-      <c r="DA41" s="7"/>
+      <c r="DA41" s="7" t="s">
+        <v>275</v>
+      </c>
       <c r="DB41" s="8"/>
       <c r="DC41" s="8"/>
       <c r="DD41" s="8"/>
-      <c r="DE41" s="9"/>
+      <c r="DE41" s="9" t="s">
+        <v>278</v>
+      </c>
       <c r="DF41" s="8"/>
       <c r="DG41" s="8"/>
       <c r="DH41" s="8"/>
+      <c r="DI41" s="7"/>
+      <c r="DJ41" s="8"/>
+      <c r="DK41" s="8"/>
+      <c r="DL41" s="8"/>
+      <c r="DM41" s="9"/>
+      <c r="DN41" s="8"/>
+      <c r="DO41" s="8"/>
+      <c r="DP41" s="8"/>
     </row>
-    <row r="42" spans="1:112" x14ac:dyDescent="0.3">
+    <row r="42" spans="1:120" x14ac:dyDescent="0.3">
       <c r="A42" s="8"/>
       <c r="B42" s="8"/>
       <c r="C42" s="8"/>
@@ -10930,8 +11943,16 @@
       <c r="DF42" s="8"/>
       <c r="DG42" s="8"/>
       <c r="DH42" s="8"/>
+      <c r="DI42" s="8"/>
+      <c r="DJ42" s="8"/>
+      <c r="DK42" s="8"/>
+      <c r="DL42" s="8"/>
+      <c r="DM42" s="8"/>
+      <c r="DN42" s="8"/>
+      <c r="DO42" s="8"/>
+      <c r="DP42" s="8"/>
     </row>
-    <row r="43" spans="1:112" x14ac:dyDescent="0.3">
+    <row r="43" spans="1:120" x14ac:dyDescent="0.3">
       <c r="A43" s="8"/>
       <c r="B43" s="8"/>
       <c r="C43" s="8"/>
@@ -11044,8 +12065,16 @@
       <c r="DF43" s="8"/>
       <c r="DG43" s="8"/>
       <c r="DH43" s="8"/>
+      <c r="DI43" s="8"/>
+      <c r="DJ43" s="8"/>
+      <c r="DK43" s="8"/>
+      <c r="DL43" s="8"/>
+      <c r="DM43" s="8"/>
+      <c r="DN43" s="8"/>
+      <c r="DO43" s="8"/>
+      <c r="DP43" s="8"/>
     </row>
-    <row r="44" spans="1:112" x14ac:dyDescent="0.3">
+    <row r="44" spans="1:120" x14ac:dyDescent="0.3">
       <c r="A44" s="8"/>
       <c r="B44" s="8"/>
       <c r="C44" s="8"/>
@@ -11158,8 +12187,16 @@
       <c r="DF44" s="8"/>
       <c r="DG44" s="8"/>
       <c r="DH44" s="8"/>
+      <c r="DI44" s="8"/>
+      <c r="DJ44" s="8"/>
+      <c r="DK44" s="8"/>
+      <c r="DL44" s="8"/>
+      <c r="DM44" s="8"/>
+      <c r="DN44" s="8"/>
+      <c r="DO44" s="8"/>
+      <c r="DP44" s="8"/>
     </row>
-    <row r="45" spans="1:112" x14ac:dyDescent="0.3">
+    <row r="45" spans="1:120" x14ac:dyDescent="0.3">
       <c r="A45" s="8"/>
       <c r="B45" s="8"/>
       <c r="C45" s="8"/>
@@ -11272,8 +12309,16 @@
       <c r="DF45" s="8"/>
       <c r="DG45" s="8"/>
       <c r="DH45" s="8"/>
+      <c r="DI45" s="8"/>
+      <c r="DJ45" s="8"/>
+      <c r="DK45" s="8"/>
+      <c r="DL45" s="8"/>
+      <c r="DM45" s="8"/>
+      <c r="DN45" s="8"/>
+      <c r="DO45" s="8"/>
+      <c r="DP45" s="8"/>
     </row>
-    <row r="46" spans="1:112" x14ac:dyDescent="0.3">
+    <row r="46" spans="1:120" x14ac:dyDescent="0.3">
       <c r="A46" s="8"/>
       <c r="B46" s="8"/>
       <c r="C46" s="8"/>
@@ -11386,8 +12431,16 @@
       <c r="DF46" s="8"/>
       <c r="DG46" s="8"/>
       <c r="DH46" s="8"/>
+      <c r="DI46" s="8"/>
+      <c r="DJ46" s="8"/>
+      <c r="DK46" s="8"/>
+      <c r="DL46" s="8"/>
+      <c r="DM46" s="8"/>
+      <c r="DN46" s="8"/>
+      <c r="DO46" s="8"/>
+      <c r="DP46" s="8"/>
     </row>
-    <row r="47" spans="1:112" x14ac:dyDescent="0.3">
+    <row r="47" spans="1:120" x14ac:dyDescent="0.3">
       <c r="A47" s="8"/>
       <c r="B47" s="8"/>
       <c r="C47" s="8"/>
@@ -11500,8 +12553,16 @@
       <c r="DF47" s="8"/>
       <c r="DG47" s="8"/>
       <c r="DH47" s="8"/>
+      <c r="DI47" s="8"/>
+      <c r="DJ47" s="8"/>
+      <c r="DK47" s="8"/>
+      <c r="DL47" s="8"/>
+      <c r="DM47" s="8"/>
+      <c r="DN47" s="8"/>
+      <c r="DO47" s="8"/>
+      <c r="DP47" s="8"/>
     </row>
-    <row r="48" spans="1:112" x14ac:dyDescent="0.3">
+    <row r="48" spans="1:120" x14ac:dyDescent="0.3">
       <c r="A48" s="8"/>
       <c r="B48" s="8"/>
       <c r="C48" s="8"/>
@@ -11614,8 +12675,16 @@
       <c r="DF48" s="8"/>
       <c r="DG48" s="8"/>
       <c r="DH48" s="8"/>
+      <c r="DI48" s="8"/>
+      <c r="DJ48" s="8"/>
+      <c r="DK48" s="8"/>
+      <c r="DL48" s="8"/>
+      <c r="DM48" s="8"/>
+      <c r="DN48" s="8"/>
+      <c r="DO48" s="8"/>
+      <c r="DP48" s="8"/>
     </row>
-    <row r="49" spans="1:112" x14ac:dyDescent="0.3">
+    <row r="49" spans="1:120" x14ac:dyDescent="0.3">
       <c r="A49" s="8"/>
       <c r="B49" s="8"/>
       <c r="C49" s="8"/>
@@ -11728,8 +12797,16 @@
       <c r="DF49" s="8"/>
       <c r="DG49" s="8"/>
       <c r="DH49" s="8"/>
+      <c r="DI49" s="8"/>
+      <c r="DJ49" s="8"/>
+      <c r="DK49" s="8"/>
+      <c r="DL49" s="8"/>
+      <c r="DM49" s="8"/>
+      <c r="DN49" s="8"/>
+      <c r="DO49" s="8"/>
+      <c r="DP49" s="8"/>
     </row>
-    <row r="50" spans="1:112" x14ac:dyDescent="0.3">
+    <row r="50" spans="1:120" x14ac:dyDescent="0.3">
       <c r="A50" s="8"/>
       <c r="B50" s="8"/>
       <c r="C50" s="8"/>
@@ -11842,8 +12919,16 @@
       <c r="DF50" s="8"/>
       <c r="DG50" s="8"/>
       <c r="DH50" s="8"/>
+      <c r="DI50" s="8"/>
+      <c r="DJ50" s="8"/>
+      <c r="DK50" s="8"/>
+      <c r="DL50" s="8"/>
+      <c r="DM50" s="8"/>
+      <c r="DN50" s="8"/>
+      <c r="DO50" s="8"/>
+      <c r="DP50" s="8"/>
     </row>
-    <row r="51" spans="1:112" x14ac:dyDescent="0.3">
+    <row r="51" spans="1:120" x14ac:dyDescent="0.3">
       <c r="A51" s="5" t="s">
         <v>6</v>
       </c>
@@ -11917,103 +13002,115 @@
       <c r="AU51" s="6"/>
       <c r="AV51" s="6"/>
       <c r="AW51" s="5" t="s">
-        <v>119</v>
+        <v>118</v>
       </c>
       <c r="AX51" s="6"/>
       <c r="AY51" s="6"/>
       <c r="AZ51" s="6"/>
       <c r="BA51" s="5" t="s">
-        <v>117</v>
+        <v>116</v>
       </c>
       <c r="BB51" s="6"/>
       <c r="BC51" s="6"/>
       <c r="BD51" s="6"/>
       <c r="BE51" s="5" t="s">
-        <v>140</v>
+        <v>139</v>
       </c>
       <c r="BF51" s="6"/>
       <c r="BG51" s="6"/>
       <c r="BH51" s="6"/>
       <c r="BI51" s="5" t="s">
-        <v>139</v>
+        <v>138</v>
       </c>
       <c r="BJ51" s="6"/>
       <c r="BK51" s="6"/>
       <c r="BL51" s="6"/>
       <c r="BM51" s="5" t="s">
-        <v>161</v>
+        <v>160</v>
       </c>
       <c r="BN51" s="6"/>
       <c r="BO51" s="6"/>
       <c r="BP51" s="6"/>
       <c r="BQ51" s="5" t="s">
-        <v>159</v>
+        <v>158</v>
       </c>
       <c r="BR51" s="6"/>
       <c r="BS51" s="6"/>
       <c r="BT51" s="6"/>
       <c r="BU51" s="5" t="s">
-        <v>181</v>
+        <v>180</v>
       </c>
       <c r="BV51" s="6"/>
       <c r="BW51" s="6"/>
       <c r="BX51" s="6"/>
       <c r="BY51" s="5" t="s">
-        <v>179</v>
+        <v>178</v>
       </c>
       <c r="BZ51" s="6"/>
       <c r="CA51" s="6"/>
       <c r="CB51" s="6"/>
       <c r="CC51" s="5" t="s">
-        <v>201</v>
+        <v>200</v>
       </c>
       <c r="CD51" s="6"/>
       <c r="CE51" s="6"/>
       <c r="CF51" s="6"/>
       <c r="CG51" s="5" t="s">
-        <v>199</v>
+        <v>198</v>
       </c>
       <c r="CH51" s="6"/>
       <c r="CI51" s="6"/>
       <c r="CJ51" s="6"/>
       <c r="CK51" s="5" t="s">
-        <v>221</v>
+        <v>220</v>
       </c>
       <c r="CL51" s="6"/>
       <c r="CM51" s="6"/>
       <c r="CN51" s="6"/>
       <c r="CO51" s="5" t="s">
-        <v>218</v>
+        <v>217</v>
       </c>
       <c r="CP51" s="6"/>
       <c r="CQ51" s="6"/>
       <c r="CR51" s="6"/>
       <c r="CS51" s="5" t="s">
-        <v>241</v>
+        <v>240</v>
       </c>
       <c r="CT51" s="6"/>
       <c r="CU51" s="6"/>
       <c r="CV51" s="6"/>
       <c r="CW51" s="5" t="s">
-        <v>240</v>
+        <v>239</v>
       </c>
       <c r="CX51" s="6"/>
       <c r="CY51" s="6"/>
       <c r="CZ51" s="6"/>
       <c r="DA51" s="5" t="s">
-        <v>262</v>
+        <v>261</v>
       </c>
       <c r="DB51" s="6"/>
       <c r="DC51" s="6"/>
       <c r="DD51" s="6"/>
       <c r="DE51" s="5" t="s">
-        <v>260</v>
+        <v>259</v>
       </c>
       <c r="DF51" s="6"/>
       <c r="DG51" s="6"/>
       <c r="DH51" s="6"/>
+      <c r="DI51" s="5" t="s">
+        <v>282</v>
+      </c>
+      <c r="DJ51" s="6"/>
+      <c r="DK51" s="6"/>
+      <c r="DL51" s="6"/>
+      <c r="DM51" s="5" t="s">
+        <v>280</v>
+      </c>
+      <c r="DN51" s="6"/>
+      <c r="DO51" s="6"/>
+      <c r="DP51" s="6"/>
     </row>
-    <row r="52" spans="1:112" x14ac:dyDescent="0.3">
+    <row r="52" spans="1:120" x14ac:dyDescent="0.3">
       <c r="A52" s="6"/>
       <c r="B52" s="6"/>
       <c r="C52" s="6"/>
@@ -12126,8 +13223,16 @@
       <c r="DF52" s="6"/>
       <c r="DG52" s="6"/>
       <c r="DH52" s="6"/>
+      <c r="DI52" s="6"/>
+      <c r="DJ52" s="6"/>
+      <c r="DK52" s="6"/>
+      <c r="DL52" s="6"/>
+      <c r="DM52" s="6"/>
+      <c r="DN52" s="6"/>
+      <c r="DO52" s="6"/>
+      <c r="DP52" s="6"/>
     </row>
-    <row r="53" spans="1:112" x14ac:dyDescent="0.3">
+    <row r="53" spans="1:120" x14ac:dyDescent="0.3">
       <c r="A53" s="6"/>
       <c r="B53" s="6"/>
       <c r="C53" s="6"/>
@@ -12240,8 +13345,16 @@
       <c r="DF53" s="6"/>
       <c r="DG53" s="6"/>
       <c r="DH53" s="6"/>
+      <c r="DI53" s="6"/>
+      <c r="DJ53" s="6"/>
+      <c r="DK53" s="6"/>
+      <c r="DL53" s="6"/>
+      <c r="DM53" s="6"/>
+      <c r="DN53" s="6"/>
+      <c r="DO53" s="6"/>
+      <c r="DP53" s="6"/>
     </row>
-    <row r="54" spans="1:112" x14ac:dyDescent="0.3">
+    <row r="54" spans="1:120" x14ac:dyDescent="0.3">
       <c r="A54" s="6"/>
       <c r="B54" s="6"/>
       <c r="C54" s="6"/>
@@ -12354,8 +13467,16 @@
       <c r="DF54" s="6"/>
       <c r="DG54" s="6"/>
       <c r="DH54" s="6"/>
+      <c r="DI54" s="6"/>
+      <c r="DJ54" s="6"/>
+      <c r="DK54" s="6"/>
+      <c r="DL54" s="6"/>
+      <c r="DM54" s="6"/>
+      <c r="DN54" s="6"/>
+      <c r="DO54" s="6"/>
+      <c r="DP54" s="6"/>
     </row>
-    <row r="55" spans="1:112" x14ac:dyDescent="0.3">
+    <row r="55" spans="1:120" x14ac:dyDescent="0.3">
       <c r="A55" s="6"/>
       <c r="B55" s="6"/>
       <c r="C55" s="6"/>
@@ -12468,8 +13589,16 @@
       <c r="DF55" s="6"/>
       <c r="DG55" s="6"/>
       <c r="DH55" s="6"/>
+      <c r="DI55" s="6"/>
+      <c r="DJ55" s="6"/>
+      <c r="DK55" s="6"/>
+      <c r="DL55" s="6"/>
+      <c r="DM55" s="6"/>
+      <c r="DN55" s="6"/>
+      <c r="DO55" s="6"/>
+      <c r="DP55" s="6"/>
     </row>
-    <row r="56" spans="1:112" x14ac:dyDescent="0.3">
+    <row r="56" spans="1:120" x14ac:dyDescent="0.3">
       <c r="A56" s="6"/>
       <c r="B56" s="6"/>
       <c r="C56" s="6"/>
@@ -12582,8 +13711,16 @@
       <c r="DF56" s="6"/>
       <c r="DG56" s="6"/>
       <c r="DH56" s="6"/>
+      <c r="DI56" s="6"/>
+      <c r="DJ56" s="6"/>
+      <c r="DK56" s="6"/>
+      <c r="DL56" s="6"/>
+      <c r="DM56" s="6"/>
+      <c r="DN56" s="6"/>
+      <c r="DO56" s="6"/>
+      <c r="DP56" s="6"/>
     </row>
-    <row r="57" spans="1:112" x14ac:dyDescent="0.3">
+    <row r="57" spans="1:120" x14ac:dyDescent="0.3">
       <c r="A57" s="6"/>
       <c r="B57" s="6"/>
       <c r="C57" s="6"/>
@@ -12696,8 +13833,16 @@
       <c r="DF57" s="6"/>
       <c r="DG57" s="6"/>
       <c r="DH57" s="6"/>
+      <c r="DI57" s="6"/>
+      <c r="DJ57" s="6"/>
+      <c r="DK57" s="6"/>
+      <c r="DL57" s="6"/>
+      <c r="DM57" s="6"/>
+      <c r="DN57" s="6"/>
+      <c r="DO57" s="6"/>
+      <c r="DP57" s="6"/>
     </row>
-    <row r="58" spans="1:112" x14ac:dyDescent="0.3">
+    <row r="58" spans="1:120" x14ac:dyDescent="0.3">
       <c r="A58" s="6"/>
       <c r="B58" s="6"/>
       <c r="C58" s="6"/>
@@ -12810,8 +13955,16 @@
       <c r="DF58" s="6"/>
       <c r="DG58" s="6"/>
       <c r="DH58" s="6"/>
+      <c r="DI58" s="6"/>
+      <c r="DJ58" s="6"/>
+      <c r="DK58" s="6"/>
+      <c r="DL58" s="6"/>
+      <c r="DM58" s="6"/>
+      <c r="DN58" s="6"/>
+      <c r="DO58" s="6"/>
+      <c r="DP58" s="6"/>
     </row>
-    <row r="59" spans="1:112" x14ac:dyDescent="0.3">
+    <row r="59" spans="1:120" x14ac:dyDescent="0.3">
       <c r="A59" s="6"/>
       <c r="B59" s="6"/>
       <c r="C59" s="6"/>
@@ -12924,8 +14077,16 @@
       <c r="DF59" s="6"/>
       <c r="DG59" s="6"/>
       <c r="DH59" s="6"/>
+      <c r="DI59" s="6"/>
+      <c r="DJ59" s="6"/>
+      <c r="DK59" s="6"/>
+      <c r="DL59" s="6"/>
+      <c r="DM59" s="6"/>
+      <c r="DN59" s="6"/>
+      <c r="DO59" s="6"/>
+      <c r="DP59" s="6"/>
     </row>
-    <row r="60" spans="1:112" x14ac:dyDescent="0.3">
+    <row r="60" spans="1:120" x14ac:dyDescent="0.3">
       <c r="A60" s="6"/>
       <c r="B60" s="6"/>
       <c r="C60" s="6"/>
@@ -13038,8 +14199,16 @@
       <c r="DF60" s="6"/>
       <c r="DG60" s="6"/>
       <c r="DH60" s="6"/>
+      <c r="DI60" s="6"/>
+      <c r="DJ60" s="6"/>
+      <c r="DK60" s="6"/>
+      <c r="DL60" s="6"/>
+      <c r="DM60" s="6"/>
+      <c r="DN60" s="6"/>
+      <c r="DO60" s="6"/>
+      <c r="DP60" s="6"/>
     </row>
-    <row r="61" spans="1:112" x14ac:dyDescent="0.3">
+    <row r="61" spans="1:120" x14ac:dyDescent="0.3">
       <c r="A61" s="5" t="s">
         <v>8</v>
       </c>
@@ -13089,7 +14258,7 @@
       <c r="AE61" s="6"/>
       <c r="AF61" s="6"/>
       <c r="AG61" s="5" t="s">
-        <v>232</v>
+        <v>231</v>
       </c>
       <c r="AH61" s="6"/>
       <c r="AI61" s="6"/>
@@ -13101,115 +14270,127 @@
       <c r="AM61" s="6"/>
       <c r="AN61" s="6"/>
       <c r="AO61" s="5" t="s">
-        <v>103</v>
+        <v>102</v>
       </c>
       <c r="AP61" s="6"/>
       <c r="AQ61" s="6"/>
       <c r="AR61" s="6"/>
       <c r="AS61" s="5" t="s">
-        <v>102</v>
+        <v>101</v>
       </c>
       <c r="AT61" s="6"/>
       <c r="AU61" s="6"/>
       <c r="AV61" s="6"/>
       <c r="AW61" s="5" t="s">
-        <v>122</v>
+        <v>121</v>
       </c>
       <c r="AX61" s="6"/>
       <c r="AY61" s="6"/>
       <c r="AZ61" s="6"/>
       <c r="BA61" s="5" t="s">
-        <v>121</v>
+        <v>120</v>
       </c>
       <c r="BB61" s="6"/>
       <c r="BC61" s="6"/>
       <c r="BD61" s="6"/>
       <c r="BE61" s="5" t="s">
-        <v>145</v>
+        <v>144</v>
       </c>
       <c r="BF61" s="6"/>
       <c r="BG61" s="6"/>
       <c r="BH61" s="6"/>
       <c r="BI61" s="5" t="s">
-        <v>144</v>
+        <v>143</v>
       </c>
       <c r="BJ61" s="6"/>
       <c r="BK61" s="6"/>
       <c r="BL61" s="6"/>
       <c r="BM61" s="5" t="s">
-        <v>165</v>
+        <v>164</v>
       </c>
       <c r="BN61" s="6"/>
       <c r="BO61" s="6"/>
       <c r="BP61" s="6"/>
       <c r="BQ61" s="5" t="s">
-        <v>163</v>
+        <v>162</v>
       </c>
       <c r="BR61" s="6"/>
       <c r="BS61" s="6"/>
       <c r="BT61" s="6"/>
       <c r="BU61" s="5" t="s">
-        <v>185</v>
+        <v>184</v>
       </c>
       <c r="BV61" s="6"/>
       <c r="BW61" s="6"/>
       <c r="BX61" s="6"/>
       <c r="BY61" s="5" t="s">
-        <v>184</v>
+        <v>183</v>
       </c>
       <c r="BZ61" s="6"/>
       <c r="CA61" s="6"/>
       <c r="CB61" s="6"/>
       <c r="CC61" s="5" t="s">
-        <v>205</v>
+        <v>204</v>
       </c>
       <c r="CD61" s="6"/>
       <c r="CE61" s="6"/>
       <c r="CF61" s="6"/>
       <c r="CG61" s="5" t="s">
-        <v>203</v>
+        <v>202</v>
       </c>
       <c r="CH61" s="6"/>
       <c r="CI61" s="6"/>
       <c r="CJ61" s="6"/>
       <c r="CK61" s="5" t="s">
-        <v>225</v>
+        <v>224</v>
       </c>
       <c r="CL61" s="6"/>
       <c r="CM61" s="6"/>
       <c r="CN61" s="6"/>
       <c r="CO61" s="5" t="s">
-        <v>223</v>
+        <v>222</v>
       </c>
       <c r="CP61" s="6"/>
       <c r="CQ61" s="6"/>
       <c r="CR61" s="6"/>
       <c r="CS61" s="5" t="s">
-        <v>245</v>
+        <v>244</v>
       </c>
       <c r="CT61" s="6"/>
       <c r="CU61" s="6"/>
       <c r="CV61" s="6"/>
       <c r="CW61" s="5" t="s">
-        <v>243</v>
+        <v>242</v>
       </c>
       <c r="CX61" s="6"/>
       <c r="CY61" s="6"/>
       <c r="CZ61" s="6"/>
       <c r="DA61" s="5" t="s">
-        <v>266</v>
+        <v>265</v>
       </c>
       <c r="DB61" s="6"/>
       <c r="DC61" s="6"/>
       <c r="DD61" s="6"/>
       <c r="DE61" s="5" t="s">
-        <v>264</v>
+        <v>263</v>
       </c>
       <c r="DF61" s="6"/>
       <c r="DG61" s="6"/>
       <c r="DH61" s="6"/>
+      <c r="DI61" s="5" t="s">
+        <v>286</v>
+      </c>
+      <c r="DJ61" s="6"/>
+      <c r="DK61" s="6"/>
+      <c r="DL61" s="6"/>
+      <c r="DM61" s="5" t="s">
+        <v>283</v>
+      </c>
+      <c r="DN61" s="6"/>
+      <c r="DO61" s="6"/>
+      <c r="DP61" s="6"/>
     </row>
-    <row r="62" spans="1:112" x14ac:dyDescent="0.3">
+    <row r="62" spans="1:120" x14ac:dyDescent="0.3">
       <c r="A62" s="6"/>
       <c r="B62" s="6"/>
       <c r="C62" s="6"/>
@@ -13322,8 +14503,16 @@
       <c r="DF62" s="6"/>
       <c r="DG62" s="6"/>
       <c r="DH62" s="6"/>
+      <c r="DI62" s="6"/>
+      <c r="DJ62" s="6"/>
+      <c r="DK62" s="6"/>
+      <c r="DL62" s="6"/>
+      <c r="DM62" s="6"/>
+      <c r="DN62" s="6"/>
+      <c r="DO62" s="6"/>
+      <c r="DP62" s="6"/>
     </row>
-    <row r="63" spans="1:112" x14ac:dyDescent="0.3">
+    <row r="63" spans="1:120" x14ac:dyDescent="0.3">
       <c r="A63" s="6"/>
       <c r="B63" s="6"/>
       <c r="C63" s="6"/>
@@ -13436,8 +14625,16 @@
       <c r="DF63" s="6"/>
       <c r="DG63" s="6"/>
       <c r="DH63" s="6"/>
+      <c r="DI63" s="6"/>
+      <c r="DJ63" s="6"/>
+      <c r="DK63" s="6"/>
+      <c r="DL63" s="6"/>
+      <c r="DM63" s="6"/>
+      <c r="DN63" s="6"/>
+      <c r="DO63" s="6"/>
+      <c r="DP63" s="6"/>
     </row>
-    <row r="64" spans="1:112" x14ac:dyDescent="0.3">
+    <row r="64" spans="1:120" x14ac:dyDescent="0.3">
       <c r="A64" s="6"/>
       <c r="B64" s="6"/>
       <c r="C64" s="6"/>
@@ -13550,8 +14747,16 @@
       <c r="DF64" s="6"/>
       <c r="DG64" s="6"/>
       <c r="DH64" s="6"/>
+      <c r="DI64" s="6"/>
+      <c r="DJ64" s="6"/>
+      <c r="DK64" s="6"/>
+      <c r="DL64" s="6"/>
+      <c r="DM64" s="6"/>
+      <c r="DN64" s="6"/>
+      <c r="DO64" s="6"/>
+      <c r="DP64" s="6"/>
     </row>
-    <row r="65" spans="1:112" x14ac:dyDescent="0.3">
+    <row r="65" spans="1:120" x14ac:dyDescent="0.3">
       <c r="A65" s="6"/>
       <c r="B65" s="6"/>
       <c r="C65" s="6"/>
@@ -13664,8 +14869,16 @@
       <c r="DF65" s="6"/>
       <c r="DG65" s="6"/>
       <c r="DH65" s="6"/>
+      <c r="DI65" s="6"/>
+      <c r="DJ65" s="6"/>
+      <c r="DK65" s="6"/>
+      <c r="DL65" s="6"/>
+      <c r="DM65" s="6"/>
+      <c r="DN65" s="6"/>
+      <c r="DO65" s="6"/>
+      <c r="DP65" s="6"/>
     </row>
-    <row r="66" spans="1:112" x14ac:dyDescent="0.3">
+    <row r="66" spans="1:120" x14ac:dyDescent="0.3">
       <c r="A66" s="6"/>
       <c r="B66" s="6"/>
       <c r="C66" s="6"/>
@@ -13778,8 +14991,16 @@
       <c r="DF66" s="6"/>
       <c r="DG66" s="6"/>
       <c r="DH66" s="6"/>
+      <c r="DI66" s="6"/>
+      <c r="DJ66" s="6"/>
+      <c r="DK66" s="6"/>
+      <c r="DL66" s="6"/>
+      <c r="DM66" s="6"/>
+      <c r="DN66" s="6"/>
+      <c r="DO66" s="6"/>
+      <c r="DP66" s="6"/>
     </row>
-    <row r="67" spans="1:112" x14ac:dyDescent="0.3">
+    <row r="67" spans="1:120" x14ac:dyDescent="0.3">
       <c r="A67" s="6"/>
       <c r="B67" s="6"/>
       <c r="C67" s="6"/>
@@ -13892,8 +15113,16 @@
       <c r="DF67" s="6"/>
       <c r="DG67" s="6"/>
       <c r="DH67" s="6"/>
+      <c r="DI67" s="6"/>
+      <c r="DJ67" s="6"/>
+      <c r="DK67" s="6"/>
+      <c r="DL67" s="6"/>
+      <c r="DM67" s="6"/>
+      <c r="DN67" s="6"/>
+      <c r="DO67" s="6"/>
+      <c r="DP67" s="6"/>
     </row>
-    <row r="68" spans="1:112" x14ac:dyDescent="0.3">
+    <row r="68" spans="1:120" x14ac:dyDescent="0.3">
       <c r="A68" s="6"/>
       <c r="B68" s="6"/>
       <c r="C68" s="6"/>
@@ -14006,8 +15235,16 @@
       <c r="DF68" s="6"/>
       <c r="DG68" s="6"/>
       <c r="DH68" s="6"/>
+      <c r="DI68" s="6"/>
+      <c r="DJ68" s="6"/>
+      <c r="DK68" s="6"/>
+      <c r="DL68" s="6"/>
+      <c r="DM68" s="6"/>
+      <c r="DN68" s="6"/>
+      <c r="DO68" s="6"/>
+      <c r="DP68" s="6"/>
     </row>
-    <row r="69" spans="1:112" x14ac:dyDescent="0.3">
+    <row r="69" spans="1:120" x14ac:dyDescent="0.3">
       <c r="A69" s="6"/>
       <c r="B69" s="6"/>
       <c r="C69" s="6"/>
@@ -14120,8 +15357,16 @@
       <c r="DF69" s="6"/>
       <c r="DG69" s="6"/>
       <c r="DH69" s="6"/>
+      <c r="DI69" s="6"/>
+      <c r="DJ69" s="6"/>
+      <c r="DK69" s="6"/>
+      <c r="DL69" s="6"/>
+      <c r="DM69" s="6"/>
+      <c r="DN69" s="6"/>
+      <c r="DO69" s="6"/>
+      <c r="DP69" s="6"/>
     </row>
-    <row r="70" spans="1:112" x14ac:dyDescent="0.3">
+    <row r="70" spans="1:120" x14ac:dyDescent="0.3">
       <c r="A70" s="6"/>
       <c r="B70" s="6"/>
       <c r="C70" s="6"/>
@@ -14234,8 +15479,16 @@
       <c r="DF70" s="6"/>
       <c r="DG70" s="6"/>
       <c r="DH70" s="6"/>
+      <c r="DI70" s="6"/>
+      <c r="DJ70" s="6"/>
+      <c r="DK70" s="6"/>
+      <c r="DL70" s="6"/>
+      <c r="DM70" s="6"/>
+      <c r="DN70" s="6"/>
+      <c r="DO70" s="6"/>
+      <c r="DP70" s="6"/>
     </row>
-    <row r="71" spans="1:112" ht="14.4" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="71" spans="1:120" ht="14.4" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A71" s="5" t="s">
         <v>11</v>
       </c>
@@ -14297,113 +15550,127 @@
       <c r="AM71" s="6"/>
       <c r="AN71" s="6"/>
       <c r="AO71" s="5" t="s">
-        <v>107</v>
+        <v>106</v>
       </c>
       <c r="AP71" s="6"/>
       <c r="AQ71" s="6"/>
       <c r="AR71" s="6"/>
       <c r="AS71" s="5" t="s">
-        <v>105</v>
+        <v>104</v>
       </c>
       <c r="AT71" s="6"/>
       <c r="AU71" s="6"/>
       <c r="AV71" s="6"/>
       <c r="AW71" s="5" t="s">
-        <v>126</v>
+        <v>125</v>
       </c>
       <c r="AX71" s="6"/>
       <c r="AY71" s="6"/>
       <c r="AZ71" s="6"/>
       <c r="BA71" s="5" t="s">
-        <v>123</v>
+        <v>122</v>
       </c>
       <c r="BB71" s="6"/>
       <c r="BC71" s="6"/>
       <c r="BD71" s="6"/>
       <c r="BE71" s="5" t="s">
-        <v>149</v>
+        <v>148</v>
       </c>
       <c r="BF71" s="6"/>
       <c r="BG71" s="6"/>
       <c r="BH71" s="6"/>
       <c r="BI71" s="5" t="s">
-        <v>146</v>
+        <v>145</v>
       </c>
       <c r="BJ71" s="6"/>
       <c r="BK71" s="6"/>
       <c r="BL71" s="6"/>
       <c r="BM71" s="5" t="s">
-        <v>169</v>
+        <v>168</v>
       </c>
       <c r="BN71" s="6"/>
       <c r="BO71" s="6"/>
       <c r="BP71" s="6"/>
       <c r="BQ71" s="5" t="s">
-        <v>167</v>
+        <v>166</v>
       </c>
       <c r="BR71" s="6"/>
       <c r="BS71" s="6"/>
       <c r="BT71" s="6"/>
       <c r="BU71" s="5" t="s">
-        <v>188</v>
+        <v>187</v>
       </c>
       <c r="BV71" s="6"/>
       <c r="BW71" s="6"/>
       <c r="BX71" s="6"/>
       <c r="BY71" s="5" t="s">
-        <v>197</v>
+        <v>196</v>
       </c>
       <c r="BZ71" s="6"/>
       <c r="CA71" s="6"/>
       <c r="CB71" s="6"/>
       <c r="CC71" s="5" t="s">
-        <v>209</v>
+        <v>208</v>
       </c>
       <c r="CD71" s="6"/>
       <c r="CE71" s="6"/>
       <c r="CF71" s="6"/>
       <c r="CG71" s="5" t="s">
-        <v>206</v>
+        <v>205</v>
       </c>
       <c r="CH71" s="6"/>
       <c r="CI71" s="6"/>
       <c r="CJ71" s="6"/>
       <c r="CK71" s="5" t="s">
-        <v>229</v>
+        <v>228</v>
       </c>
       <c r="CL71" s="6"/>
       <c r="CM71" s="6"/>
       <c r="CN71" s="6"/>
       <c r="CO71" s="5" t="s">
-        <v>227</v>
+        <v>226</v>
       </c>
       <c r="CP71" s="6"/>
       <c r="CQ71" s="6"/>
       <c r="CR71" s="6"/>
       <c r="CS71" s="5" t="s">
-        <v>250</v>
+        <v>249</v>
       </c>
       <c r="CT71" s="6"/>
       <c r="CU71" s="6"/>
       <c r="CV71" s="6"/>
       <c r="CW71" s="5" t="s">
-        <v>248</v>
+        <v>247</v>
       </c>
       <c r="CX71" s="6"/>
       <c r="CY71" s="6"/>
       <c r="CZ71" s="6"/>
-      <c r="DA71" s="5"/>
+      <c r="DA71" s="5" t="s">
+        <v>269</v>
+      </c>
       <c r="DB71" s="6"/>
       <c r="DC71" s="6"/>
       <c r="DD71" s="6"/>
       <c r="DE71" s="5" t="s">
-        <v>268</v>
+        <v>267</v>
       </c>
       <c r="DF71" s="6"/>
       <c r="DG71" s="6"/>
       <c r="DH71" s="6"/>
+      <c r="DI71" s="5" t="s">
+        <v>289</v>
+      </c>
+      <c r="DJ71" s="6"/>
+      <c r="DK71" s="6"/>
+      <c r="DL71" s="6"/>
+      <c r="DM71" s="5" t="s">
+        <v>290</v>
+      </c>
+      <c r="DN71" s="6"/>
+      <c r="DO71" s="6"/>
+      <c r="DP71" s="6"/>
     </row>
-    <row r="72" spans="1:112" x14ac:dyDescent="0.3">
+    <row r="72" spans="1:120" x14ac:dyDescent="0.3">
       <c r="A72" s="6"/>
       <c r="B72" s="6"/>
       <c r="C72" s="6"/>
@@ -14516,8 +15783,16 @@
       <c r="DF72" s="6"/>
       <c r="DG72" s="6"/>
       <c r="DH72" s="6"/>
+      <c r="DI72" s="6"/>
+      <c r="DJ72" s="6"/>
+      <c r="DK72" s="6"/>
+      <c r="DL72" s="6"/>
+      <c r="DM72" s="6"/>
+      <c r="DN72" s="6"/>
+      <c r="DO72" s="6"/>
+      <c r="DP72" s="6"/>
     </row>
-    <row r="73" spans="1:112" x14ac:dyDescent="0.3">
+    <row r="73" spans="1:120" x14ac:dyDescent="0.3">
       <c r="A73" s="6"/>
       <c r="B73" s="6"/>
       <c r="C73" s="6"/>
@@ -14630,8 +15905,16 @@
       <c r="DF73" s="6"/>
       <c r="DG73" s="6"/>
       <c r="DH73" s="6"/>
+      <c r="DI73" s="6"/>
+      <c r="DJ73" s="6"/>
+      <c r="DK73" s="6"/>
+      <c r="DL73" s="6"/>
+      <c r="DM73" s="6"/>
+      <c r="DN73" s="6"/>
+      <c r="DO73" s="6"/>
+      <c r="DP73" s="6"/>
     </row>
-    <row r="74" spans="1:112" x14ac:dyDescent="0.3">
+    <row r="74" spans="1:120" x14ac:dyDescent="0.3">
       <c r="A74" s="6"/>
       <c r="B74" s="6"/>
       <c r="C74" s="6"/>
@@ -14744,8 +16027,16 @@
       <c r="DF74" s="6"/>
       <c r="DG74" s="6"/>
       <c r="DH74" s="6"/>
+      <c r="DI74" s="6"/>
+      <c r="DJ74" s="6"/>
+      <c r="DK74" s="6"/>
+      <c r="DL74" s="6"/>
+      <c r="DM74" s="6"/>
+      <c r="DN74" s="6"/>
+      <c r="DO74" s="6"/>
+      <c r="DP74" s="6"/>
     </row>
-    <row r="75" spans="1:112" x14ac:dyDescent="0.3">
+    <row r="75" spans="1:120" x14ac:dyDescent="0.3">
       <c r="A75" s="6"/>
       <c r="B75" s="6"/>
       <c r="C75" s="6"/>
@@ -14858,8 +16149,16 @@
       <c r="DF75" s="6"/>
       <c r="DG75" s="6"/>
       <c r="DH75" s="6"/>
+      <c r="DI75" s="6"/>
+      <c r="DJ75" s="6"/>
+      <c r="DK75" s="6"/>
+      <c r="DL75" s="6"/>
+      <c r="DM75" s="6"/>
+      <c r="DN75" s="6"/>
+      <c r="DO75" s="6"/>
+      <c r="DP75" s="6"/>
     </row>
-    <row r="76" spans="1:112" x14ac:dyDescent="0.3">
+    <row r="76" spans="1:120" x14ac:dyDescent="0.3">
       <c r="A76" s="6"/>
       <c r="B76" s="6"/>
       <c r="C76" s="6"/>
@@ -14972,8 +16271,16 @@
       <c r="DF76" s="6"/>
       <c r="DG76" s="6"/>
       <c r="DH76" s="6"/>
+      <c r="DI76" s="6"/>
+      <c r="DJ76" s="6"/>
+      <c r="DK76" s="6"/>
+      <c r="DL76" s="6"/>
+      <c r="DM76" s="6"/>
+      <c r="DN76" s="6"/>
+      <c r="DO76" s="6"/>
+      <c r="DP76" s="6"/>
     </row>
-    <row r="77" spans="1:112" x14ac:dyDescent="0.3">
+    <row r="77" spans="1:120" x14ac:dyDescent="0.3">
       <c r="A77" s="6"/>
       <c r="B77" s="6"/>
       <c r="C77" s="6"/>
@@ -15086,8 +16393,16 @@
       <c r="DF77" s="6"/>
       <c r="DG77" s="6"/>
       <c r="DH77" s="6"/>
+      <c r="DI77" s="6"/>
+      <c r="DJ77" s="6"/>
+      <c r="DK77" s="6"/>
+      <c r="DL77" s="6"/>
+      <c r="DM77" s="6"/>
+      <c r="DN77" s="6"/>
+      <c r="DO77" s="6"/>
+      <c r="DP77" s="6"/>
     </row>
-    <row r="78" spans="1:112" x14ac:dyDescent="0.3">
+    <row r="78" spans="1:120" x14ac:dyDescent="0.3">
       <c r="A78" s="6"/>
       <c r="B78" s="6"/>
       <c r="C78" s="6"/>
@@ -15200,8 +16515,16 @@
       <c r="DF78" s="6"/>
       <c r="DG78" s="6"/>
       <c r="DH78" s="6"/>
+      <c r="DI78" s="6"/>
+      <c r="DJ78" s="6"/>
+      <c r="DK78" s="6"/>
+      <c r="DL78" s="6"/>
+      <c r="DM78" s="6"/>
+      <c r="DN78" s="6"/>
+      <c r="DO78" s="6"/>
+      <c r="DP78" s="6"/>
     </row>
-    <row r="79" spans="1:112" x14ac:dyDescent="0.3">
+    <row r="79" spans="1:120" x14ac:dyDescent="0.3">
       <c r="A79" s="6"/>
       <c r="B79" s="6"/>
       <c r="C79" s="6"/>
@@ -15314,8 +16637,16 @@
       <c r="DF79" s="6"/>
       <c r="DG79" s="6"/>
       <c r="DH79" s="6"/>
+      <c r="DI79" s="6"/>
+      <c r="DJ79" s="6"/>
+      <c r="DK79" s="6"/>
+      <c r="DL79" s="6"/>
+      <c r="DM79" s="6"/>
+      <c r="DN79" s="6"/>
+      <c r="DO79" s="6"/>
+      <c r="DP79" s="6"/>
     </row>
-    <row r="80" spans="1:112" x14ac:dyDescent="0.3">
+    <row r="80" spans="1:120" x14ac:dyDescent="0.3">
       <c r="A80" s="6"/>
       <c r="B80" s="6"/>
       <c r="C80" s="6"/>
@@ -15428,8 +16759,16 @@
       <c r="DF80" s="6"/>
       <c r="DG80" s="6"/>
       <c r="DH80" s="6"/>
+      <c r="DI80" s="6"/>
+      <c r="DJ80" s="6"/>
+      <c r="DK80" s="6"/>
+      <c r="DL80" s="6"/>
+      <c r="DM80" s="6"/>
+      <c r="DN80" s="6"/>
+      <c r="DO80" s="6"/>
+      <c r="DP80" s="6"/>
     </row>
-    <row r="81" spans="1:112" x14ac:dyDescent="0.3">
+    <row r="81" spans="1:120" x14ac:dyDescent="0.3">
       <c r="A81" s="5" t="s">
         <v>15</v>
       </c>
@@ -15491,111 +16830,123 @@
       <c r="AM81" s="6"/>
       <c r="AN81" s="6"/>
       <c r="AO81" s="5" t="s">
-        <v>111</v>
+        <v>110</v>
       </c>
       <c r="AP81" s="6"/>
       <c r="AQ81" s="6"/>
       <c r="AR81" s="6"/>
       <c r="AS81" s="5" t="s">
-        <v>109</v>
+        <v>108</v>
       </c>
       <c r="AT81" s="6"/>
       <c r="AU81" s="6"/>
       <c r="AV81" s="6"/>
       <c r="AW81" s="5" t="s">
-        <v>133</v>
+        <v>132</v>
       </c>
       <c r="AX81" s="6"/>
       <c r="AY81" s="6"/>
       <c r="AZ81" s="6"/>
       <c r="BA81" s="5" t="s">
-        <v>130</v>
+        <v>129</v>
       </c>
       <c r="BB81" s="6"/>
       <c r="BC81" s="6"/>
       <c r="BD81" s="6"/>
       <c r="BE81" s="5" t="s">
-        <v>152</v>
+        <v>151</v>
       </c>
       <c r="BF81" s="6"/>
       <c r="BG81" s="6"/>
       <c r="BH81" s="6"/>
       <c r="BI81" s="5" t="s">
-        <v>150</v>
+        <v>149</v>
       </c>
       <c r="BJ81" s="6"/>
       <c r="BK81" s="6"/>
       <c r="BL81" s="6"/>
       <c r="BM81" s="5" t="s">
-        <v>173</v>
+        <v>172</v>
       </c>
       <c r="BN81" s="6"/>
       <c r="BO81" s="6"/>
       <c r="BP81" s="6"/>
       <c r="BQ81" s="5" t="s">
-        <v>171</v>
+        <v>170</v>
       </c>
       <c r="BR81" s="6"/>
       <c r="BS81" s="6"/>
       <c r="BT81" s="6"/>
       <c r="BU81" s="5" t="s">
-        <v>191</v>
+        <v>190</v>
       </c>
       <c r="BV81" s="6"/>
       <c r="BW81" s="6"/>
       <c r="BX81" s="6"/>
       <c r="BY81" s="5" t="s">
-        <v>190</v>
+        <v>189</v>
       </c>
       <c r="BZ81" s="6"/>
       <c r="CA81" s="6"/>
       <c r="CB81" s="6"/>
       <c r="CC81" s="5" t="s">
-        <v>213</v>
+        <v>212</v>
       </c>
       <c r="CD81" s="6"/>
       <c r="CE81" s="6"/>
       <c r="CF81" s="6"/>
       <c r="CG81" s="5" t="s">
-        <v>211</v>
+        <v>210</v>
       </c>
       <c r="CH81" s="6"/>
       <c r="CI81" s="6"/>
       <c r="CJ81" s="6"/>
       <c r="CK81" s="5" t="s">
-        <v>234</v>
+        <v>233</v>
       </c>
       <c r="CL81" s="6"/>
       <c r="CM81" s="6"/>
       <c r="CN81" s="6"/>
       <c r="CO81" s="5" t="s">
-        <v>231</v>
+        <v>230</v>
       </c>
       <c r="CP81" s="6"/>
       <c r="CQ81" s="6"/>
       <c r="CR81" s="6"/>
       <c r="CS81" s="5" t="s">
-        <v>251</v>
+        <v>250</v>
       </c>
       <c r="CT81" s="6"/>
       <c r="CU81" s="6"/>
       <c r="CV81" s="6"/>
       <c r="CW81" s="5" t="s">
-        <v>254</v>
+        <v>253</v>
       </c>
       <c r="CX81" s="6"/>
       <c r="CY81" s="6"/>
       <c r="CZ81" s="6"/>
-      <c r="DA81" s="5"/>
+      <c r="DA81" s="5" t="s">
+        <v>274</v>
+      </c>
       <c r="DB81" s="6"/>
       <c r="DC81" s="6"/>
       <c r="DD81" s="6"/>
-      <c r="DE81" s="5"/>
+      <c r="DE81" s="5" t="s">
+        <v>270</v>
+      </c>
       <c r="DF81" s="6"/>
       <c r="DG81" s="6"/>
       <c r="DH81" s="6"/>
+      <c r="DI81" s="5"/>
+      <c r="DJ81" s="6"/>
+      <c r="DK81" s="6"/>
+      <c r="DL81" s="6"/>
+      <c r="DM81" s="5"/>
+      <c r="DN81" s="6"/>
+      <c r="DO81" s="6"/>
+      <c r="DP81" s="6"/>
     </row>
-    <row r="82" spans="1:112" x14ac:dyDescent="0.3">
+    <row r="82" spans="1:120" x14ac:dyDescent="0.3">
       <c r="A82" s="6"/>
       <c r="B82" s="6"/>
       <c r="C82" s="6"/>
@@ -15708,8 +17059,16 @@
       <c r="DF82" s="6"/>
       <c r="DG82" s="6"/>
       <c r="DH82" s="6"/>
+      <c r="DI82" s="6"/>
+      <c r="DJ82" s="6"/>
+      <c r="DK82" s="6"/>
+      <c r="DL82" s="6"/>
+      <c r="DM82" s="6"/>
+      <c r="DN82" s="6"/>
+      <c r="DO82" s="6"/>
+      <c r="DP82" s="6"/>
     </row>
-    <row r="83" spans="1:112" x14ac:dyDescent="0.3">
+    <row r="83" spans="1:120" x14ac:dyDescent="0.3">
       <c r="A83" s="6"/>
       <c r="B83" s="6"/>
       <c r="C83" s="6"/>
@@ -15822,8 +17181,16 @@
       <c r="DF83" s="6"/>
       <c r="DG83" s="6"/>
       <c r="DH83" s="6"/>
+      <c r="DI83" s="6"/>
+      <c r="DJ83" s="6"/>
+      <c r="DK83" s="6"/>
+      <c r="DL83" s="6"/>
+      <c r="DM83" s="6"/>
+      <c r="DN83" s="6"/>
+      <c r="DO83" s="6"/>
+      <c r="DP83" s="6"/>
     </row>
-    <row r="84" spans="1:112" x14ac:dyDescent="0.3">
+    <row r="84" spans="1:120" x14ac:dyDescent="0.3">
       <c r="A84" s="6"/>
       <c r="B84" s="6"/>
       <c r="C84" s="6"/>
@@ -15936,8 +17303,16 @@
       <c r="DF84" s="6"/>
       <c r="DG84" s="6"/>
       <c r="DH84" s="6"/>
+      <c r="DI84" s="6"/>
+      <c r="DJ84" s="6"/>
+      <c r="DK84" s="6"/>
+      <c r="DL84" s="6"/>
+      <c r="DM84" s="6"/>
+      <c r="DN84" s="6"/>
+      <c r="DO84" s="6"/>
+      <c r="DP84" s="6"/>
     </row>
-    <row r="85" spans="1:112" x14ac:dyDescent="0.3">
+    <row r="85" spans="1:120" x14ac:dyDescent="0.3">
       <c r="A85" s="6"/>
       <c r="B85" s="6"/>
       <c r="C85" s="6"/>
@@ -16050,8 +17425,16 @@
       <c r="DF85" s="6"/>
       <c r="DG85" s="6"/>
       <c r="DH85" s="6"/>
+      <c r="DI85" s="6"/>
+      <c r="DJ85" s="6"/>
+      <c r="DK85" s="6"/>
+      <c r="DL85" s="6"/>
+      <c r="DM85" s="6"/>
+      <c r="DN85" s="6"/>
+      <c r="DO85" s="6"/>
+      <c r="DP85" s="6"/>
     </row>
-    <row r="86" spans="1:112" x14ac:dyDescent="0.3">
+    <row r="86" spans="1:120" x14ac:dyDescent="0.3">
       <c r="A86" s="6"/>
       <c r="B86" s="6"/>
       <c r="C86" s="6"/>
@@ -16164,8 +17547,16 @@
       <c r="DF86" s="6"/>
       <c r="DG86" s="6"/>
       <c r="DH86" s="6"/>
+      <c r="DI86" s="6"/>
+      <c r="DJ86" s="6"/>
+      <c r="DK86" s="6"/>
+      <c r="DL86" s="6"/>
+      <c r="DM86" s="6"/>
+      <c r="DN86" s="6"/>
+      <c r="DO86" s="6"/>
+      <c r="DP86" s="6"/>
     </row>
-    <row r="87" spans="1:112" x14ac:dyDescent="0.3">
+    <row r="87" spans="1:120" x14ac:dyDescent="0.3">
       <c r="A87" s="6"/>
       <c r="B87" s="6"/>
       <c r="C87" s="6"/>
@@ -16278,8 +17669,16 @@
       <c r="DF87" s="6"/>
       <c r="DG87" s="6"/>
       <c r="DH87" s="6"/>
+      <c r="DI87" s="6"/>
+      <c r="DJ87" s="6"/>
+      <c r="DK87" s="6"/>
+      <c r="DL87" s="6"/>
+      <c r="DM87" s="6"/>
+      <c r="DN87" s="6"/>
+      <c r="DO87" s="6"/>
+      <c r="DP87" s="6"/>
     </row>
-    <row r="88" spans="1:112" x14ac:dyDescent="0.3">
+    <row r="88" spans="1:120" x14ac:dyDescent="0.3">
       <c r="A88" s="6"/>
       <c r="B88" s="6"/>
       <c r="C88" s="6"/>
@@ -16392,8 +17791,16 @@
       <c r="DF88" s="6"/>
       <c r="DG88" s="6"/>
       <c r="DH88" s="6"/>
+      <c r="DI88" s="6"/>
+      <c r="DJ88" s="6"/>
+      <c r="DK88" s="6"/>
+      <c r="DL88" s="6"/>
+      <c r="DM88" s="6"/>
+      <c r="DN88" s="6"/>
+      <c r="DO88" s="6"/>
+      <c r="DP88" s="6"/>
     </row>
-    <row r="89" spans="1:112" x14ac:dyDescent="0.3">
+    <row r="89" spans="1:120" x14ac:dyDescent="0.3">
       <c r="A89" s="6"/>
       <c r="B89" s="6"/>
       <c r="C89" s="6"/>
@@ -16506,8 +17913,16 @@
       <c r="DF89" s="6"/>
       <c r="DG89" s="6"/>
       <c r="DH89" s="6"/>
+      <c r="DI89" s="6"/>
+      <c r="DJ89" s="6"/>
+      <c r="DK89" s="6"/>
+      <c r="DL89" s="6"/>
+      <c r="DM89" s="6"/>
+      <c r="DN89" s="6"/>
+      <c r="DO89" s="6"/>
+      <c r="DP89" s="6"/>
     </row>
-    <row r="90" spans="1:112" x14ac:dyDescent="0.3">
+    <row r="90" spans="1:120" x14ac:dyDescent="0.3">
       <c r="A90" s="6"/>
       <c r="B90" s="6"/>
       <c r="C90" s="6"/>
@@ -16620,8 +18035,16 @@
       <c r="DF90" s="6"/>
       <c r="DG90" s="6"/>
       <c r="DH90" s="6"/>
+      <c r="DI90" s="6"/>
+      <c r="DJ90" s="6"/>
+      <c r="DK90" s="6"/>
+      <c r="DL90" s="6"/>
+      <c r="DM90" s="6"/>
+      <c r="DN90" s="6"/>
+      <c r="DO90" s="6"/>
+      <c r="DP90" s="6"/>
     </row>
-    <row r="91" spans="1:112" x14ac:dyDescent="0.3">
+    <row r="91" spans="1:120" x14ac:dyDescent="0.3">
       <c r="A91" s="5" t="s">
         <v>19</v>
       </c>
@@ -16683,111 +18106,123 @@
       <c r="AM91" s="6"/>
       <c r="AN91" s="6"/>
       <c r="AO91" s="5" t="s">
-        <v>115</v>
+        <v>114</v>
       </c>
       <c r="AP91" s="6"/>
       <c r="AQ91" s="6"/>
       <c r="AR91" s="6"/>
       <c r="AS91" s="5" t="s">
-        <v>113</v>
+        <v>112</v>
       </c>
       <c r="AT91" s="6"/>
       <c r="AU91" s="6"/>
       <c r="AV91" s="6"/>
       <c r="AW91" s="5" t="s">
-        <v>136</v>
+        <v>135</v>
       </c>
       <c r="AX91" s="6"/>
       <c r="AY91" s="6"/>
       <c r="AZ91" s="6"/>
       <c r="BA91" s="5" t="s">
-        <v>135</v>
+        <v>134</v>
       </c>
       <c r="BB91" s="6"/>
       <c r="BC91" s="6"/>
       <c r="BD91" s="6"/>
       <c r="BE91" s="5" t="s">
-        <v>157</v>
+        <v>156</v>
       </c>
       <c r="BF91" s="6"/>
       <c r="BG91" s="6"/>
       <c r="BH91" s="6"/>
       <c r="BI91" s="5" t="s">
-        <v>155</v>
+        <v>154</v>
       </c>
       <c r="BJ91" s="6"/>
       <c r="BK91" s="6"/>
       <c r="BL91" s="6"/>
       <c r="BM91" s="5" t="s">
-        <v>176</v>
+        <v>175</v>
       </c>
       <c r="BN91" s="6"/>
       <c r="BO91" s="6"/>
       <c r="BP91" s="6"/>
       <c r="BQ91" s="5" t="s">
-        <v>175</v>
+        <v>174</v>
       </c>
       <c r="BR91" s="6"/>
       <c r="BS91" s="6"/>
       <c r="BT91" s="6"/>
       <c r="BU91" s="5" t="s">
-        <v>196</v>
+        <v>195</v>
       </c>
       <c r="BV91" s="6"/>
       <c r="BW91" s="6"/>
       <c r="BX91" s="6"/>
       <c r="BY91" s="5" t="s">
-        <v>193</v>
+        <v>192</v>
       </c>
       <c r="BZ91" s="6"/>
       <c r="CA91" s="6"/>
       <c r="CB91" s="6"/>
       <c r="CC91" s="5" t="s">
-        <v>217</v>
+        <v>216</v>
       </c>
       <c r="CD91" s="6"/>
       <c r="CE91" s="6"/>
       <c r="CF91" s="6"/>
       <c r="CG91" s="5" t="s">
-        <v>214</v>
+        <v>213</v>
       </c>
       <c r="CH91" s="6"/>
       <c r="CI91" s="6"/>
       <c r="CJ91" s="6"/>
       <c r="CK91" s="5" t="s">
-        <v>238</v>
+        <v>237</v>
       </c>
       <c r="CL91" s="6"/>
       <c r="CM91" s="6"/>
       <c r="CN91" s="6"/>
       <c r="CO91" s="5" t="s">
-        <v>236</v>
+        <v>235</v>
       </c>
       <c r="CP91" s="6"/>
       <c r="CQ91" s="6"/>
       <c r="CR91" s="6"/>
       <c r="CS91" s="5" t="s">
-        <v>257</v>
+        <v>256</v>
       </c>
       <c r="CT91" s="6"/>
       <c r="CU91" s="6"/>
       <c r="CV91" s="6"/>
       <c r="CW91" s="5" t="s">
-        <v>258</v>
+        <v>257</v>
       </c>
       <c r="CX91" s="6"/>
       <c r="CY91" s="6"/>
       <c r="CZ91" s="6"/>
-      <c r="DA91" s="5"/>
+      <c r="DA91" s="5" t="s">
+        <v>277</v>
+      </c>
       <c r="DB91" s="6"/>
       <c r="DC91" s="6"/>
       <c r="DD91" s="6"/>
-      <c r="DE91" s="5"/>
+      <c r="DE91" s="5" t="s">
+        <v>276</v>
+      </c>
       <c r="DF91" s="6"/>
       <c r="DG91" s="6"/>
       <c r="DH91" s="6"/>
+      <c r="DI91" s="5"/>
+      <c r="DJ91" s="6"/>
+      <c r="DK91" s="6"/>
+      <c r="DL91" s="6"/>
+      <c r="DM91" s="5"/>
+      <c r="DN91" s="6"/>
+      <c r="DO91" s="6"/>
+      <c r="DP91" s="6"/>
     </row>
-    <row r="92" spans="1:112" x14ac:dyDescent="0.3">
+    <row r="92" spans="1:120" x14ac:dyDescent="0.3">
       <c r="A92" s="6"/>
       <c r="B92" s="6"/>
       <c r="C92" s="6"/>
@@ -16900,8 +18335,16 @@
       <c r="DF92" s="6"/>
       <c r="DG92" s="6"/>
       <c r="DH92" s="6"/>
+      <c r="DI92" s="6"/>
+      <c r="DJ92" s="6"/>
+      <c r="DK92" s="6"/>
+      <c r="DL92" s="6"/>
+      <c r="DM92" s="6"/>
+      <c r="DN92" s="6"/>
+      <c r="DO92" s="6"/>
+      <c r="DP92" s="6"/>
     </row>
-    <row r="93" spans="1:112" x14ac:dyDescent="0.3">
+    <row r="93" spans="1:120" x14ac:dyDescent="0.3">
       <c r="A93" s="6"/>
       <c r="B93" s="6"/>
       <c r="C93" s="6"/>
@@ -17014,8 +18457,16 @@
       <c r="DF93" s="6"/>
       <c r="DG93" s="6"/>
       <c r="DH93" s="6"/>
+      <c r="DI93" s="6"/>
+      <c r="DJ93" s="6"/>
+      <c r="DK93" s="6"/>
+      <c r="DL93" s="6"/>
+      <c r="DM93" s="6"/>
+      <c r="DN93" s="6"/>
+      <c r="DO93" s="6"/>
+      <c r="DP93" s="6"/>
     </row>
-    <row r="94" spans="1:112" x14ac:dyDescent="0.3">
+    <row r="94" spans="1:120" x14ac:dyDescent="0.3">
       <c r="A94" s="6"/>
       <c r="B94" s="6"/>
       <c r="C94" s="6"/>
@@ -17128,8 +18579,16 @@
       <c r="DF94" s="6"/>
       <c r="DG94" s="6"/>
       <c r="DH94" s="6"/>
+      <c r="DI94" s="6"/>
+      <c r="DJ94" s="6"/>
+      <c r="DK94" s="6"/>
+      <c r="DL94" s="6"/>
+      <c r="DM94" s="6"/>
+      <c r="DN94" s="6"/>
+      <c r="DO94" s="6"/>
+      <c r="DP94" s="6"/>
     </row>
-    <row r="95" spans="1:112" x14ac:dyDescent="0.3">
+    <row r="95" spans="1:120" x14ac:dyDescent="0.3">
       <c r="A95" s="6"/>
       <c r="B95" s="6"/>
       <c r="C95" s="6"/>
@@ -17242,8 +18701,16 @@
       <c r="DF95" s="6"/>
       <c r="DG95" s="6"/>
       <c r="DH95" s="6"/>
+      <c r="DI95" s="6"/>
+      <c r="DJ95" s="6"/>
+      <c r="DK95" s="6"/>
+      <c r="DL95" s="6"/>
+      <c r="DM95" s="6"/>
+      <c r="DN95" s="6"/>
+      <c r="DO95" s="6"/>
+      <c r="DP95" s="6"/>
     </row>
-    <row r="96" spans="1:112" x14ac:dyDescent="0.3">
+    <row r="96" spans="1:120" x14ac:dyDescent="0.3">
       <c r="A96" s="6"/>
       <c r="B96" s="6"/>
       <c r="C96" s="6"/>
@@ -17356,8 +18823,16 @@
       <c r="DF96" s="6"/>
       <c r="DG96" s="6"/>
       <c r="DH96" s="6"/>
+      <c r="DI96" s="6"/>
+      <c r="DJ96" s="6"/>
+      <c r="DK96" s="6"/>
+      <c r="DL96" s="6"/>
+      <c r="DM96" s="6"/>
+      <c r="DN96" s="6"/>
+      <c r="DO96" s="6"/>
+      <c r="DP96" s="6"/>
     </row>
-    <row r="97" spans="1:112" x14ac:dyDescent="0.3">
+    <row r="97" spans="1:120" x14ac:dyDescent="0.3">
       <c r="A97" s="6"/>
       <c r="B97" s="6"/>
       <c r="C97" s="6"/>
@@ -17470,8 +18945,16 @@
       <c r="DF97" s="6"/>
       <c r="DG97" s="6"/>
       <c r="DH97" s="6"/>
+      <c r="DI97" s="6"/>
+      <c r="DJ97" s="6"/>
+      <c r="DK97" s="6"/>
+      <c r="DL97" s="6"/>
+      <c r="DM97" s="6"/>
+      <c r="DN97" s="6"/>
+      <c r="DO97" s="6"/>
+      <c r="DP97" s="6"/>
     </row>
-    <row r="98" spans="1:112" x14ac:dyDescent="0.3">
+    <row r="98" spans="1:120" x14ac:dyDescent="0.3">
       <c r="A98" s="6"/>
       <c r="B98" s="6"/>
       <c r="C98" s="6"/>
@@ -17584,8 +19067,16 @@
       <c r="DF98" s="6"/>
       <c r="DG98" s="6"/>
       <c r="DH98" s="6"/>
+      <c r="DI98" s="6"/>
+      <c r="DJ98" s="6"/>
+      <c r="DK98" s="6"/>
+      <c r="DL98" s="6"/>
+      <c r="DM98" s="6"/>
+      <c r="DN98" s="6"/>
+      <c r="DO98" s="6"/>
+      <c r="DP98" s="6"/>
     </row>
-    <row r="99" spans="1:112" x14ac:dyDescent="0.3">
+    <row r="99" spans="1:120" x14ac:dyDescent="0.3">
       <c r="A99" s="6"/>
       <c r="B99" s="6"/>
       <c r="C99" s="6"/>
@@ -17698,8 +19189,16 @@
       <c r="DF99" s="6"/>
       <c r="DG99" s="6"/>
       <c r="DH99" s="6"/>
+      <c r="DI99" s="6"/>
+      <c r="DJ99" s="6"/>
+      <c r="DK99" s="6"/>
+      <c r="DL99" s="6"/>
+      <c r="DM99" s="6"/>
+      <c r="DN99" s="6"/>
+      <c r="DO99" s="6"/>
+      <c r="DP99" s="6"/>
     </row>
-    <row r="100" spans="1:112" x14ac:dyDescent="0.3">
+    <row r="100" spans="1:120" x14ac:dyDescent="0.3">
       <c r="A100" s="6"/>
       <c r="B100" s="6"/>
       <c r="C100" s="6"/>
@@ -17812,8 +19311,16 @@
       <c r="DF100" s="6"/>
       <c r="DG100" s="6"/>
       <c r="DH100" s="6"/>
+      <c r="DI100" s="6"/>
+      <c r="DJ100" s="6"/>
+      <c r="DK100" s="6"/>
+      <c r="DL100" s="6"/>
+      <c r="DM100" s="6"/>
+      <c r="DN100" s="6"/>
+      <c r="DO100" s="6"/>
+      <c r="DP100" s="6"/>
     </row>
-    <row r="101" spans="1:112" ht="14.4" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="101" spans="1:120" ht="14.4" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A101" s="1"/>
       <c r="B101" s="2"/>
       <c r="C101" s="2"/>
@@ -17827,7 +19334,7 @@
       <c r="K101" s="4"/>
       <c r="L101" s="4"/>
     </row>
-    <row r="102" spans="1:112" x14ac:dyDescent="0.3">
+    <row r="102" spans="1:120" x14ac:dyDescent="0.3">
       <c r="A102" s="2"/>
       <c r="B102" s="3"/>
       <c r="C102" s="4"/>
@@ -17841,7 +19348,7 @@
       <c r="K102" s="4"/>
       <c r="L102" s="4"/>
     </row>
-    <row r="103" spans="1:112" x14ac:dyDescent="0.3">
+    <row r="103" spans="1:120" x14ac:dyDescent="0.3">
       <c r="A103" s="2"/>
       <c r="B103" s="4"/>
       <c r="C103" s="4"/>
@@ -17855,7 +19362,7 @@
       <c r="K103" s="4"/>
       <c r="L103" s="4"/>
     </row>
-    <row r="104" spans="1:112" x14ac:dyDescent="0.3">
+    <row r="104" spans="1:120" x14ac:dyDescent="0.3">
       <c r="A104" s="2"/>
       <c r="B104" s="4"/>
       <c r="C104" s="4"/>
@@ -17869,7 +19376,7 @@
       <c r="K104" s="4"/>
       <c r="L104" s="4"/>
     </row>
-    <row r="105" spans="1:112" x14ac:dyDescent="0.3">
+    <row r="105" spans="1:120" x14ac:dyDescent="0.3">
       <c r="A105" s="2"/>
       <c r="B105" s="4"/>
       <c r="C105" s="4"/>
@@ -17883,7 +19390,7 @@
       <c r="K105" s="4"/>
       <c r="L105" s="4"/>
     </row>
-    <row r="106" spans="1:112" x14ac:dyDescent="0.3">
+    <row r="106" spans="1:120" x14ac:dyDescent="0.3">
       <c r="A106" s="2"/>
       <c r="B106" s="4"/>
       <c r="C106" s="4"/>
@@ -17897,7 +19404,7 @@
       <c r="K106" s="4"/>
       <c r="L106" s="4"/>
     </row>
-    <row r="107" spans="1:112" x14ac:dyDescent="0.3">
+    <row r="107" spans="1:120" x14ac:dyDescent="0.3">
       <c r="A107" s="2"/>
       <c r="B107" s="4"/>
       <c r="C107" s="4"/>
@@ -17911,7 +19418,7 @@
       <c r="K107" s="4"/>
       <c r="L107" s="4"/>
     </row>
-    <row r="108" spans="1:112" x14ac:dyDescent="0.3">
+    <row r="108" spans="1:120" x14ac:dyDescent="0.3">
       <c r="A108" s="2"/>
       <c r="B108" s="4"/>
       <c r="C108" s="4"/>
@@ -17925,7 +19432,7 @@
       <c r="K108" s="4"/>
       <c r="L108" s="4"/>
     </row>
-    <row r="109" spans="1:112" x14ac:dyDescent="0.3">
+    <row r="109" spans="1:120" x14ac:dyDescent="0.3">
       <c r="A109" s="2"/>
       <c r="B109" s="4"/>
       <c r="C109" s="4"/>
@@ -17939,7 +19446,7 @@
       <c r="K109" s="4"/>
       <c r="L109" s="4"/>
     </row>
-    <row r="110" spans="1:112" x14ac:dyDescent="0.3">
+    <row r="110" spans="1:120" x14ac:dyDescent="0.3">
       <c r="A110" s="2"/>
       <c r="B110" s="4"/>
       <c r="C110" s="4"/>
@@ -17953,7 +19460,7 @@
       <c r="K110" s="4"/>
       <c r="L110" s="4"/>
     </row>
-    <row r="111" spans="1:112" ht="14.4" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="111" spans="1:120" ht="14.4" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A111" s="1"/>
       <c r="B111" s="4"/>
       <c r="C111" s="4"/>
@@ -17967,7 +19474,7 @@
       <c r="K111" s="4"/>
       <c r="L111" s="4"/>
     </row>
-    <row r="112" spans="1:112" x14ac:dyDescent="0.3">
+    <row r="112" spans="1:120" x14ac:dyDescent="0.3">
       <c r="A112" s="2"/>
       <c r="B112" s="3"/>
       <c r="C112" s="4"/>
@@ -18520,107 +20027,183 @@
       <c r="E151" s="4"/>
     </row>
   </sheetData>
-  <mergeCells count="280">
-    <mergeCell ref="DA51:DD60"/>
-    <mergeCell ref="DE51:DH60"/>
-    <mergeCell ref="DA61:DD70"/>
-    <mergeCell ref="DE61:DH70"/>
-    <mergeCell ref="DA71:DD80"/>
-    <mergeCell ref="DE71:DH80"/>
-    <mergeCell ref="DA81:DD90"/>
-    <mergeCell ref="DE81:DH90"/>
-    <mergeCell ref="DA91:DD100"/>
-    <mergeCell ref="DE91:DH100"/>
-    <mergeCell ref="DA1:DD10"/>
-    <mergeCell ref="DE1:DH10"/>
-    <mergeCell ref="DA11:DD20"/>
-    <mergeCell ref="DE11:DH20"/>
-    <mergeCell ref="DA21:DD30"/>
-    <mergeCell ref="DE21:DH30"/>
-    <mergeCell ref="DA31:DD40"/>
-    <mergeCell ref="DE31:DH40"/>
-    <mergeCell ref="DA41:DD50"/>
-    <mergeCell ref="DE41:DH50"/>
-    <mergeCell ref="CS51:CV60"/>
-    <mergeCell ref="CW51:CZ60"/>
-    <mergeCell ref="CS61:CV70"/>
-    <mergeCell ref="CW61:CZ70"/>
-    <mergeCell ref="CS71:CV80"/>
-    <mergeCell ref="CW71:CZ80"/>
-    <mergeCell ref="CS81:CV90"/>
-    <mergeCell ref="CW81:CZ90"/>
-    <mergeCell ref="CS91:CV100"/>
-    <mergeCell ref="CW91:CZ100"/>
-    <mergeCell ref="CS1:CV10"/>
-    <mergeCell ref="CW1:CZ10"/>
-    <mergeCell ref="CS11:CV20"/>
-    <mergeCell ref="CW11:CZ20"/>
-    <mergeCell ref="CS21:CV30"/>
-    <mergeCell ref="CW21:CZ30"/>
-    <mergeCell ref="CS31:CV40"/>
-    <mergeCell ref="CW31:CZ40"/>
-    <mergeCell ref="CS41:CV50"/>
-    <mergeCell ref="CW41:CZ50"/>
-    <mergeCell ref="BU51:BX60"/>
-    <mergeCell ref="BY51:CB60"/>
-    <mergeCell ref="BU61:BX70"/>
-    <mergeCell ref="BY61:CB70"/>
-    <mergeCell ref="BU71:BX80"/>
-    <mergeCell ref="BY71:CB80"/>
-    <mergeCell ref="BU81:BX90"/>
-    <mergeCell ref="BY81:CB90"/>
-    <mergeCell ref="BU91:BX100"/>
-    <mergeCell ref="BY91:CB100"/>
-    <mergeCell ref="BU1:BX10"/>
-    <mergeCell ref="BY1:CB10"/>
-    <mergeCell ref="BU11:BX20"/>
-    <mergeCell ref="BY11:CB20"/>
-    <mergeCell ref="BU21:BX30"/>
-    <mergeCell ref="BY21:CB30"/>
-    <mergeCell ref="BU31:BX40"/>
-    <mergeCell ref="BY31:CB40"/>
-    <mergeCell ref="BU41:BX50"/>
-    <mergeCell ref="BY41:CB50"/>
-    <mergeCell ref="BM51:BP60"/>
-    <mergeCell ref="BQ51:BT60"/>
-    <mergeCell ref="BM61:BP70"/>
-    <mergeCell ref="BQ61:BT70"/>
-    <mergeCell ref="BM71:BP80"/>
-    <mergeCell ref="BQ71:BT80"/>
-    <mergeCell ref="BM81:BP90"/>
-    <mergeCell ref="BQ81:BT90"/>
-    <mergeCell ref="BM91:BP100"/>
-    <mergeCell ref="BQ91:BT100"/>
-    <mergeCell ref="BM1:BP10"/>
-    <mergeCell ref="BQ1:BT10"/>
-    <mergeCell ref="BM11:BP20"/>
-    <mergeCell ref="BQ11:BT20"/>
-    <mergeCell ref="BM21:BP30"/>
-    <mergeCell ref="BQ21:BT30"/>
-    <mergeCell ref="BM31:BP40"/>
-    <mergeCell ref="BQ31:BT40"/>
-    <mergeCell ref="BM41:BP50"/>
-    <mergeCell ref="BQ41:BT50"/>
-    <mergeCell ref="BE51:BH60"/>
-    <mergeCell ref="BI51:BL60"/>
-    <mergeCell ref="BE61:BH70"/>
-    <mergeCell ref="BI61:BL70"/>
-    <mergeCell ref="BE71:BH80"/>
-    <mergeCell ref="BI71:BL80"/>
-    <mergeCell ref="BE81:BH90"/>
-    <mergeCell ref="BI81:BL90"/>
-    <mergeCell ref="BE91:BH100"/>
-    <mergeCell ref="BI91:BL100"/>
-    <mergeCell ref="BE1:BH10"/>
-    <mergeCell ref="BI1:BL10"/>
-    <mergeCell ref="BE11:BH20"/>
-    <mergeCell ref="BI11:BL20"/>
-    <mergeCell ref="BE21:BH30"/>
-    <mergeCell ref="BI21:BL30"/>
-    <mergeCell ref="BE31:BH40"/>
-    <mergeCell ref="BI31:BL40"/>
-    <mergeCell ref="BE41:BH50"/>
-    <mergeCell ref="BI41:BL50"/>
+  <mergeCells count="300">
+    <mergeCell ref="DI51:DL60"/>
+    <mergeCell ref="DM51:DP60"/>
+    <mergeCell ref="DI61:DL70"/>
+    <mergeCell ref="DM61:DP70"/>
+    <mergeCell ref="DI71:DL80"/>
+    <mergeCell ref="DM71:DP80"/>
+    <mergeCell ref="DI81:DL90"/>
+    <mergeCell ref="DM81:DP90"/>
+    <mergeCell ref="DI91:DL100"/>
+    <mergeCell ref="DM91:DP100"/>
+    <mergeCell ref="DI1:DL10"/>
+    <mergeCell ref="DM1:DP10"/>
+    <mergeCell ref="DI11:DL20"/>
+    <mergeCell ref="DM11:DP20"/>
+    <mergeCell ref="DI21:DL30"/>
+    <mergeCell ref="DM21:DP30"/>
+    <mergeCell ref="DI31:DL40"/>
+    <mergeCell ref="DM31:DP40"/>
+    <mergeCell ref="DI41:DL50"/>
+    <mergeCell ref="DM41:DP50"/>
+    <mergeCell ref="CK51:CN60"/>
+    <mergeCell ref="CO51:CR60"/>
+    <mergeCell ref="CK61:CN70"/>
+    <mergeCell ref="CO61:CR70"/>
+    <mergeCell ref="CK71:CN80"/>
+    <mergeCell ref="CO71:CR80"/>
+    <mergeCell ref="CK81:CN90"/>
+    <mergeCell ref="CO81:CR90"/>
+    <mergeCell ref="CK91:CN100"/>
+    <mergeCell ref="CO91:CR100"/>
+    <mergeCell ref="CK1:CN10"/>
+    <mergeCell ref="CO1:CR10"/>
+    <mergeCell ref="CK11:CN20"/>
+    <mergeCell ref="CO11:CR20"/>
+    <mergeCell ref="CK21:CN30"/>
+    <mergeCell ref="CO21:CR30"/>
+    <mergeCell ref="CK31:CN40"/>
+    <mergeCell ref="CO31:CR40"/>
+    <mergeCell ref="CK41:CN50"/>
+    <mergeCell ref="CO41:CR50"/>
+    <mergeCell ref="CC51:CF60"/>
+    <mergeCell ref="CG51:CJ60"/>
+    <mergeCell ref="CC61:CF70"/>
+    <mergeCell ref="CG61:CJ70"/>
+    <mergeCell ref="CC71:CF80"/>
+    <mergeCell ref="CG71:CJ80"/>
+    <mergeCell ref="CC81:CF90"/>
+    <mergeCell ref="CG81:CJ90"/>
+    <mergeCell ref="CC91:CF100"/>
+    <mergeCell ref="CG91:CJ100"/>
+    <mergeCell ref="CC1:CF10"/>
+    <mergeCell ref="CG1:CJ10"/>
+    <mergeCell ref="CC11:CF20"/>
+    <mergeCell ref="CG11:CJ20"/>
+    <mergeCell ref="CC21:CF30"/>
+    <mergeCell ref="CG21:CJ30"/>
+    <mergeCell ref="CC31:CF40"/>
+    <mergeCell ref="CG31:CJ40"/>
+    <mergeCell ref="CC41:CF50"/>
+    <mergeCell ref="CG41:CJ50"/>
+    <mergeCell ref="AS91:AV100"/>
+    <mergeCell ref="AS61:AV70"/>
+    <mergeCell ref="AO71:AR80"/>
+    <mergeCell ref="AS71:AV80"/>
+    <mergeCell ref="AO81:AR90"/>
+    <mergeCell ref="AS81:AV90"/>
+    <mergeCell ref="AO31:AR40"/>
+    <mergeCell ref="AS31:AV40"/>
+    <mergeCell ref="AO41:AR50"/>
+    <mergeCell ref="AS41:AV50"/>
+    <mergeCell ref="AO51:AR60"/>
+    <mergeCell ref="AS51:AV60"/>
+    <mergeCell ref="AO1:AR10"/>
+    <mergeCell ref="AS1:AV10"/>
+    <mergeCell ref="AO11:AR20"/>
+    <mergeCell ref="AS11:AV20"/>
+    <mergeCell ref="AO21:AR30"/>
+    <mergeCell ref="AS21:AV30"/>
+    <mergeCell ref="AG81:AJ90"/>
+    <mergeCell ref="AK81:AN90"/>
+    <mergeCell ref="AG91:AJ100"/>
+    <mergeCell ref="AK91:AN100"/>
+    <mergeCell ref="AO91:AR100"/>
+    <mergeCell ref="AG51:AJ60"/>
+    <mergeCell ref="AK51:AN60"/>
+    <mergeCell ref="AG61:AJ70"/>
+    <mergeCell ref="AK61:AN70"/>
+    <mergeCell ref="AO61:AR70"/>
+    <mergeCell ref="AG1:AJ10"/>
+    <mergeCell ref="AK1:AN10"/>
+    <mergeCell ref="AG11:AJ20"/>
+    <mergeCell ref="AK11:AN20"/>
+    <mergeCell ref="AG21:AJ30"/>
+    <mergeCell ref="AK21:AN30"/>
+    <mergeCell ref="AG31:AJ40"/>
+    <mergeCell ref="AK31:AN40"/>
+    <mergeCell ref="AG41:AJ50"/>
+    <mergeCell ref="AK41:AN50"/>
+    <mergeCell ref="AG71:AJ80"/>
+    <mergeCell ref="AK71:AN80"/>
+    <mergeCell ref="A1:D10"/>
+    <mergeCell ref="E1:H10"/>
+    <mergeCell ref="A11:D20"/>
+    <mergeCell ref="E11:H20"/>
+    <mergeCell ref="A21:D30"/>
+    <mergeCell ref="E21:H30"/>
+    <mergeCell ref="M31:P40"/>
+    <mergeCell ref="I41:L50"/>
+    <mergeCell ref="M41:P50"/>
+    <mergeCell ref="A31:D40"/>
+    <mergeCell ref="E31:H40"/>
+    <mergeCell ref="A41:D50"/>
+    <mergeCell ref="E41:H50"/>
+    <mergeCell ref="I31:L40"/>
+    <mergeCell ref="I1:L10"/>
+    <mergeCell ref="M1:P10"/>
+    <mergeCell ref="I11:L20"/>
+    <mergeCell ref="M11:P20"/>
+    <mergeCell ref="I21:L30"/>
+    <mergeCell ref="M21:P30"/>
+    <mergeCell ref="A81:D90"/>
+    <mergeCell ref="E81:H90"/>
+    <mergeCell ref="A91:D100"/>
+    <mergeCell ref="E91:H100"/>
+    <mergeCell ref="A51:D60"/>
+    <mergeCell ref="E51:H60"/>
+    <mergeCell ref="A61:D70"/>
+    <mergeCell ref="E61:H70"/>
+    <mergeCell ref="A71:D80"/>
+    <mergeCell ref="E71:H80"/>
+    <mergeCell ref="I81:L90"/>
+    <mergeCell ref="M81:P90"/>
+    <mergeCell ref="I91:L100"/>
+    <mergeCell ref="M91:P100"/>
+    <mergeCell ref="I51:L60"/>
+    <mergeCell ref="M51:P60"/>
+    <mergeCell ref="I61:L70"/>
+    <mergeCell ref="M61:P70"/>
+    <mergeCell ref="I71:L80"/>
+    <mergeCell ref="M71:P80"/>
+    <mergeCell ref="Q1:T10"/>
+    <mergeCell ref="U1:X10"/>
+    <mergeCell ref="Y1:AB10"/>
+    <mergeCell ref="AC1:AF10"/>
+    <mergeCell ref="Q11:T20"/>
+    <mergeCell ref="U11:X20"/>
+    <mergeCell ref="Y11:AB20"/>
+    <mergeCell ref="AC11:AF20"/>
+    <mergeCell ref="Q21:T30"/>
+    <mergeCell ref="U21:X30"/>
+    <mergeCell ref="Y21:AB30"/>
+    <mergeCell ref="AC21:AF30"/>
+    <mergeCell ref="Q31:T40"/>
+    <mergeCell ref="U31:X40"/>
+    <mergeCell ref="Y31:AB40"/>
+    <mergeCell ref="AC31:AF40"/>
+    <mergeCell ref="Q41:T50"/>
+    <mergeCell ref="U41:X50"/>
+    <mergeCell ref="Y41:AB50"/>
+    <mergeCell ref="AC41:AF50"/>
+    <mergeCell ref="Q51:T60"/>
+    <mergeCell ref="U51:X60"/>
+    <mergeCell ref="Y51:AB60"/>
+    <mergeCell ref="AC51:AF60"/>
+    <mergeCell ref="Q61:T70"/>
+    <mergeCell ref="U61:X70"/>
+    <mergeCell ref="Y61:AB70"/>
+    <mergeCell ref="AC61:AF70"/>
+    <mergeCell ref="Q71:T80"/>
+    <mergeCell ref="U71:X80"/>
+    <mergeCell ref="Y71:AB80"/>
+    <mergeCell ref="AC71:AF80"/>
+    <mergeCell ref="Q81:T90"/>
+    <mergeCell ref="U81:X90"/>
+    <mergeCell ref="Y81:AB90"/>
+    <mergeCell ref="AC81:AF90"/>
     <mergeCell ref="Q91:T100"/>
     <mergeCell ref="U91:X100"/>
     <mergeCell ref="Y91:AB100"/>
@@ -18645,162 +20228,106 @@
     <mergeCell ref="BA81:BD90"/>
     <mergeCell ref="AW91:AZ100"/>
     <mergeCell ref="BA91:BD100"/>
-    <mergeCell ref="Q61:T70"/>
-    <mergeCell ref="U61:X70"/>
-    <mergeCell ref="Y61:AB70"/>
-    <mergeCell ref="AC61:AF70"/>
-    <mergeCell ref="Q71:T80"/>
-    <mergeCell ref="U71:X80"/>
-    <mergeCell ref="Y71:AB80"/>
-    <mergeCell ref="AC71:AF80"/>
-    <mergeCell ref="Q81:T90"/>
-    <mergeCell ref="U81:X90"/>
-    <mergeCell ref="Y81:AB90"/>
-    <mergeCell ref="AC81:AF90"/>
-    <mergeCell ref="Q31:T40"/>
-    <mergeCell ref="U31:X40"/>
-    <mergeCell ref="Y31:AB40"/>
-    <mergeCell ref="AC31:AF40"/>
-    <mergeCell ref="Q41:T50"/>
-    <mergeCell ref="U41:X50"/>
-    <mergeCell ref="Y41:AB50"/>
-    <mergeCell ref="AC41:AF50"/>
-    <mergeCell ref="Q51:T60"/>
-    <mergeCell ref="U51:X60"/>
-    <mergeCell ref="Y51:AB60"/>
-    <mergeCell ref="AC51:AF60"/>
-    <mergeCell ref="Q1:T10"/>
-    <mergeCell ref="U1:X10"/>
-    <mergeCell ref="Y1:AB10"/>
-    <mergeCell ref="AC1:AF10"/>
-    <mergeCell ref="Q11:T20"/>
-    <mergeCell ref="U11:X20"/>
-    <mergeCell ref="Y11:AB20"/>
-    <mergeCell ref="AC11:AF20"/>
-    <mergeCell ref="Q21:T30"/>
-    <mergeCell ref="U21:X30"/>
-    <mergeCell ref="Y21:AB30"/>
-    <mergeCell ref="AC21:AF30"/>
-    <mergeCell ref="I81:L90"/>
-    <mergeCell ref="M81:P90"/>
-    <mergeCell ref="I91:L100"/>
-    <mergeCell ref="M91:P100"/>
-    <mergeCell ref="I51:L60"/>
-    <mergeCell ref="M51:P60"/>
-    <mergeCell ref="I61:L70"/>
-    <mergeCell ref="M61:P70"/>
-    <mergeCell ref="I71:L80"/>
-    <mergeCell ref="M71:P80"/>
-    <mergeCell ref="A81:D90"/>
-    <mergeCell ref="E81:H90"/>
-    <mergeCell ref="A91:D100"/>
-    <mergeCell ref="E91:H100"/>
-    <mergeCell ref="A51:D60"/>
-    <mergeCell ref="E51:H60"/>
-    <mergeCell ref="A61:D70"/>
-    <mergeCell ref="E61:H70"/>
-    <mergeCell ref="A71:D80"/>
-    <mergeCell ref="E71:H80"/>
-    <mergeCell ref="AG41:AJ50"/>
-    <mergeCell ref="AK41:AN50"/>
-    <mergeCell ref="AG71:AJ80"/>
-    <mergeCell ref="AK71:AN80"/>
-    <mergeCell ref="A1:D10"/>
-    <mergeCell ref="E1:H10"/>
-    <mergeCell ref="A11:D20"/>
-    <mergeCell ref="E11:H20"/>
-    <mergeCell ref="A21:D30"/>
-    <mergeCell ref="E21:H30"/>
-    <mergeCell ref="M31:P40"/>
-    <mergeCell ref="I41:L50"/>
-    <mergeCell ref="M41:P50"/>
-    <mergeCell ref="A31:D40"/>
-    <mergeCell ref="E31:H40"/>
-    <mergeCell ref="A41:D50"/>
-    <mergeCell ref="E41:H50"/>
-    <mergeCell ref="I31:L40"/>
-    <mergeCell ref="I1:L10"/>
-    <mergeCell ref="M1:P10"/>
-    <mergeCell ref="I11:L20"/>
-    <mergeCell ref="M11:P20"/>
-    <mergeCell ref="I21:L30"/>
-    <mergeCell ref="M21:P30"/>
-    <mergeCell ref="AO1:AR10"/>
-    <mergeCell ref="AS1:AV10"/>
-    <mergeCell ref="AO11:AR20"/>
-    <mergeCell ref="AS11:AV20"/>
-    <mergeCell ref="AO21:AR30"/>
-    <mergeCell ref="AS21:AV30"/>
-    <mergeCell ref="AG81:AJ90"/>
-    <mergeCell ref="AK81:AN90"/>
-    <mergeCell ref="AG91:AJ100"/>
-    <mergeCell ref="AK91:AN100"/>
-    <mergeCell ref="AO91:AR100"/>
-    <mergeCell ref="AG51:AJ60"/>
-    <mergeCell ref="AK51:AN60"/>
-    <mergeCell ref="AG61:AJ70"/>
-    <mergeCell ref="AK61:AN70"/>
-    <mergeCell ref="AO61:AR70"/>
-    <mergeCell ref="AG1:AJ10"/>
-    <mergeCell ref="AK1:AN10"/>
-    <mergeCell ref="AG11:AJ20"/>
-    <mergeCell ref="AK11:AN20"/>
-    <mergeCell ref="AG21:AJ30"/>
-    <mergeCell ref="AK21:AN30"/>
-    <mergeCell ref="AG31:AJ40"/>
-    <mergeCell ref="AK31:AN40"/>
-    <mergeCell ref="AS91:AV100"/>
-    <mergeCell ref="AS61:AV70"/>
-    <mergeCell ref="AO71:AR80"/>
-    <mergeCell ref="AS71:AV80"/>
-    <mergeCell ref="AO81:AR90"/>
-    <mergeCell ref="AS81:AV90"/>
-    <mergeCell ref="AO31:AR40"/>
-    <mergeCell ref="AS31:AV40"/>
-    <mergeCell ref="AO41:AR50"/>
-    <mergeCell ref="AS41:AV50"/>
-    <mergeCell ref="AO51:AR60"/>
-    <mergeCell ref="AS51:AV60"/>
-    <mergeCell ref="CC1:CF10"/>
-    <mergeCell ref="CG1:CJ10"/>
-    <mergeCell ref="CC11:CF20"/>
-    <mergeCell ref="CG11:CJ20"/>
-    <mergeCell ref="CC21:CF30"/>
-    <mergeCell ref="CG21:CJ30"/>
-    <mergeCell ref="CC31:CF40"/>
-    <mergeCell ref="CG31:CJ40"/>
-    <mergeCell ref="CC41:CF50"/>
-    <mergeCell ref="CG41:CJ50"/>
-    <mergeCell ref="CC51:CF60"/>
-    <mergeCell ref="CG51:CJ60"/>
-    <mergeCell ref="CC61:CF70"/>
-    <mergeCell ref="CG61:CJ70"/>
-    <mergeCell ref="CC71:CF80"/>
-    <mergeCell ref="CG71:CJ80"/>
-    <mergeCell ref="CC81:CF90"/>
-    <mergeCell ref="CG81:CJ90"/>
-    <mergeCell ref="CC91:CF100"/>
-    <mergeCell ref="CG91:CJ100"/>
-    <mergeCell ref="CK1:CN10"/>
-    <mergeCell ref="CO1:CR10"/>
-    <mergeCell ref="CK11:CN20"/>
-    <mergeCell ref="CO11:CR20"/>
-    <mergeCell ref="CK21:CN30"/>
-    <mergeCell ref="CO21:CR30"/>
-    <mergeCell ref="CK31:CN40"/>
-    <mergeCell ref="CO31:CR40"/>
-    <mergeCell ref="CK41:CN50"/>
-    <mergeCell ref="CO41:CR50"/>
-    <mergeCell ref="CK51:CN60"/>
-    <mergeCell ref="CO51:CR60"/>
-    <mergeCell ref="CK61:CN70"/>
-    <mergeCell ref="CO61:CR70"/>
-    <mergeCell ref="CK71:CN80"/>
-    <mergeCell ref="CO71:CR80"/>
-    <mergeCell ref="CK81:CN90"/>
-    <mergeCell ref="CO81:CR90"/>
-    <mergeCell ref="CK91:CN100"/>
-    <mergeCell ref="CO91:CR100"/>
+    <mergeCell ref="BE1:BH10"/>
+    <mergeCell ref="BI1:BL10"/>
+    <mergeCell ref="BE11:BH20"/>
+    <mergeCell ref="BI11:BL20"/>
+    <mergeCell ref="BE21:BH30"/>
+    <mergeCell ref="BI21:BL30"/>
+    <mergeCell ref="BE31:BH40"/>
+    <mergeCell ref="BI31:BL40"/>
+    <mergeCell ref="BE41:BH50"/>
+    <mergeCell ref="BI41:BL50"/>
+    <mergeCell ref="BE51:BH60"/>
+    <mergeCell ref="BI51:BL60"/>
+    <mergeCell ref="BE61:BH70"/>
+    <mergeCell ref="BI61:BL70"/>
+    <mergeCell ref="BE71:BH80"/>
+    <mergeCell ref="BI71:BL80"/>
+    <mergeCell ref="BE81:BH90"/>
+    <mergeCell ref="BI81:BL90"/>
+    <mergeCell ref="BE91:BH100"/>
+    <mergeCell ref="BI91:BL100"/>
+    <mergeCell ref="BM1:BP10"/>
+    <mergeCell ref="BQ1:BT10"/>
+    <mergeCell ref="BM11:BP20"/>
+    <mergeCell ref="BQ11:BT20"/>
+    <mergeCell ref="BM21:BP30"/>
+    <mergeCell ref="BQ21:BT30"/>
+    <mergeCell ref="BM31:BP40"/>
+    <mergeCell ref="BQ31:BT40"/>
+    <mergeCell ref="BM41:BP50"/>
+    <mergeCell ref="BQ41:BT50"/>
+    <mergeCell ref="BM51:BP60"/>
+    <mergeCell ref="BQ51:BT60"/>
+    <mergeCell ref="BM61:BP70"/>
+    <mergeCell ref="BQ61:BT70"/>
+    <mergeCell ref="BM71:BP80"/>
+    <mergeCell ref="BQ71:BT80"/>
+    <mergeCell ref="BM81:BP90"/>
+    <mergeCell ref="BQ81:BT90"/>
+    <mergeCell ref="BM91:BP100"/>
+    <mergeCell ref="BQ91:BT100"/>
+    <mergeCell ref="BU1:BX10"/>
+    <mergeCell ref="BY1:CB10"/>
+    <mergeCell ref="BU11:BX20"/>
+    <mergeCell ref="BY11:CB20"/>
+    <mergeCell ref="BU21:BX30"/>
+    <mergeCell ref="BY21:CB30"/>
+    <mergeCell ref="BU31:BX40"/>
+    <mergeCell ref="BY31:CB40"/>
+    <mergeCell ref="BU41:BX50"/>
+    <mergeCell ref="BY41:CB50"/>
+    <mergeCell ref="BU51:BX60"/>
+    <mergeCell ref="BY51:CB60"/>
+    <mergeCell ref="BU61:BX70"/>
+    <mergeCell ref="BY61:CB70"/>
+    <mergeCell ref="BU71:BX80"/>
+    <mergeCell ref="BY71:CB80"/>
+    <mergeCell ref="BU81:BX90"/>
+    <mergeCell ref="BY81:CB90"/>
+    <mergeCell ref="BU91:BX100"/>
+    <mergeCell ref="BY91:CB100"/>
+    <mergeCell ref="CS1:CV10"/>
+    <mergeCell ref="CW1:CZ10"/>
+    <mergeCell ref="CS11:CV20"/>
+    <mergeCell ref="CW11:CZ20"/>
+    <mergeCell ref="CS21:CV30"/>
+    <mergeCell ref="CW21:CZ30"/>
+    <mergeCell ref="CS31:CV40"/>
+    <mergeCell ref="CW31:CZ40"/>
+    <mergeCell ref="CS41:CV50"/>
+    <mergeCell ref="CW41:CZ50"/>
+    <mergeCell ref="CS51:CV60"/>
+    <mergeCell ref="CW51:CZ60"/>
+    <mergeCell ref="CS61:CV70"/>
+    <mergeCell ref="CW61:CZ70"/>
+    <mergeCell ref="CS71:CV80"/>
+    <mergeCell ref="CW71:CZ80"/>
+    <mergeCell ref="CS81:CV90"/>
+    <mergeCell ref="CW81:CZ90"/>
+    <mergeCell ref="CS91:CV100"/>
+    <mergeCell ref="CW91:CZ100"/>
+    <mergeCell ref="DA1:DD10"/>
+    <mergeCell ref="DE1:DH10"/>
+    <mergeCell ref="DA11:DD20"/>
+    <mergeCell ref="DE11:DH20"/>
+    <mergeCell ref="DA21:DD30"/>
+    <mergeCell ref="DE21:DH30"/>
+    <mergeCell ref="DA31:DD40"/>
+    <mergeCell ref="DE31:DH40"/>
+    <mergeCell ref="DA41:DD50"/>
+    <mergeCell ref="DE41:DH50"/>
+    <mergeCell ref="DA51:DD60"/>
+    <mergeCell ref="DE51:DH60"/>
+    <mergeCell ref="DA61:DD70"/>
+    <mergeCell ref="DE61:DH70"/>
+    <mergeCell ref="DA71:DD80"/>
+    <mergeCell ref="DE71:DH80"/>
+    <mergeCell ref="DA81:DD90"/>
+    <mergeCell ref="DE81:DH90"/>
+    <mergeCell ref="DA91:DD100"/>
+    <mergeCell ref="DE91:DH100"/>
   </mergeCells>
   <printOptions horizontalCentered="1" verticalCentered="1"/>
   <pageMargins left="0.6692913385826772" right="0.6692913385826772" top="0.74803149606299213" bottom="0.74803149606299213" header="0.31496062992125984" footer="0.31496062992125984"/>

</xml_diff>

<commit_message>
Print was messed up, repaired
</commit_message>
<xml_diff>
--- a/tanulókártyák/Tanulókártyák.xlsx
+++ b/tanulókártyák/Tanulókártyák.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\atesz\OneDrive\Desktop\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{C8FC1C67-2A45-4257-AA32-C39BD9A3BB22}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{851F31B6-9251-447D-82FC-1E667113CFC4}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12576" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -25,7 +25,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="341" uniqueCount="340">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="340" uniqueCount="339">
   <si>
     <r>
       <rPr>
@@ -6131,9 +6131,6 @@
       </rPr>
       <t xml:space="preserve"> - Megmutatja, mennyi extra memória kell az algoritmusnak.</t>
     </r>
-  </si>
-  <si>
-    <t xml:space="preserve">spring annotiációk </t>
   </si>
   <si>
     <r>
@@ -7412,10 +7409,10 @@
     <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="top" wrapText="1" shrinkToFit="1"/>
     </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="1" xfId="0" quotePrefix="1" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="top" wrapText="1" shrinkToFit="1"/>
     </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="1" xfId="0" quotePrefix="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="top" wrapText="1" shrinkToFit="1"/>
     </xf>
   </cellXfs>
@@ -7748,7 +7745,7 @@
       <c r="AA1" s="8"/>
       <c r="AB1" s="8"/>
       <c r="AC1" s="7" t="s">
-        <v>339</v>
+        <v>338</v>
       </c>
       <c r="AD1" s="8"/>
       <c r="AE1" s="8"/>
@@ -7886,25 +7883,25 @@
       <c r="DO1" s="8"/>
       <c r="DP1" s="8"/>
       <c r="DQ1" s="7" t="s">
-        <v>298</v>
+        <v>297</v>
       </c>
       <c r="DR1" s="8"/>
       <c r="DS1" s="8"/>
       <c r="DT1" s="8"/>
       <c r="DU1" s="7" t="s">
-        <v>299</v>
+        <v>298</v>
       </c>
       <c r="DV1" s="8"/>
       <c r="DW1" s="8"/>
       <c r="DX1" s="8"/>
       <c r="DY1" s="7" t="s">
-        <v>318</v>
+        <v>317</v>
       </c>
       <c r="DZ1" s="8"/>
       <c r="EA1" s="8"/>
       <c r="EB1" s="8"/>
       <c r="EC1" s="7" t="s">
-        <v>319</v>
+        <v>318</v>
       </c>
       <c r="ED1" s="8"/>
       <c r="EE1" s="8"/>
@@ -9334,25 +9331,25 @@
       <c r="DO11" s="8"/>
       <c r="DP11" s="8"/>
       <c r="DQ11" s="7" t="s">
-        <v>300</v>
+        <v>299</v>
       </c>
       <c r="DR11" s="8"/>
       <c r="DS11" s="8"/>
       <c r="DT11" s="8"/>
       <c r="DU11" s="7" t="s">
-        <v>311</v>
+        <v>310</v>
       </c>
       <c r="DV11" s="8"/>
       <c r="DW11" s="8"/>
       <c r="DX11" s="8"/>
       <c r="DY11" s="7" t="s">
-        <v>317</v>
+        <v>316</v>
       </c>
       <c r="DZ11" s="8"/>
       <c r="EA11" s="8"/>
       <c r="EB11" s="8"/>
       <c r="EC11" s="7" t="s">
-        <v>331</v>
+        <v>330</v>
       </c>
       <c r="ED11" s="8"/>
       <c r="EE11" s="8"/>
@@ -10781,26 +10778,26 @@
       <c r="DN21" s="8"/>
       <c r="DO21" s="8"/>
       <c r="DP21" s="8"/>
-      <c r="DQ21" s="10" t="s">
-        <v>305</v>
+      <c r="DQ21" s="9" t="s">
+        <v>304</v>
       </c>
       <c r="DR21" s="8"/>
       <c r="DS21" s="8"/>
       <c r="DT21" s="8"/>
       <c r="DU21" s="7" t="s">
-        <v>307</v>
+        <v>306</v>
       </c>
       <c r="DV21" s="8"/>
       <c r="DW21" s="8"/>
       <c r="DX21" s="8"/>
-      <c r="DY21" s="10" t="s">
-        <v>324</v>
+      <c r="DY21" s="9" t="s">
+        <v>323</v>
       </c>
       <c r="DZ21" s="8"/>
       <c r="EA21" s="8"/>
       <c r="EB21" s="8"/>
       <c r="EC21" s="7" t="s">
-        <v>325</v>
+        <v>324</v>
       </c>
       <c r="ED21" s="8"/>
       <c r="EE21" s="8"/>
@@ -12218,37 +12215,37 @@
       <c r="DG31" s="8"/>
       <c r="DH31" s="8"/>
       <c r="DI31" s="7" t="s">
-        <v>292</v>
+        <v>291</v>
       </c>
       <c r="DJ31" s="8"/>
       <c r="DK31" s="8"/>
       <c r="DL31" s="8"/>
       <c r="DM31" s="7" t="s">
-        <v>290</v>
+        <v>289</v>
       </c>
       <c r="DN31" s="8"/>
       <c r="DO31" s="8"/>
       <c r="DP31" s="8"/>
       <c r="DQ31" s="7" t="s">
-        <v>309</v>
+        <v>308</v>
       </c>
       <c r="DR31" s="8"/>
       <c r="DS31" s="8"/>
       <c r="DT31" s="8"/>
       <c r="DU31" s="7" t="s">
-        <v>313</v>
+        <v>312</v>
       </c>
       <c r="DV31" s="8"/>
       <c r="DW31" s="8"/>
       <c r="DX31" s="8"/>
       <c r="DY31" s="7" t="s">
-        <v>328</v>
+        <v>327</v>
       </c>
       <c r="DZ31" s="8"/>
       <c r="EA31" s="8"/>
       <c r="EB31" s="8"/>
       <c r="EC31" s="7" t="s">
-        <v>327</v>
+        <v>326</v>
       </c>
       <c r="ED31" s="8"/>
       <c r="EE31" s="8"/>
@@ -13599,7 +13596,7 @@
       <c r="BN41" s="8"/>
       <c r="BO41" s="8"/>
       <c r="BP41" s="8"/>
-      <c r="BQ41" s="9" t="s">
+      <c r="BQ41" s="10" t="s">
         <v>174</v>
       </c>
       <c r="BR41" s="8"/>
@@ -13611,7 +13608,7 @@
       <c r="BV41" s="8"/>
       <c r="BW41" s="8"/>
       <c r="BX41" s="8"/>
-      <c r="BY41" s="9" t="s">
+      <c r="BY41" s="10" t="s">
         <v>192</v>
       </c>
       <c r="BZ41" s="8"/>
@@ -13623,7 +13620,7 @@
       <c r="CD41" s="8"/>
       <c r="CE41" s="8"/>
       <c r="CF41" s="8"/>
-      <c r="CG41" s="9" t="s">
+      <c r="CG41" s="10" t="s">
         <v>213</v>
       </c>
       <c r="CH41" s="8"/>
@@ -13635,7 +13632,7 @@
       <c r="CL41" s="8"/>
       <c r="CM41" s="8"/>
       <c r="CN41" s="8"/>
-      <c r="CO41" s="9" t="s">
+      <c r="CO41" s="10" t="s">
         <v>234</v>
       </c>
       <c r="CP41" s="8"/>
@@ -13647,7 +13644,7 @@
       <c r="CT41" s="8"/>
       <c r="CU41" s="8"/>
       <c r="CV41" s="8"/>
-      <c r="CW41" s="9" t="s">
+      <c r="CW41" s="10" t="s">
         <v>253</v>
       </c>
       <c r="CX41" s="8"/>
@@ -13659,44 +13656,44 @@
       <c r="DB41" s="8"/>
       <c r="DC41" s="8"/>
       <c r="DD41" s="8"/>
-      <c r="DE41" s="9" t="s">
+      <c r="DE41" s="10" t="s">
         <v>275</v>
       </c>
       <c r="DF41" s="8"/>
       <c r="DG41" s="8"/>
       <c r="DH41" s="8"/>
       <c r="DI41" s="7" t="s">
-        <v>297</v>
+        <v>296</v>
       </c>
       <c r="DJ41" s="8"/>
       <c r="DK41" s="8"/>
       <c r="DL41" s="8"/>
-      <c r="DM41" s="9" t="s">
-        <v>296</v>
+      <c r="DM41" s="10" t="s">
+        <v>295</v>
       </c>
       <c r="DN41" s="8"/>
       <c r="DO41" s="8"/>
       <c r="DP41" s="8"/>
       <c r="DQ41" s="7" t="s">
-        <v>314</v>
+        <v>313</v>
       </c>
       <c r="DR41" s="8"/>
       <c r="DS41" s="8"/>
       <c r="DT41" s="8"/>
-      <c r="DU41" s="9" t="s">
-        <v>320</v>
+      <c r="DU41" s="10" t="s">
+        <v>319</v>
       </c>
       <c r="DV41" s="8"/>
       <c r="DW41" s="8"/>
       <c r="DX41" s="8"/>
       <c r="DY41" s="7" t="s">
-        <v>333</v>
+        <v>332</v>
       </c>
       <c r="DZ41" s="8"/>
       <c r="EA41" s="8"/>
       <c r="EB41" s="8"/>
-      <c r="EC41" s="9" t="s">
-        <v>336</v>
+      <c r="EC41" s="10" t="s">
+        <v>335</v>
       </c>
       <c r="ED41" s="8"/>
       <c r="EE41" s="8"/>
@@ -15126,25 +15123,25 @@
       <c r="DO51" s="6"/>
       <c r="DP51" s="6"/>
       <c r="DQ51" s="5" t="s">
-        <v>302</v>
+        <v>301</v>
       </c>
       <c r="DR51" s="6"/>
       <c r="DS51" s="6"/>
       <c r="DT51" s="6"/>
       <c r="DU51" s="5" t="s">
-        <v>301</v>
+        <v>300</v>
       </c>
       <c r="DV51" s="6"/>
       <c r="DW51" s="6"/>
       <c r="DX51" s="6"/>
       <c r="DY51" s="5" t="s">
-        <v>322</v>
+        <v>321</v>
       </c>
       <c r="DZ51" s="6"/>
       <c r="EA51" s="6"/>
       <c r="EB51" s="6"/>
       <c r="EC51" s="5" t="s">
-        <v>321</v>
+        <v>320</v>
       </c>
       <c r="ED51" s="6"/>
       <c r="EE51" s="6"/>
@@ -16430,7 +16427,7 @@
       <c r="W61" s="6"/>
       <c r="X61" s="6"/>
       <c r="Y61" s="5" t="s">
-        <v>338</v>
+        <v>337</v>
       </c>
       <c r="Z61" s="6"/>
       <c r="AA61" s="6"/>
@@ -16574,25 +16571,25 @@
       <c r="DO61" s="6"/>
       <c r="DP61" s="6"/>
       <c r="DQ61" s="5" t="s">
-        <v>304</v>
+        <v>303</v>
       </c>
       <c r="DR61" s="6"/>
       <c r="DS61" s="6"/>
       <c r="DT61" s="6"/>
       <c r="DU61" s="5" t="s">
-        <v>303</v>
+        <v>302</v>
       </c>
       <c r="DV61" s="6"/>
       <c r="DW61" s="6"/>
       <c r="DX61" s="6"/>
       <c r="DY61" s="5" t="s">
-        <v>335</v>
+        <v>334</v>
       </c>
       <c r="DZ61" s="6"/>
       <c r="EA61" s="6"/>
       <c r="EB61" s="6"/>
       <c r="EC61" s="5" t="s">
-        <v>323</v>
+        <v>322</v>
       </c>
       <c r="ED61" s="6"/>
       <c r="EE61" s="6"/>
@@ -18022,25 +18019,25 @@
       <c r="DO71" s="6"/>
       <c r="DP71" s="6"/>
       <c r="DQ71" s="5" t="s">
-        <v>308</v>
+        <v>307</v>
       </c>
       <c r="DR71" s="6"/>
       <c r="DS71" s="6"/>
       <c r="DT71" s="6"/>
       <c r="DU71" s="5" t="s">
-        <v>306</v>
+        <v>305</v>
       </c>
       <c r="DV71" s="6"/>
       <c r="DW71" s="6"/>
       <c r="DX71" s="6"/>
       <c r="DY71" s="5" t="s">
-        <v>326</v>
+        <v>325</v>
       </c>
       <c r="DZ71" s="6"/>
       <c r="EA71" s="6"/>
       <c r="EB71" s="6"/>
       <c r="EC71" s="5" t="s">
-        <v>332</v>
+        <v>331</v>
       </c>
       <c r="ED71" s="6"/>
       <c r="EE71" s="6"/>
@@ -19458,37 +19455,37 @@
       <c r="DG81" s="6"/>
       <c r="DH81" s="6"/>
       <c r="DI81" s="5" t="s">
-        <v>291</v>
+        <v>290</v>
       </c>
       <c r="DJ81" s="6"/>
       <c r="DK81" s="6"/>
       <c r="DL81" s="6"/>
       <c r="DM81" s="5" t="s">
-        <v>293</v>
+        <v>292</v>
       </c>
       <c r="DN81" s="6"/>
       <c r="DO81" s="6"/>
       <c r="DP81" s="6"/>
       <c r="DQ81" s="5" t="s">
-        <v>312</v>
+        <v>311</v>
       </c>
       <c r="DR81" s="6"/>
       <c r="DS81" s="6"/>
       <c r="DT81" s="6"/>
       <c r="DU81" s="5" t="s">
-        <v>310</v>
+        <v>309</v>
       </c>
       <c r="DV81" s="6"/>
       <c r="DW81" s="6"/>
       <c r="DX81" s="6"/>
       <c r="DY81" s="5" t="s">
-        <v>330</v>
+        <v>329</v>
       </c>
       <c r="DZ81" s="6"/>
       <c r="EA81" s="6"/>
       <c r="EB81" s="6"/>
       <c r="EC81" s="5" t="s">
-        <v>329</v>
+        <v>328</v>
       </c>
       <c r="ED81" s="6"/>
       <c r="EE81" s="6"/>
@@ -20906,37 +20903,37 @@
       <c r="DG91" s="6"/>
       <c r="DH91" s="6"/>
       <c r="DI91" s="5" t="s">
-        <v>294</v>
+        <v>293</v>
       </c>
       <c r="DJ91" s="6"/>
       <c r="DK91" s="6"/>
       <c r="DL91" s="6"/>
       <c r="DM91" s="5" t="s">
-        <v>295</v>
+        <v>294</v>
       </c>
       <c r="DN91" s="6"/>
       <c r="DO91" s="6"/>
       <c r="DP91" s="6"/>
       <c r="DQ91" s="5" t="s">
-        <v>316</v>
+        <v>315</v>
       </c>
       <c r="DR91" s="6"/>
       <c r="DS91" s="6"/>
       <c r="DT91" s="6"/>
       <c r="DU91" s="5" t="s">
-        <v>315</v>
+        <v>314</v>
       </c>
       <c r="DV91" s="6"/>
       <c r="DW91" s="6"/>
       <c r="DX91" s="6"/>
       <c r="DY91" s="5" t="s">
-        <v>337</v>
+        <v>336</v>
       </c>
       <c r="DZ91" s="6"/>
       <c r="EA91" s="6"/>
       <c r="EB91" s="6"/>
       <c r="EC91" s="5" t="s">
-        <v>334</v>
+        <v>333</v>
       </c>
       <c r="ED91" s="6"/>
       <c r="EE91" s="6"/>
@@ -22253,9 +22250,6 @@
       <c r="J105" s="4"/>
       <c r="K105" s="4"/>
       <c r="L105" s="4"/>
-      <c r="DM105" t="s">
-        <v>289</v>
-      </c>
     </row>
     <row r="106" spans="1:136" x14ac:dyDescent="0.3">
       <c r="A106" s="2"/>
@@ -22895,118 +22889,210 @@
     </row>
   </sheetData>
   <mergeCells count="340">
-    <mergeCell ref="DY51:EB60"/>
-    <mergeCell ref="EC51:EF60"/>
-    <mergeCell ref="DY71:EB80"/>
-    <mergeCell ref="EC71:EF80"/>
-    <mergeCell ref="DY81:EB90"/>
-    <mergeCell ref="EC81:EF90"/>
-    <mergeCell ref="DY91:EB100"/>
-    <mergeCell ref="EC91:EF100"/>
-    <mergeCell ref="DY61:EB70"/>
-    <mergeCell ref="EC61:EF70"/>
-    <mergeCell ref="DY1:EB10"/>
-    <mergeCell ref="EC1:EF10"/>
-    <mergeCell ref="DY11:EB20"/>
-    <mergeCell ref="EC11:EF20"/>
-    <mergeCell ref="DY21:EB30"/>
-    <mergeCell ref="EC21:EF30"/>
-    <mergeCell ref="DY31:EB40"/>
-    <mergeCell ref="EC31:EF40"/>
-    <mergeCell ref="DY41:EB50"/>
-    <mergeCell ref="EC41:EF50"/>
-    <mergeCell ref="DQ51:DT60"/>
-    <mergeCell ref="DU51:DX60"/>
-    <mergeCell ref="DQ61:DT70"/>
-    <mergeCell ref="DU61:DX70"/>
-    <mergeCell ref="DQ71:DT80"/>
-    <mergeCell ref="DU71:DX80"/>
-    <mergeCell ref="DQ81:DT90"/>
-    <mergeCell ref="DU81:DX90"/>
-    <mergeCell ref="DQ91:DT100"/>
-    <mergeCell ref="DU91:DX100"/>
-    <mergeCell ref="DQ1:DT10"/>
-    <mergeCell ref="DU1:DX10"/>
-    <mergeCell ref="DQ11:DT20"/>
-    <mergeCell ref="DU11:DX20"/>
-    <mergeCell ref="DQ21:DT30"/>
-    <mergeCell ref="DU21:DX30"/>
-    <mergeCell ref="DQ31:DT40"/>
-    <mergeCell ref="DU31:DX40"/>
-    <mergeCell ref="DQ41:DT50"/>
-    <mergeCell ref="DU41:DX50"/>
-    <mergeCell ref="DI51:DL60"/>
-    <mergeCell ref="DM51:DP60"/>
-    <mergeCell ref="DI61:DL70"/>
-    <mergeCell ref="DM61:DP70"/>
-    <mergeCell ref="DI71:DL80"/>
-    <mergeCell ref="DM71:DP80"/>
-    <mergeCell ref="DI81:DL90"/>
-    <mergeCell ref="DM81:DP90"/>
-    <mergeCell ref="DI91:DL100"/>
-    <mergeCell ref="DM91:DP100"/>
-    <mergeCell ref="DI1:DL10"/>
-    <mergeCell ref="DM1:DP10"/>
-    <mergeCell ref="DI11:DL20"/>
-    <mergeCell ref="DM11:DP20"/>
-    <mergeCell ref="DI21:DL30"/>
-    <mergeCell ref="DM21:DP30"/>
-    <mergeCell ref="DI31:DL40"/>
-    <mergeCell ref="DM31:DP40"/>
-    <mergeCell ref="DI41:DL50"/>
-    <mergeCell ref="DM41:DP50"/>
-    <mergeCell ref="CK51:CN60"/>
-    <mergeCell ref="CO51:CR60"/>
-    <mergeCell ref="CK61:CN70"/>
-    <mergeCell ref="CO61:CR70"/>
-    <mergeCell ref="CK71:CN80"/>
-    <mergeCell ref="CO71:CR80"/>
-    <mergeCell ref="CK81:CN90"/>
-    <mergeCell ref="CO81:CR90"/>
-    <mergeCell ref="CK91:CN100"/>
-    <mergeCell ref="CO91:CR100"/>
-    <mergeCell ref="CK1:CN10"/>
-    <mergeCell ref="CO1:CR10"/>
-    <mergeCell ref="CK11:CN20"/>
-    <mergeCell ref="CO11:CR20"/>
-    <mergeCell ref="CK21:CN30"/>
-    <mergeCell ref="CO21:CR30"/>
-    <mergeCell ref="CK31:CN40"/>
-    <mergeCell ref="CO31:CR40"/>
-    <mergeCell ref="CK41:CN50"/>
-    <mergeCell ref="CO41:CR50"/>
-    <mergeCell ref="CC51:CF60"/>
-    <mergeCell ref="CG51:CJ60"/>
-    <mergeCell ref="CC61:CF70"/>
-    <mergeCell ref="CG61:CJ70"/>
-    <mergeCell ref="CC71:CF80"/>
-    <mergeCell ref="CG71:CJ80"/>
-    <mergeCell ref="CC81:CF90"/>
-    <mergeCell ref="CG81:CJ90"/>
-    <mergeCell ref="CC91:CF100"/>
-    <mergeCell ref="CG91:CJ100"/>
-    <mergeCell ref="CC1:CF10"/>
-    <mergeCell ref="CG1:CJ10"/>
-    <mergeCell ref="CC11:CF20"/>
-    <mergeCell ref="CG11:CJ20"/>
-    <mergeCell ref="CC21:CF30"/>
-    <mergeCell ref="CG21:CJ30"/>
-    <mergeCell ref="CC31:CF40"/>
-    <mergeCell ref="CG31:CJ40"/>
-    <mergeCell ref="CC41:CF50"/>
-    <mergeCell ref="CG41:CJ50"/>
-    <mergeCell ref="AS91:AV100"/>
-    <mergeCell ref="AS61:AV70"/>
-    <mergeCell ref="AO71:AR80"/>
-    <mergeCell ref="AS71:AV80"/>
-    <mergeCell ref="AO81:AR90"/>
-    <mergeCell ref="AS81:AV90"/>
-    <mergeCell ref="AO31:AR40"/>
-    <mergeCell ref="AS31:AV40"/>
-    <mergeCell ref="AO41:AR50"/>
-    <mergeCell ref="AS41:AV50"/>
-    <mergeCell ref="AO51:AR60"/>
-    <mergeCell ref="AS51:AV60"/>
+    <mergeCell ref="DA51:DD60"/>
+    <mergeCell ref="DE51:DH60"/>
+    <mergeCell ref="DA61:DD70"/>
+    <mergeCell ref="DE61:DH70"/>
+    <mergeCell ref="DA71:DD80"/>
+    <mergeCell ref="DE71:DH80"/>
+    <mergeCell ref="DA81:DD90"/>
+    <mergeCell ref="DE81:DH90"/>
+    <mergeCell ref="DA91:DD100"/>
+    <mergeCell ref="DE91:DH100"/>
+    <mergeCell ref="DA1:DD10"/>
+    <mergeCell ref="DE1:DH10"/>
+    <mergeCell ref="DA11:DD20"/>
+    <mergeCell ref="DE11:DH20"/>
+    <mergeCell ref="DA21:DD30"/>
+    <mergeCell ref="DE21:DH30"/>
+    <mergeCell ref="DA31:DD40"/>
+    <mergeCell ref="DE31:DH40"/>
+    <mergeCell ref="DA41:DD50"/>
+    <mergeCell ref="DE41:DH50"/>
+    <mergeCell ref="CS51:CV60"/>
+    <mergeCell ref="CW51:CZ60"/>
+    <mergeCell ref="CS61:CV70"/>
+    <mergeCell ref="CW61:CZ70"/>
+    <mergeCell ref="CS71:CV80"/>
+    <mergeCell ref="CW71:CZ80"/>
+    <mergeCell ref="CS81:CV90"/>
+    <mergeCell ref="CW81:CZ90"/>
+    <mergeCell ref="CS91:CV100"/>
+    <mergeCell ref="CW91:CZ100"/>
+    <mergeCell ref="CS1:CV10"/>
+    <mergeCell ref="CW1:CZ10"/>
+    <mergeCell ref="CS11:CV20"/>
+    <mergeCell ref="CW11:CZ20"/>
+    <mergeCell ref="CS21:CV30"/>
+    <mergeCell ref="CW21:CZ30"/>
+    <mergeCell ref="CS31:CV40"/>
+    <mergeCell ref="CW31:CZ40"/>
+    <mergeCell ref="CS41:CV50"/>
+    <mergeCell ref="CW41:CZ50"/>
+    <mergeCell ref="BU51:BX60"/>
+    <mergeCell ref="BY51:CB60"/>
+    <mergeCell ref="BU61:BX70"/>
+    <mergeCell ref="BY61:CB70"/>
+    <mergeCell ref="BU71:BX80"/>
+    <mergeCell ref="BY71:CB80"/>
+    <mergeCell ref="BU81:BX90"/>
+    <mergeCell ref="BY81:CB90"/>
+    <mergeCell ref="BU91:BX100"/>
+    <mergeCell ref="BY91:CB100"/>
+    <mergeCell ref="BU1:BX10"/>
+    <mergeCell ref="BY1:CB10"/>
+    <mergeCell ref="BU11:BX20"/>
+    <mergeCell ref="BY11:CB20"/>
+    <mergeCell ref="BU21:BX30"/>
+    <mergeCell ref="BY21:CB30"/>
+    <mergeCell ref="BU31:BX40"/>
+    <mergeCell ref="BY31:CB40"/>
+    <mergeCell ref="BU41:BX50"/>
+    <mergeCell ref="BY41:CB50"/>
+    <mergeCell ref="BM51:BP60"/>
+    <mergeCell ref="BQ51:BT60"/>
+    <mergeCell ref="BM61:BP70"/>
+    <mergeCell ref="BQ61:BT70"/>
+    <mergeCell ref="BM71:BP80"/>
+    <mergeCell ref="BQ71:BT80"/>
+    <mergeCell ref="BM81:BP90"/>
+    <mergeCell ref="BQ81:BT90"/>
+    <mergeCell ref="BM91:BP100"/>
+    <mergeCell ref="BQ91:BT100"/>
+    <mergeCell ref="BM1:BP10"/>
+    <mergeCell ref="BQ1:BT10"/>
+    <mergeCell ref="BM11:BP20"/>
+    <mergeCell ref="BQ11:BT20"/>
+    <mergeCell ref="BM21:BP30"/>
+    <mergeCell ref="BQ21:BT30"/>
+    <mergeCell ref="BM31:BP40"/>
+    <mergeCell ref="BQ31:BT40"/>
+    <mergeCell ref="BM41:BP50"/>
+    <mergeCell ref="BQ41:BT50"/>
+    <mergeCell ref="BE51:BH60"/>
+    <mergeCell ref="BI51:BL60"/>
+    <mergeCell ref="BE61:BH70"/>
+    <mergeCell ref="BI61:BL70"/>
+    <mergeCell ref="BE71:BH80"/>
+    <mergeCell ref="BI71:BL80"/>
+    <mergeCell ref="BE81:BH90"/>
+    <mergeCell ref="BI81:BL90"/>
+    <mergeCell ref="BE91:BH100"/>
+    <mergeCell ref="BI91:BL100"/>
+    <mergeCell ref="BE1:BH10"/>
+    <mergeCell ref="BI1:BL10"/>
+    <mergeCell ref="BE11:BH20"/>
+    <mergeCell ref="BI11:BL20"/>
+    <mergeCell ref="BE21:BH30"/>
+    <mergeCell ref="BI21:BL30"/>
+    <mergeCell ref="BE31:BH40"/>
+    <mergeCell ref="BI31:BL40"/>
+    <mergeCell ref="BE41:BH50"/>
+    <mergeCell ref="BI41:BL50"/>
+    <mergeCell ref="Q91:T100"/>
+    <mergeCell ref="U91:X100"/>
+    <mergeCell ref="Y91:AB100"/>
+    <mergeCell ref="AC91:AF100"/>
+    <mergeCell ref="AW1:AZ10"/>
+    <mergeCell ref="BA1:BD10"/>
+    <mergeCell ref="AW11:AZ20"/>
+    <mergeCell ref="BA11:BD20"/>
+    <mergeCell ref="AW21:AZ30"/>
+    <mergeCell ref="BA21:BD30"/>
+    <mergeCell ref="AW31:AZ40"/>
+    <mergeCell ref="BA31:BD40"/>
+    <mergeCell ref="AW41:AZ50"/>
+    <mergeCell ref="BA41:BD50"/>
+    <mergeCell ref="AW51:AZ60"/>
+    <mergeCell ref="BA51:BD60"/>
+    <mergeCell ref="AW61:AZ70"/>
+    <mergeCell ref="BA61:BD70"/>
+    <mergeCell ref="AW71:AZ80"/>
+    <mergeCell ref="BA71:BD80"/>
+    <mergeCell ref="AW81:AZ90"/>
+    <mergeCell ref="BA81:BD90"/>
+    <mergeCell ref="AW91:AZ100"/>
+    <mergeCell ref="BA91:BD100"/>
+    <mergeCell ref="Q61:T70"/>
+    <mergeCell ref="U61:X70"/>
+    <mergeCell ref="Y61:AB70"/>
+    <mergeCell ref="AC61:AF70"/>
+    <mergeCell ref="Q71:T80"/>
+    <mergeCell ref="U71:X80"/>
+    <mergeCell ref="Y71:AB80"/>
+    <mergeCell ref="AC71:AF80"/>
+    <mergeCell ref="Q81:T90"/>
+    <mergeCell ref="U81:X90"/>
+    <mergeCell ref="Y81:AB90"/>
+    <mergeCell ref="AC81:AF90"/>
+    <mergeCell ref="Q31:T40"/>
+    <mergeCell ref="U31:X40"/>
+    <mergeCell ref="Y31:AB40"/>
+    <mergeCell ref="AC31:AF40"/>
+    <mergeCell ref="Q41:T50"/>
+    <mergeCell ref="U41:X50"/>
+    <mergeCell ref="Y41:AB50"/>
+    <mergeCell ref="AC41:AF50"/>
+    <mergeCell ref="Q51:T60"/>
+    <mergeCell ref="U51:X60"/>
+    <mergeCell ref="Y51:AB60"/>
+    <mergeCell ref="AC51:AF60"/>
+    <mergeCell ref="Q1:T10"/>
+    <mergeCell ref="U1:X10"/>
+    <mergeCell ref="Y1:AB10"/>
+    <mergeCell ref="AC1:AF10"/>
+    <mergeCell ref="Q11:T20"/>
+    <mergeCell ref="U11:X20"/>
+    <mergeCell ref="Y11:AB20"/>
+    <mergeCell ref="AC11:AF20"/>
+    <mergeCell ref="Q21:T30"/>
+    <mergeCell ref="U21:X30"/>
+    <mergeCell ref="Y21:AB30"/>
+    <mergeCell ref="AC21:AF30"/>
+    <mergeCell ref="I81:L90"/>
+    <mergeCell ref="M81:P90"/>
+    <mergeCell ref="I91:L100"/>
+    <mergeCell ref="M91:P100"/>
+    <mergeCell ref="I51:L60"/>
+    <mergeCell ref="M51:P60"/>
+    <mergeCell ref="I61:L70"/>
+    <mergeCell ref="M61:P70"/>
+    <mergeCell ref="I71:L80"/>
+    <mergeCell ref="M71:P80"/>
+    <mergeCell ref="A81:D90"/>
+    <mergeCell ref="E81:H90"/>
+    <mergeCell ref="A91:D100"/>
+    <mergeCell ref="E91:H100"/>
+    <mergeCell ref="A51:D60"/>
+    <mergeCell ref="E51:H60"/>
+    <mergeCell ref="A61:D70"/>
+    <mergeCell ref="E61:H70"/>
+    <mergeCell ref="A71:D80"/>
+    <mergeCell ref="E71:H80"/>
+    <mergeCell ref="AG41:AJ50"/>
+    <mergeCell ref="AK41:AN50"/>
+    <mergeCell ref="AG71:AJ80"/>
+    <mergeCell ref="AK71:AN80"/>
+    <mergeCell ref="A1:D10"/>
+    <mergeCell ref="E1:H10"/>
+    <mergeCell ref="A11:D20"/>
+    <mergeCell ref="E11:H20"/>
+    <mergeCell ref="A21:D30"/>
+    <mergeCell ref="E21:H30"/>
+    <mergeCell ref="M31:P40"/>
+    <mergeCell ref="I41:L50"/>
+    <mergeCell ref="M41:P50"/>
+    <mergeCell ref="A31:D40"/>
+    <mergeCell ref="E31:H40"/>
+    <mergeCell ref="A41:D50"/>
+    <mergeCell ref="E41:H50"/>
+    <mergeCell ref="I31:L40"/>
+    <mergeCell ref="I1:L10"/>
+    <mergeCell ref="M1:P10"/>
+    <mergeCell ref="I11:L20"/>
+    <mergeCell ref="M11:P20"/>
+    <mergeCell ref="I21:L30"/>
+    <mergeCell ref="M21:P30"/>
     <mergeCell ref="AO1:AR10"/>
     <mergeCell ref="AS1:AV10"/>
     <mergeCell ref="AO11:AR20"/>
@@ -23031,213 +23117,121 @@
     <mergeCell ref="AK21:AN30"/>
     <mergeCell ref="AG31:AJ40"/>
     <mergeCell ref="AK31:AN40"/>
-    <mergeCell ref="AG41:AJ50"/>
-    <mergeCell ref="AK41:AN50"/>
-    <mergeCell ref="AG71:AJ80"/>
-    <mergeCell ref="AK71:AN80"/>
-    <mergeCell ref="A1:D10"/>
-    <mergeCell ref="E1:H10"/>
-    <mergeCell ref="A11:D20"/>
-    <mergeCell ref="E11:H20"/>
-    <mergeCell ref="A21:D30"/>
-    <mergeCell ref="E21:H30"/>
-    <mergeCell ref="M31:P40"/>
-    <mergeCell ref="I41:L50"/>
-    <mergeCell ref="M41:P50"/>
-    <mergeCell ref="A31:D40"/>
-    <mergeCell ref="E31:H40"/>
-    <mergeCell ref="A41:D50"/>
-    <mergeCell ref="E41:H50"/>
-    <mergeCell ref="I31:L40"/>
-    <mergeCell ref="I1:L10"/>
-    <mergeCell ref="M1:P10"/>
-    <mergeCell ref="I11:L20"/>
-    <mergeCell ref="M11:P20"/>
-    <mergeCell ref="I21:L30"/>
-    <mergeCell ref="M21:P30"/>
-    <mergeCell ref="A81:D90"/>
-    <mergeCell ref="E81:H90"/>
-    <mergeCell ref="A91:D100"/>
-    <mergeCell ref="E91:H100"/>
-    <mergeCell ref="A51:D60"/>
-    <mergeCell ref="E51:H60"/>
-    <mergeCell ref="A61:D70"/>
-    <mergeCell ref="E61:H70"/>
-    <mergeCell ref="A71:D80"/>
-    <mergeCell ref="E71:H80"/>
-    <mergeCell ref="I81:L90"/>
-    <mergeCell ref="M81:P90"/>
-    <mergeCell ref="I91:L100"/>
-    <mergeCell ref="M91:P100"/>
-    <mergeCell ref="I51:L60"/>
-    <mergeCell ref="M51:P60"/>
-    <mergeCell ref="I61:L70"/>
-    <mergeCell ref="M61:P70"/>
-    <mergeCell ref="I71:L80"/>
-    <mergeCell ref="M71:P80"/>
-    <mergeCell ref="Q1:T10"/>
-    <mergeCell ref="U1:X10"/>
-    <mergeCell ref="Y1:AB10"/>
-    <mergeCell ref="AC1:AF10"/>
-    <mergeCell ref="Q11:T20"/>
-    <mergeCell ref="U11:X20"/>
-    <mergeCell ref="Y11:AB20"/>
-    <mergeCell ref="AC11:AF20"/>
-    <mergeCell ref="Q21:T30"/>
-    <mergeCell ref="U21:X30"/>
-    <mergeCell ref="Y21:AB30"/>
-    <mergeCell ref="AC21:AF30"/>
-    <mergeCell ref="Q31:T40"/>
-    <mergeCell ref="U31:X40"/>
-    <mergeCell ref="Y31:AB40"/>
-    <mergeCell ref="AC31:AF40"/>
-    <mergeCell ref="Q41:T50"/>
-    <mergeCell ref="U41:X50"/>
-    <mergeCell ref="Y41:AB50"/>
-    <mergeCell ref="AC41:AF50"/>
-    <mergeCell ref="Q51:T60"/>
-    <mergeCell ref="U51:X60"/>
-    <mergeCell ref="Y51:AB60"/>
-    <mergeCell ref="AC51:AF60"/>
-    <mergeCell ref="Q61:T70"/>
-    <mergeCell ref="U61:X70"/>
-    <mergeCell ref="Y61:AB70"/>
-    <mergeCell ref="AC61:AF70"/>
-    <mergeCell ref="Q71:T80"/>
-    <mergeCell ref="U71:X80"/>
-    <mergeCell ref="Y71:AB80"/>
-    <mergeCell ref="AC71:AF80"/>
-    <mergeCell ref="Q81:T90"/>
-    <mergeCell ref="U81:X90"/>
-    <mergeCell ref="Y81:AB90"/>
-    <mergeCell ref="AC81:AF90"/>
-    <mergeCell ref="Q91:T100"/>
-    <mergeCell ref="U91:X100"/>
-    <mergeCell ref="Y91:AB100"/>
-    <mergeCell ref="AC91:AF100"/>
-    <mergeCell ref="AW1:AZ10"/>
-    <mergeCell ref="BA1:BD10"/>
-    <mergeCell ref="AW11:AZ20"/>
-    <mergeCell ref="BA11:BD20"/>
-    <mergeCell ref="AW21:AZ30"/>
-    <mergeCell ref="BA21:BD30"/>
-    <mergeCell ref="AW31:AZ40"/>
-    <mergeCell ref="BA31:BD40"/>
-    <mergeCell ref="AW41:AZ50"/>
-    <mergeCell ref="BA41:BD50"/>
-    <mergeCell ref="AW51:AZ60"/>
-    <mergeCell ref="BA51:BD60"/>
-    <mergeCell ref="AW61:AZ70"/>
-    <mergeCell ref="BA61:BD70"/>
-    <mergeCell ref="AW71:AZ80"/>
-    <mergeCell ref="BA71:BD80"/>
-    <mergeCell ref="AW81:AZ90"/>
-    <mergeCell ref="BA81:BD90"/>
-    <mergeCell ref="AW91:AZ100"/>
-    <mergeCell ref="BA91:BD100"/>
-    <mergeCell ref="BE1:BH10"/>
-    <mergeCell ref="BI1:BL10"/>
-    <mergeCell ref="BE11:BH20"/>
-    <mergeCell ref="BI11:BL20"/>
-    <mergeCell ref="BE21:BH30"/>
-    <mergeCell ref="BI21:BL30"/>
-    <mergeCell ref="BE31:BH40"/>
-    <mergeCell ref="BI31:BL40"/>
-    <mergeCell ref="BE41:BH50"/>
-    <mergeCell ref="BI41:BL50"/>
-    <mergeCell ref="BE51:BH60"/>
-    <mergeCell ref="BI51:BL60"/>
-    <mergeCell ref="BE61:BH70"/>
-    <mergeCell ref="BI61:BL70"/>
-    <mergeCell ref="BE71:BH80"/>
-    <mergeCell ref="BI71:BL80"/>
-    <mergeCell ref="BE81:BH90"/>
-    <mergeCell ref="BI81:BL90"/>
-    <mergeCell ref="BE91:BH100"/>
-    <mergeCell ref="BI91:BL100"/>
-    <mergeCell ref="BM1:BP10"/>
-    <mergeCell ref="BQ1:BT10"/>
-    <mergeCell ref="BM11:BP20"/>
-    <mergeCell ref="BQ11:BT20"/>
-    <mergeCell ref="BM21:BP30"/>
-    <mergeCell ref="BQ21:BT30"/>
-    <mergeCell ref="BM31:BP40"/>
-    <mergeCell ref="BQ31:BT40"/>
-    <mergeCell ref="BM41:BP50"/>
-    <mergeCell ref="BQ41:BT50"/>
-    <mergeCell ref="BM51:BP60"/>
-    <mergeCell ref="BQ51:BT60"/>
-    <mergeCell ref="BM61:BP70"/>
-    <mergeCell ref="BQ61:BT70"/>
-    <mergeCell ref="BM71:BP80"/>
-    <mergeCell ref="BQ71:BT80"/>
-    <mergeCell ref="BM81:BP90"/>
-    <mergeCell ref="BQ81:BT90"/>
-    <mergeCell ref="BM91:BP100"/>
-    <mergeCell ref="BQ91:BT100"/>
-    <mergeCell ref="BU1:BX10"/>
-    <mergeCell ref="BY1:CB10"/>
-    <mergeCell ref="BU11:BX20"/>
-    <mergeCell ref="BY11:CB20"/>
-    <mergeCell ref="BU21:BX30"/>
-    <mergeCell ref="BY21:CB30"/>
-    <mergeCell ref="BU31:BX40"/>
-    <mergeCell ref="BY31:CB40"/>
-    <mergeCell ref="BU41:BX50"/>
-    <mergeCell ref="BY41:CB50"/>
-    <mergeCell ref="BU51:BX60"/>
-    <mergeCell ref="BY51:CB60"/>
-    <mergeCell ref="BU61:BX70"/>
-    <mergeCell ref="BY61:CB70"/>
-    <mergeCell ref="BU71:BX80"/>
-    <mergeCell ref="BY71:CB80"/>
-    <mergeCell ref="BU81:BX90"/>
-    <mergeCell ref="BY81:CB90"/>
-    <mergeCell ref="BU91:BX100"/>
-    <mergeCell ref="BY91:CB100"/>
-    <mergeCell ref="CS1:CV10"/>
-    <mergeCell ref="CW1:CZ10"/>
-    <mergeCell ref="CS11:CV20"/>
-    <mergeCell ref="CW11:CZ20"/>
-    <mergeCell ref="CS21:CV30"/>
-    <mergeCell ref="CW21:CZ30"/>
-    <mergeCell ref="CS31:CV40"/>
-    <mergeCell ref="CW31:CZ40"/>
-    <mergeCell ref="CS41:CV50"/>
-    <mergeCell ref="CW41:CZ50"/>
-    <mergeCell ref="CS51:CV60"/>
-    <mergeCell ref="CW51:CZ60"/>
-    <mergeCell ref="CS61:CV70"/>
-    <mergeCell ref="CW61:CZ70"/>
-    <mergeCell ref="CS71:CV80"/>
-    <mergeCell ref="CW71:CZ80"/>
-    <mergeCell ref="CS81:CV90"/>
-    <mergeCell ref="CW81:CZ90"/>
-    <mergeCell ref="CS91:CV100"/>
-    <mergeCell ref="CW91:CZ100"/>
-    <mergeCell ref="DA1:DD10"/>
-    <mergeCell ref="DE1:DH10"/>
-    <mergeCell ref="DA11:DD20"/>
-    <mergeCell ref="DE11:DH20"/>
-    <mergeCell ref="DA21:DD30"/>
-    <mergeCell ref="DE21:DH30"/>
-    <mergeCell ref="DA31:DD40"/>
-    <mergeCell ref="DE31:DH40"/>
-    <mergeCell ref="DA41:DD50"/>
-    <mergeCell ref="DE41:DH50"/>
-    <mergeCell ref="DA51:DD60"/>
-    <mergeCell ref="DE51:DH60"/>
-    <mergeCell ref="DA61:DD70"/>
-    <mergeCell ref="DE61:DH70"/>
-    <mergeCell ref="DA71:DD80"/>
-    <mergeCell ref="DE71:DH80"/>
-    <mergeCell ref="DA81:DD90"/>
-    <mergeCell ref="DE81:DH90"/>
-    <mergeCell ref="DA91:DD100"/>
-    <mergeCell ref="DE91:DH100"/>
+    <mergeCell ref="AS91:AV100"/>
+    <mergeCell ref="AS61:AV70"/>
+    <mergeCell ref="AO71:AR80"/>
+    <mergeCell ref="AS71:AV80"/>
+    <mergeCell ref="AO81:AR90"/>
+    <mergeCell ref="AS81:AV90"/>
+    <mergeCell ref="AO31:AR40"/>
+    <mergeCell ref="AS31:AV40"/>
+    <mergeCell ref="AO41:AR50"/>
+    <mergeCell ref="AS41:AV50"/>
+    <mergeCell ref="AO51:AR60"/>
+    <mergeCell ref="AS51:AV60"/>
+    <mergeCell ref="CC1:CF10"/>
+    <mergeCell ref="CG1:CJ10"/>
+    <mergeCell ref="CC11:CF20"/>
+    <mergeCell ref="CG11:CJ20"/>
+    <mergeCell ref="CC21:CF30"/>
+    <mergeCell ref="CG21:CJ30"/>
+    <mergeCell ref="CC31:CF40"/>
+    <mergeCell ref="CG31:CJ40"/>
+    <mergeCell ref="CC41:CF50"/>
+    <mergeCell ref="CG41:CJ50"/>
+    <mergeCell ref="CC51:CF60"/>
+    <mergeCell ref="CG51:CJ60"/>
+    <mergeCell ref="CC61:CF70"/>
+    <mergeCell ref="CG61:CJ70"/>
+    <mergeCell ref="CC71:CF80"/>
+    <mergeCell ref="CG71:CJ80"/>
+    <mergeCell ref="CC81:CF90"/>
+    <mergeCell ref="CG81:CJ90"/>
+    <mergeCell ref="CC91:CF100"/>
+    <mergeCell ref="CG91:CJ100"/>
+    <mergeCell ref="CK1:CN10"/>
+    <mergeCell ref="CO1:CR10"/>
+    <mergeCell ref="CK11:CN20"/>
+    <mergeCell ref="CO11:CR20"/>
+    <mergeCell ref="CK21:CN30"/>
+    <mergeCell ref="CO21:CR30"/>
+    <mergeCell ref="CK31:CN40"/>
+    <mergeCell ref="CO31:CR40"/>
+    <mergeCell ref="CK41:CN50"/>
+    <mergeCell ref="CO41:CR50"/>
+    <mergeCell ref="CK51:CN60"/>
+    <mergeCell ref="CO51:CR60"/>
+    <mergeCell ref="CK61:CN70"/>
+    <mergeCell ref="CO61:CR70"/>
+    <mergeCell ref="CK71:CN80"/>
+    <mergeCell ref="CO71:CR80"/>
+    <mergeCell ref="CK81:CN90"/>
+    <mergeCell ref="CO81:CR90"/>
+    <mergeCell ref="CK91:CN100"/>
+    <mergeCell ref="CO91:CR100"/>
+    <mergeCell ref="DI1:DL10"/>
+    <mergeCell ref="DM1:DP10"/>
+    <mergeCell ref="DI11:DL20"/>
+    <mergeCell ref="DM11:DP20"/>
+    <mergeCell ref="DI21:DL30"/>
+    <mergeCell ref="DM21:DP30"/>
+    <mergeCell ref="DI31:DL40"/>
+    <mergeCell ref="DM31:DP40"/>
+    <mergeCell ref="DI41:DL50"/>
+    <mergeCell ref="DM41:DP50"/>
+    <mergeCell ref="DI51:DL60"/>
+    <mergeCell ref="DM51:DP60"/>
+    <mergeCell ref="DI61:DL70"/>
+    <mergeCell ref="DM61:DP70"/>
+    <mergeCell ref="DI71:DL80"/>
+    <mergeCell ref="DM71:DP80"/>
+    <mergeCell ref="DI81:DL90"/>
+    <mergeCell ref="DM81:DP90"/>
+    <mergeCell ref="DI91:DL100"/>
+    <mergeCell ref="DM91:DP100"/>
+    <mergeCell ref="DQ1:DT10"/>
+    <mergeCell ref="DU1:DX10"/>
+    <mergeCell ref="DQ11:DT20"/>
+    <mergeCell ref="DU11:DX20"/>
+    <mergeCell ref="DQ21:DT30"/>
+    <mergeCell ref="DU21:DX30"/>
+    <mergeCell ref="DQ31:DT40"/>
+    <mergeCell ref="DU31:DX40"/>
+    <mergeCell ref="DQ41:DT50"/>
+    <mergeCell ref="DU41:DX50"/>
+    <mergeCell ref="DQ51:DT60"/>
+    <mergeCell ref="DU51:DX60"/>
+    <mergeCell ref="DQ61:DT70"/>
+    <mergeCell ref="DU61:DX70"/>
+    <mergeCell ref="DQ71:DT80"/>
+    <mergeCell ref="DU71:DX80"/>
+    <mergeCell ref="DQ81:DT90"/>
+    <mergeCell ref="DU81:DX90"/>
+    <mergeCell ref="DQ91:DT100"/>
+    <mergeCell ref="DU91:DX100"/>
+    <mergeCell ref="DY1:EB10"/>
+    <mergeCell ref="EC1:EF10"/>
+    <mergeCell ref="DY11:EB20"/>
+    <mergeCell ref="EC11:EF20"/>
+    <mergeCell ref="DY21:EB30"/>
+    <mergeCell ref="EC21:EF30"/>
+    <mergeCell ref="DY31:EB40"/>
+    <mergeCell ref="EC31:EF40"/>
+    <mergeCell ref="DY41:EB50"/>
+    <mergeCell ref="EC41:EF50"/>
+    <mergeCell ref="DY51:EB60"/>
+    <mergeCell ref="EC51:EF60"/>
+    <mergeCell ref="DY71:EB80"/>
+    <mergeCell ref="EC71:EF80"/>
+    <mergeCell ref="DY81:EB90"/>
+    <mergeCell ref="EC81:EF90"/>
+    <mergeCell ref="DY91:EB100"/>
+    <mergeCell ref="EC91:EF100"/>
+    <mergeCell ref="DY61:EB70"/>
+    <mergeCell ref="EC61:EF70"/>
   </mergeCells>
   <printOptions horizontalCentered="1" verticalCentered="1"/>
-  <pageMargins left="0.6692913385826772" right="0.6692913385826772" top="0.74803149606299213" bottom="0.74803149606299213" header="0.31496062992125984" footer="0.31496062992125984"/>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup paperSize="9" orientation="portrait" horizontalDpi="300" verticalDpi="300" r:id="rId1"/>
 </worksheet>
 </file>
</xml_diff>